<commit_message>
Update Gitai application with new expense tracking features, including multiple JSON files for M2 diesel records and new images. Increment data snapshot version in config.js for improved data management. Update Excel workbooks to reflect recent changes.
</commit_message>
<xml_diff>
--- a/Gitai-M1.xlsx
+++ b/Gitai-M1.xlsx
@@ -468,7 +468,7 @@
         <v>Gitai.xlsx</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-07-31T13:53:14.631Z</v>
+        <v>2026-07-31T14:05:49.498Z</v>
       </c>
       <c r="E2">
         <v>1174</v>
@@ -39689,7 +39689,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B44" t="str">
         <v>2022-03-14</v>
@@ -39712,7 +39712,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B45" t="str">
         <v>2022-03-18</v>
@@ -39735,7 +39735,7 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B46" t="str">
         <v>2022-03-22</v>
@@ -39758,7 +39758,7 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B47" t="str">
         <v>2022-03-22</v>
@@ -39781,7 +39781,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B48" t="str">
         <v>2022-03-22</v>
@@ -39804,7 +39804,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B49" t="str">
         <v>2022-03-22</v>
@@ -39827,7 +39827,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B50" t="str">
         <v>2022-03-22</v>
@@ -39850,7 +39850,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B51" t="str">
         <v>2022-03-31</v>
@@ -39873,7 +39873,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B52" t="str">
         <v>2022-04-04</v>
@@ -39896,7 +39896,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B53" t="str">
         <v>2022-04-07</v>
@@ -39919,7 +39919,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B54" t="str">
         <v>2022-04-07</v>
@@ -39942,7 +39942,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B55" t="str">
         <v>2022-04-08</v>
@@ -39965,7 +39965,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B56" t="str">
         <v>2022-04-09</v>
@@ -39988,7 +39988,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B57" t="str">
         <v>2022-04-11</v>
@@ -40011,7 +40011,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B58" t="str">
         <v>2022-04-11</v>
@@ -40034,7 +40034,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B59" t="str">
         <v>2022-04-11</v>
@@ -40057,7 +40057,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B60" t="str">
         <v>2022-04-13</v>
@@ -40080,7 +40080,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B61" t="str">
         <v>2022-04-13</v>
@@ -40103,7 +40103,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B62" t="str">
         <v>2022-04-14</v>
@@ -40126,7 +40126,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B63" t="str">
         <v>2022-04-15</v>
@@ -40149,7 +40149,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B64" t="str">
         <v>2022-04-16</v>
@@ -40172,7 +40172,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B65" t="str">
         <v>2022-04-17</v>
@@ -40195,7 +40195,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B66" t="str">
         <v>2022-04-18</v>
@@ -40218,7 +40218,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B67" t="str">
         <v>2022-04-19</v>
@@ -40241,7 +40241,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B68" t="str">
         <v>2022-04-20</v>
@@ -40264,7 +40264,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B69" t="str">
         <v>2022-04-21</v>
@@ -40287,7 +40287,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B70" t="str">
         <v>2022-04-21</v>
@@ -40310,7 +40310,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B71" t="str">
         <v>2022-04-22</v>
@@ -40333,7 +40333,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B72" t="str">
         <v>2022-04-22</v>
@@ -40356,7 +40356,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B73" t="str">
         <v>2022-04-24</v>
@@ -40379,7 +40379,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B74" t="str">
         <v>2022-04-25</v>
@@ -40402,7 +40402,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B75" t="str">
         <v>2022-04-26</v>
@@ -40425,7 +40425,7 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B76" t="str">
         <v>2022-04-26</v>
@@ -40448,7 +40448,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B77" t="str">
         <v>2022-04-26</v>
@@ -40471,7 +40471,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B78" t="str">
         <v>2022-04-28</v>
@@ -40494,7 +40494,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B79" t="str">
         <v>2022-04-28</v>
@@ -40517,7 +40517,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B80" t="str">
         <v>2022-04-29</v>
@@ -40540,7 +40540,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B81" t="str">
         <v>2022-04-29</v>
@@ -40563,7 +40563,7 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B82" t="str">
         <v>2022-05-01</v>
@@ -40586,7 +40586,7 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B83" t="str">
         <v>2022-05-03</v>
@@ -40609,7 +40609,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B84" t="str">
         <v>2022-05-04</v>
@@ -40632,7 +40632,7 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B85" t="str">
         <v>2022-05-04</v>
@@ -40655,7 +40655,7 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B86" t="str">
         <v>2022-05-06</v>
@@ -40678,7 +40678,7 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B87" t="str">
         <v>2022-05-06</v>
@@ -40701,7 +40701,7 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B88" t="str">
         <v>2022-05-07</v>
@@ -40724,7 +40724,7 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B89" t="str">
         <v>2022-05-07</v>
@@ -40747,7 +40747,7 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B90" t="str">
         <v>2022-05-09</v>
@@ -40770,7 +40770,7 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B91" t="str">
         <v>2022-05-09</v>
@@ -40793,7 +40793,7 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B92" t="str">
         <v>2022-05-09</v>
@@ -40816,7 +40816,7 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B93" t="str">
         <v>2022-05-09</v>
@@ -40839,7 +40839,7 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B94" t="str">
         <v>2022-05-10</v>
@@ -40862,7 +40862,7 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B95" t="str">
         <v>2022-05-11</v>
@@ -40885,7 +40885,7 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B96" t="str">
         <v>2022-05-11</v>
@@ -40908,7 +40908,7 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B97" t="str">
         <v>2022-05-11</v>
@@ -40931,7 +40931,7 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B98" t="str">
         <v>2022-05-12</v>
@@ -40954,7 +40954,7 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B99" t="str">
         <v>2022-05-12</v>
@@ -40977,7 +40977,7 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B100" t="str">
         <v>2022-05-13</v>
@@ -41000,7 +41000,7 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B101" t="str">
         <v>2022-05-14</v>
@@ -41023,7 +41023,7 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B102" t="str">
         <v>2022-05-14</v>
@@ -41046,7 +41046,7 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B103" t="str">
         <v>2022-05-16</v>
@@ -41069,7 +41069,7 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B104" t="str">
         <v>2022-05-18</v>
@@ -41092,7 +41092,7 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B105" t="str">
         <v>2022-05-19</v>
@@ -41115,7 +41115,7 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B106" t="str">
         <v>2022-05-19</v>
@@ -41138,7 +41138,7 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B107" t="str">
         <v>2022-05-20</v>
@@ -41161,7 +41161,7 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B108" t="str">
         <v>2022-05-21</v>
@@ -41184,7 +41184,7 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B109" t="str">
         <v>2022-05-22</v>
@@ -41207,7 +41207,7 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B110" t="str">
         <v>2022-05-23</v>
@@ -41230,7 +41230,7 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B111" t="str">
         <v>2022-05-23</v>
@@ -41253,7 +41253,7 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B112" t="str">
         <v>2022-05-24</v>
@@ -41276,7 +41276,7 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B113" t="str">
         <v>2022-05-26</v>
@@ -41299,7 +41299,7 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B114" t="str">
         <v>2022-05-27</v>
@@ -41322,7 +41322,7 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B115" t="str">
         <v>2022-05-28</v>
@@ -41345,7 +41345,7 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="B116" t="str">
         <v>2022-05-30</v>
@@ -41368,7 +41368,7 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B117" t="str">
         <v>2022-05-30</v>
@@ -41391,7 +41391,7 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B118" t="str">
         <v>2022-06-01</v>
@@ -41414,7 +41414,7 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="B119" t="str">
         <v>2022-06-03</v>
@@ -41437,7 +41437,7 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B120" t="str">
         <v>2022-06-03</v>
@@ -41460,7 +41460,7 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B121" t="str">
         <v>2022-06-06</v>
@@ -41483,7 +41483,7 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B122" t="str">
         <v>2022-06-08</v>
@@ -41506,7 +41506,7 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="B123" t="str">
         <v>2022-06-09</v>
@@ -41529,7 +41529,7 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B124" t="str">
         <v>2022-06-13</v>
@@ -41552,7 +41552,7 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B125" t="str">
         <v>2022-06-13</v>
@@ -41575,7 +41575,7 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B126" t="str">
         <v>2022-06-15</v>
@@ -41598,7 +41598,7 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B127" t="str">
         <v>2022-06-16</v>
@@ -41621,7 +41621,7 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B128" t="str">
         <v>2022-06-16</v>
@@ -41644,7 +41644,7 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B129" t="str">
         <v>2022-06-16</v>
@@ -41667,7 +41667,7 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="B130" t="str">
         <v>2022-06-17</v>
@@ -41690,7 +41690,7 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B131" t="str">
         <v>2022-06-20</v>
@@ -41713,7 +41713,7 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B132" t="str">
         <v>2022-06-27</v>
@@ -41736,7 +41736,7 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B133" t="str">
         <v>2022-06-27</v>
@@ -41759,7 +41759,7 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B134" t="str">
         <v>2022-09-06</v>
@@ -41782,7 +41782,7 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B135" t="str">
         <v>2022-09-17</v>
@@ -41805,7 +41805,7 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B136" t="str">
         <v>2022-09-22</v>
@@ -41828,7 +41828,7 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B137" t="str">
         <v>2022-10-31</v>
@@ -41851,7 +41851,7 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B138" t="str">
         <v>2022-10-31</v>
@@ -41874,7 +41874,7 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B139" t="str">
         <v>2022-11-10</v>
@@ -41897,7 +41897,7 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B140" t="str">
         <v>2022-11-13</v>
@@ -41920,7 +41920,7 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="B141" t="str">
         <v>2022-11-14</v>
@@ -41943,7 +41943,7 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="B142" t="str">
         <v>2022-11-16</v>
@@ -41966,7 +41966,7 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B143" t="str">
         <v>2022-11-19</v>
@@ -41989,7 +41989,7 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="B144" t="str">
         <v>2022-11-20</v>
@@ -42012,7 +42012,7 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B145" t="str">
         <v>2022-11-27</v>
@@ -42035,7 +42035,7 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="B146" t="str">
         <v>2022-12-04</v>
@@ -42058,7 +42058,7 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="B147" t="str">
         <v>2022-12-07</v>
@@ -42081,7 +42081,7 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B148" t="str">
         <v>2022-12-09</v>
@@ -42104,7 +42104,7 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="B149" t="str">
         <v>2022-12-10</v>
@@ -42127,7 +42127,7 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B150" t="str">
         <v>2022-12-12</v>
@@ -42150,7 +42150,7 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B151" t="str">
         <v>2022-12-21</v>
@@ -42173,7 +42173,7 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B152" t="str">
         <v>2022-12-28</v>
@@ -42196,7 +42196,7 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B153" t="str">
         <v>2023-01-07</v>
@@ -42219,7 +42219,7 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B154" t="str">
         <v>2023-01-07</v>
@@ -42242,7 +42242,7 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B155" t="str">
         <v>2023-01-11</v>
@@ -42265,7 +42265,7 @@
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="B156" t="str">
         <v>2023-01-12</v>
@@ -42288,7 +42288,7 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B157" t="str">
         <v>2023-01-17</v>
@@ -42311,7 +42311,7 @@
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B158" t="str">
         <v>2023-01-19</v>
@@ -42334,7 +42334,7 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B159" t="str">
         <v>2023-01-20</v>
@@ -42357,7 +42357,7 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B160" t="str">
         <v>2023-01-21</v>
@@ -42380,7 +42380,7 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="B161" t="str">
         <v>2023-01-24</v>
@@ -42403,7 +42403,7 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B162" t="str">
         <v>2023-01-29</v>
@@ -42426,7 +42426,7 @@
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B163" t="str">
         <v>2023-01-30</v>
@@ -42449,7 +42449,7 @@
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B164" t="str">
         <v>2023-02-05</v>
@@ -42472,7 +42472,7 @@
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B165" t="str">
         <v>2023-02-06</v>
@@ -42495,7 +42495,7 @@
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="B166" t="str">
         <v>2023-02-08</v>
@@ -42518,7 +42518,7 @@
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B167" t="str">
         <v>2023-02-10</v>
@@ -42541,7 +42541,7 @@
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="B168" t="str">
         <v>2023-02-11</v>
@@ -42564,7 +42564,7 @@
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="B169" t="str">
         <v>2023-02-13</v>
@@ -42587,7 +42587,7 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="B170" t="str">
         <v>2023-02-14</v>
@@ -42610,7 +42610,7 @@
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="B171" t="str">
         <v>2023-02-15</v>
@@ -42633,7 +42633,7 @@
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B172" t="str">
         <v>2023-02-18</v>
@@ -42656,7 +42656,7 @@
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="B173" t="str">
         <v>2023-02-19</v>
@@ -42679,7 +42679,7 @@
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B174" t="str">
         <v>2023-02-24</v>
@@ -42702,7 +42702,7 @@
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="B175" t="str">
         <v>2023-02-24</v>
@@ -42725,7 +42725,7 @@
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="B176" t="str">
         <v>2023-03-09</v>
@@ -42748,7 +42748,7 @@
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="B177" t="str">
         <v>2023-03-11</v>
@@ -42771,7 +42771,7 @@
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="B178" t="str">
         <v>2023-03-15</v>
@@ -42794,7 +42794,7 @@
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="B179" t="str">
         <v>2023-03-15</v>
@@ -42817,7 +42817,7 @@
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="B180" t="str">
         <v>2023-03-23</v>
@@ -42840,7 +42840,7 @@
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="B181" t="str">
         <v>2023-03-27</v>
@@ -42863,7 +42863,7 @@
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="B182" t="str">
         <v>2023-03-31</v>
@@ -42886,7 +42886,7 @@
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="B183" t="str">
         <v>2023-04-03</v>
@@ -42909,7 +42909,7 @@
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="B184" t="str">
         <v>2023-04-07</v>
@@ -42932,7 +42932,7 @@
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B185" t="str">
         <v>2023-04-08</v>
@@ -42955,7 +42955,7 @@
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="B186" t="str">
         <v>2023-04-10</v>
@@ -42978,7 +42978,7 @@
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="B187" t="str">
         <v>2023-04-11</v>
@@ -43001,7 +43001,7 @@
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="B188" t="str">
         <v>2023-04-12</v>
@@ -43024,7 +43024,7 @@
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B189" t="str">
         <v>2023-04-13</v>
@@ -43047,7 +43047,7 @@
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="B190" t="str">
         <v>2023-04-16</v>
@@ -43070,7 +43070,7 @@
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="B191" t="str">
         <v>2023-04-18</v>
@@ -43093,7 +43093,7 @@
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="B192" t="str">
         <v>2023-09-28</v>
@@ -43116,7 +43116,7 @@
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="B193" t="str">
         <v>2023-09-28</v>
@@ -43139,7 +43139,7 @@
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="B194" t="str">
         <v>2023-09-29</v>
@@ -43162,7 +43162,7 @@
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="B195" t="str">
         <v>2023-09-29</v>
@@ -43185,7 +43185,7 @@
     </row>
     <row r="196">
       <c r="A196" t="str">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="B196" t="str">
         <v>2023-09-29</v>
@@ -43208,7 +43208,7 @@
     </row>
     <row r="197">
       <c r="A197" t="str">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="B197" t="str">
         <v>2023-09-29</v>
@@ -43231,7 +43231,7 @@
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="B198" t="str">
         <v>2023-10-10</v>
@@ -43254,7 +43254,7 @@
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="B199" t="str">
         <v>2023-10-10</v>
@@ -43277,7 +43277,7 @@
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v>199</v>
+        <v>220</v>
       </c>
       <c r="B200" t="str">
         <v>2023-11-23</v>
@@ -43300,7 +43300,7 @@
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v>200</v>
+        <v>222</v>
       </c>
       <c r="B201" t="str">
         <v>2023-11-26</v>
@@ -43323,7 +43323,7 @@
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v>201</v>
+        <v>224</v>
       </c>
       <c r="B202" t="str">
         <v>2023-12-01</v>
@@ -43346,7 +43346,7 @@
     </row>
     <row r="203">
       <c r="A203" t="str">
-        <v>202</v>
+        <v>225</v>
       </c>
       <c r="B203" t="str">
         <v>2023-12-04</v>
@@ -43369,7 +43369,7 @@
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v>203</v>
+        <v>226</v>
       </c>
       <c r="B204" t="str">
         <v>2023-12-05</v>
@@ -43392,7 +43392,7 @@
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v>204</v>
+        <v>227</v>
       </c>
       <c r="B205" t="str">
         <v>2023-12-06</v>
@@ -43415,7 +43415,7 @@
     </row>
     <row r="206">
       <c r="A206" t="str">
-        <v>205</v>
+        <v>228</v>
       </c>
       <c r="B206" t="str">
         <v>2023-12-07</v>
@@ -43438,7 +43438,7 @@
     </row>
     <row r="207">
       <c r="A207" t="str">
-        <v>206</v>
+        <v>229</v>
       </c>
       <c r="B207" t="str">
         <v>2023-12-07</v>
@@ -43461,7 +43461,7 @@
     </row>
     <row r="208">
       <c r="A208" t="str">
-        <v>207</v>
+        <v>230</v>
       </c>
       <c r="B208" t="str">
         <v>2023-12-08</v>
@@ -43484,7 +43484,7 @@
     </row>
     <row r="209">
       <c r="A209" t="str">
-        <v>208</v>
+        <v>231</v>
       </c>
       <c r="B209" t="str">
         <v>2023-12-09</v>
@@ -43507,7 +43507,7 @@
     </row>
     <row r="210">
       <c r="A210" t="str">
-        <v>209</v>
+        <v>232</v>
       </c>
       <c r="B210" t="str">
         <v>2023-12-10</v>
@@ -43530,7 +43530,7 @@
     </row>
     <row r="211">
       <c r="A211" t="str">
-        <v>210</v>
+        <v>234</v>
       </c>
       <c r="B211" t="str">
         <v>2023-12-11</v>
@@ -43553,7 +43553,7 @@
     </row>
     <row r="212">
       <c r="A212" t="str">
-        <v>211</v>
+        <v>235</v>
       </c>
       <c r="B212" t="str">
         <v>2023-12-11</v>
@@ -43576,7 +43576,7 @@
     </row>
     <row r="213">
       <c r="A213" t="str">
-        <v>212</v>
+        <v>236</v>
       </c>
       <c r="B213" t="str">
         <v>2023-12-11</v>
@@ -43599,7 +43599,7 @@
     </row>
     <row r="214">
       <c r="A214" t="str">
-        <v>213</v>
+        <v>237</v>
       </c>
       <c r="B214" t="str">
         <v>2023-12-11</v>
@@ -43622,7 +43622,7 @@
     </row>
     <row r="215">
       <c r="A215" t="str">
-        <v>214</v>
+        <v>238</v>
       </c>
       <c r="B215" t="str">
         <v>2023-12-11</v>
@@ -43645,7 +43645,7 @@
     </row>
     <row r="216">
       <c r="A216" t="str">
-        <v>215</v>
+        <v>239</v>
       </c>
       <c r="B216" t="str">
         <v>2023-12-11</v>
@@ -43668,7 +43668,7 @@
     </row>
     <row r="217">
       <c r="A217" t="str">
-        <v>216</v>
+        <v>240</v>
       </c>
       <c r="B217" t="str">
         <v>2023-12-11</v>
@@ -43691,7 +43691,7 @@
     </row>
     <row r="218">
       <c r="A218" t="str">
-        <v>217</v>
+        <v>241</v>
       </c>
       <c r="B218" t="str">
         <v>2023-12-11</v>
@@ -43714,7 +43714,7 @@
     </row>
     <row r="219">
       <c r="A219" t="str">
-        <v>218</v>
+        <v>242</v>
       </c>
       <c r="B219" t="str">
         <v>2023-12-11</v>
@@ -43737,7 +43737,7 @@
     </row>
     <row r="220">
       <c r="A220" t="str">
-        <v>219</v>
+        <v>243</v>
       </c>
       <c r="B220" t="str">
         <v>2023-12-16</v>
@@ -43760,7 +43760,7 @@
     </row>
     <row r="221">
       <c r="A221" t="str">
-        <v>220</v>
+        <v>244</v>
       </c>
       <c r="B221" t="str">
         <v>2023-12-18</v>
@@ -43783,7 +43783,7 @@
     </row>
     <row r="222">
       <c r="A222" t="str">
-        <v>221</v>
+        <v>250</v>
       </c>
       <c r="B222" t="str">
         <v>2024-01-06</v>
@@ -43806,7 +43806,7 @@
     </row>
     <row r="223">
       <c r="A223" t="str">
-        <v>222</v>
+        <v>251</v>
       </c>
       <c r="B223" t="str">
         <v>2024-01-06</v>
@@ -43829,7 +43829,7 @@
     </row>
     <row r="224">
       <c r="A224" t="str">
-        <v>223</v>
+        <v>252</v>
       </c>
       <c r="B224" t="str">
         <v>2024-01-06</v>
@@ -43852,7 +43852,7 @@
     </row>
     <row r="225">
       <c r="A225" t="str">
-        <v>224</v>
+        <v>253</v>
       </c>
       <c r="B225" t="str">
         <v>2024-01-06</v>
@@ -43875,7 +43875,7 @@
     </row>
     <row r="226">
       <c r="A226" t="str">
-        <v>225</v>
+        <v>254</v>
       </c>
       <c r="B226" t="str">
         <v>2024-01-07</v>
@@ -43898,7 +43898,7 @@
     </row>
     <row r="227">
       <c r="A227" t="str">
-        <v>226</v>
+        <v>255</v>
       </c>
       <c r="B227" t="str">
         <v>2024-01-07</v>
@@ -43921,7 +43921,7 @@
     </row>
     <row r="228">
       <c r="A228" t="str">
-        <v>227</v>
+        <v>256</v>
       </c>
       <c r="B228" t="str">
         <v>2024-01-07</v>
@@ -43944,7 +43944,7 @@
     </row>
     <row r="229">
       <c r="A229" t="str">
-        <v>228</v>
+        <v>257</v>
       </c>
       <c r="B229" t="str">
         <v>2024-01-07</v>
@@ -43967,7 +43967,7 @@
     </row>
     <row r="230">
       <c r="A230" t="str">
-        <v>229</v>
+        <v>258</v>
       </c>
       <c r="B230" t="str">
         <v>2024-01-08</v>
@@ -43990,7 +43990,7 @@
     </row>
     <row r="231">
       <c r="A231" t="str">
-        <v>230</v>
+        <v>259</v>
       </c>
       <c r="B231" t="str">
         <v>2024-01-10</v>
@@ -44013,7 +44013,7 @@
     </row>
     <row r="232">
       <c r="A232" t="str">
-        <v>231</v>
+        <v>260</v>
       </c>
       <c r="B232" t="str">
         <v>2024-01-11</v>
@@ -44036,7 +44036,7 @@
     </row>
     <row r="233">
       <c r="A233" t="str">
-        <v>232</v>
+        <v>261</v>
       </c>
       <c r="B233" t="str">
         <v>2024-01-11</v>
@@ -44059,7 +44059,7 @@
     </row>
     <row r="234">
       <c r="A234" t="str">
-        <v>233</v>
+        <v>262</v>
       </c>
       <c r="B234" t="str">
         <v>2024-01-11</v>
@@ -44082,7 +44082,7 @@
     </row>
     <row r="235">
       <c r="A235" t="str">
-        <v>234</v>
+        <v>266</v>
       </c>
       <c r="B235" t="str">
         <v>2024-01-17</v>
@@ -44105,7 +44105,7 @@
     </row>
     <row r="236">
       <c r="A236" t="str">
-        <v>235</v>
+        <v>267</v>
       </c>
       <c r="B236" t="str">
         <v>2024-01-18</v>
@@ -44128,7 +44128,7 @@
     </row>
     <row r="237">
       <c r="A237" t="str">
-        <v>236</v>
+        <v>268</v>
       </c>
       <c r="B237" t="str">
         <v>2024-01-19</v>
@@ -44151,7 +44151,7 @@
     </row>
     <row r="238">
       <c r="A238" t="str">
-        <v>237</v>
+        <v>269</v>
       </c>
       <c r="B238" t="str">
         <v>2024-01-19</v>
@@ -44174,7 +44174,7 @@
     </row>
     <row r="239">
       <c r="A239" t="str">
-        <v>238</v>
+        <v>270</v>
       </c>
       <c r="B239" t="str">
         <v>2024-01-19</v>
@@ -44197,7 +44197,7 @@
     </row>
     <row r="240">
       <c r="A240" t="str">
-        <v>239</v>
+        <v>271</v>
       </c>
       <c r="B240" t="str">
         <v>2024-01-20</v>
@@ -44220,7 +44220,7 @@
     </row>
     <row r="241">
       <c r="A241" t="str">
-        <v>240</v>
+        <v>272</v>
       </c>
       <c r="B241" t="str">
         <v>2024-01-22</v>
@@ -44243,7 +44243,7 @@
     </row>
     <row r="242">
       <c r="A242" t="str">
-        <v>241</v>
+        <v>273</v>
       </c>
       <c r="B242" t="str">
         <v>2024-01-22</v>
@@ -44266,7 +44266,7 @@
     </row>
     <row r="243">
       <c r="A243" t="str">
-        <v>242</v>
+        <v>274</v>
       </c>
       <c r="B243" t="str">
         <v>2024-01-22</v>
@@ -44289,7 +44289,7 @@
     </row>
     <row r="244">
       <c r="A244" t="str">
-        <v>243</v>
+        <v>275</v>
       </c>
       <c r="B244" t="str">
         <v>2024-01-24</v>
@@ -44312,7 +44312,7 @@
     </row>
     <row r="245">
       <c r="A245" t="str">
-        <v>244</v>
+        <v>276</v>
       </c>
       <c r="B245" t="str">
         <v>2024-01-25</v>
@@ -44335,7 +44335,7 @@
     </row>
     <row r="246">
       <c r="A246" t="str">
-        <v>245</v>
+        <v>277</v>
       </c>
       <c r="B246" t="str">
         <v>2024-01-27</v>
@@ -44358,7 +44358,7 @@
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v>246</v>
+        <v>278</v>
       </c>
       <c r="B247" t="str">
         <v>2024-01-28</v>
@@ -44381,7 +44381,7 @@
     </row>
     <row r="248">
       <c r="A248" t="str">
-        <v>247</v>
+        <v>279</v>
       </c>
       <c r="B248" t="str">
         <v>2024-01-29</v>
@@ -44404,7 +44404,7 @@
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v>248</v>
+        <v>280</v>
       </c>
       <c r="B249" t="str">
         <v>2024-01-29</v>
@@ -44427,7 +44427,7 @@
     </row>
     <row r="250">
       <c r="A250" t="str">
-        <v>249</v>
+        <v>281</v>
       </c>
       <c r="B250" t="str">
         <v>2024-02-01</v>
@@ -44450,7 +44450,7 @@
     </row>
     <row r="251">
       <c r="A251" t="str">
-        <v>250</v>
+        <v>282</v>
       </c>
       <c r="B251" t="str">
         <v>2024-02-01</v>
@@ -44473,7 +44473,7 @@
     </row>
     <row r="252">
       <c r="A252" t="str">
-        <v>251</v>
+        <v>283</v>
       </c>
       <c r="B252" t="str">
         <v>2024-02-02</v>
@@ -44496,7 +44496,7 @@
     </row>
     <row r="253">
       <c r="A253" t="str">
-        <v>252</v>
+        <v>284</v>
       </c>
       <c r="B253" t="str">
         <v>2024-02-03</v>
@@ -44519,7 +44519,7 @@
     </row>
     <row r="254">
       <c r="A254" t="str">
-        <v>253</v>
+        <v>285</v>
       </c>
       <c r="B254" t="str">
         <v>2024-02-03</v>
@@ -44542,7 +44542,7 @@
     </row>
     <row r="255">
       <c r="A255" t="str">
-        <v>254</v>
+        <v>286</v>
       </c>
       <c r="B255" t="str">
         <v>2024-02-06</v>
@@ -44565,7 +44565,7 @@
     </row>
     <row r="256">
       <c r="A256" t="str">
-        <v>255</v>
+        <v>287</v>
       </c>
       <c r="B256" t="str">
         <v>2024-02-06</v>
@@ -44588,7 +44588,7 @@
     </row>
     <row r="257">
       <c r="A257" t="str">
-        <v>256</v>
+        <v>288</v>
       </c>
       <c r="B257" t="str">
         <v>2024-02-06</v>
@@ -44611,7 +44611,7 @@
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>257</v>
+        <v>289</v>
       </c>
       <c r="B258" t="str">
         <v>2024-02-06</v>
@@ -44634,7 +44634,7 @@
     </row>
     <row r="259">
       <c r="A259" t="str">
-        <v>258</v>
+        <v>290</v>
       </c>
       <c r="B259" t="str">
         <v>2024-02-08</v>
@@ -44657,7 +44657,7 @@
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>259</v>
+        <v>291</v>
       </c>
       <c r="B260" t="str">
         <v>2024-02-10</v>
@@ -44680,7 +44680,7 @@
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>260</v>
+        <v>292</v>
       </c>
       <c r="B261" t="str">
         <v>2024-02-11</v>
@@ -44703,7 +44703,7 @@
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>261</v>
+        <v>294</v>
       </c>
       <c r="B262" t="str">
         <v>2024-02-13</v>
@@ -44726,7 +44726,7 @@
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>262</v>
+        <v>295</v>
       </c>
       <c r="B263" t="str">
         <v>2024-02-14</v>
@@ -44749,7 +44749,7 @@
     </row>
     <row r="264">
       <c r="A264" t="str">
-        <v>263</v>
+        <v>296</v>
       </c>
       <c r="B264" t="str">
         <v>2024-02-14</v>
@@ -44772,7 +44772,7 @@
     </row>
     <row r="265">
       <c r="A265" t="str">
-        <v>264</v>
+        <v>297</v>
       </c>
       <c r="B265" t="str">
         <v>2024-02-14</v>
@@ -44795,7 +44795,7 @@
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>265</v>
+        <v>298</v>
       </c>
       <c r="B266" t="str">
         <v>2024-02-15</v>
@@ -44818,7 +44818,7 @@
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>266</v>
+        <v>299</v>
       </c>
       <c r="B267" t="str">
         <v>2024-02-15</v>
@@ -44841,7 +44841,7 @@
     </row>
     <row r="268">
       <c r="A268" t="str">
-        <v>267</v>
+        <v>300</v>
       </c>
       <c r="B268" t="str">
         <v>2024-02-16</v>
@@ -44864,7 +44864,7 @@
     </row>
     <row r="269">
       <c r="A269" t="str">
-        <v>268</v>
+        <v>302</v>
       </c>
       <c r="B269" t="str">
         <v>2024-02-24</v>
@@ -44887,7 +44887,7 @@
     </row>
     <row r="270">
       <c r="A270" t="str">
-        <v>269</v>
+        <v>304</v>
       </c>
       <c r="B270" t="str">
         <v>2024-02-25</v>
@@ -44910,7 +44910,7 @@
     </row>
     <row r="271">
       <c r="A271" t="str">
-        <v>270</v>
+        <v>305</v>
       </c>
       <c r="B271" t="str">
         <v>2024-02-26</v>
@@ -44933,7 +44933,7 @@
     </row>
     <row r="272">
       <c r="A272" t="str">
-        <v>271</v>
+        <v>308</v>
       </c>
       <c r="B272" t="str">
         <v>2024-02-28</v>
@@ -44956,7 +44956,7 @@
     </row>
     <row r="273">
       <c r="A273" t="str">
-        <v>272</v>
+        <v>309</v>
       </c>
       <c r="B273" t="str">
         <v>2024-02-29</v>
@@ -44979,7 +44979,7 @@
     </row>
     <row r="274">
       <c r="A274" t="str">
-        <v>273</v>
+        <v>311</v>
       </c>
       <c r="B274" t="str">
         <v>2024-03-01</v>
@@ -45002,7 +45002,7 @@
     </row>
     <row r="275">
       <c r="A275" t="str">
-        <v>274</v>
+        <v>313</v>
       </c>
       <c r="B275" t="str">
         <v>2024-03-02</v>
@@ -45025,7 +45025,7 @@
     </row>
     <row r="276">
       <c r="A276" t="str">
-        <v>275</v>
+        <v>314</v>
       </c>
       <c r="B276" t="str">
         <v>2024-03-02</v>
@@ -45048,7 +45048,7 @@
     </row>
     <row r="277">
       <c r="A277" t="str">
-        <v>276</v>
+        <v>315</v>
       </c>
       <c r="B277" t="str">
         <v>2024-03-03</v>
@@ -45071,7 +45071,7 @@
     </row>
     <row r="278">
       <c r="A278" t="str">
-        <v>277</v>
+        <v>316</v>
       </c>
       <c r="B278" t="str">
         <v>2024-03-04</v>
@@ -45094,7 +45094,7 @@
     </row>
     <row r="279">
       <c r="A279" t="str">
-        <v>278</v>
+        <v>317</v>
       </c>
       <c r="B279" t="str">
         <v>2024-03-05</v>
@@ -45117,7 +45117,7 @@
     </row>
     <row r="280">
       <c r="A280" t="str">
-        <v>279</v>
+        <v>318</v>
       </c>
       <c r="B280" t="str">
         <v>2024-03-05</v>
@@ -45140,7 +45140,7 @@
     </row>
     <row r="281">
       <c r="A281" t="str">
-        <v>280</v>
+        <v>319</v>
       </c>
       <c r="B281" t="str">
         <v>2024-03-06</v>
@@ -45163,7 +45163,7 @@
     </row>
     <row r="282">
       <c r="A282" t="str">
-        <v>281</v>
+        <v>321</v>
       </c>
       <c r="B282" t="str">
         <v>2024-03-07</v>
@@ -45186,7 +45186,7 @@
     </row>
     <row r="283">
       <c r="A283" t="str">
-        <v>282</v>
+        <v>325</v>
       </c>
       <c r="B283" t="str">
         <v>2024-03-14</v>
@@ -45209,7 +45209,7 @@
     </row>
     <row r="284">
       <c r="A284" t="str">
-        <v>283</v>
+        <v>326</v>
       </c>
       <c r="B284" t="str">
         <v>2024-03-14</v>
@@ -45232,7 +45232,7 @@
     </row>
     <row r="285">
       <c r="A285" t="str">
-        <v>284</v>
+        <v>327</v>
       </c>
       <c r="B285" t="str">
         <v>2024-03-14</v>
@@ -45255,7 +45255,7 @@
     </row>
     <row r="286">
       <c r="A286" t="str">
-        <v>285</v>
+        <v>328</v>
       </c>
       <c r="B286" t="str">
         <v>2024-03-14</v>
@@ -45278,7 +45278,7 @@
     </row>
     <row r="287">
       <c r="A287" t="str">
-        <v>286</v>
+        <v>329</v>
       </c>
       <c r="B287" t="str">
         <v>2024-03-14</v>
@@ -45301,7 +45301,7 @@
     </row>
     <row r="288">
       <c r="A288" t="str">
-        <v>287</v>
+        <v>330</v>
       </c>
       <c r="B288" t="str">
         <v>2024-03-14</v>
@@ -45324,7 +45324,7 @@
     </row>
     <row r="289">
       <c r="A289" t="str">
-        <v>288</v>
+        <v>331</v>
       </c>
       <c r="B289" t="str">
         <v>2024-03-14</v>
@@ -45347,7 +45347,7 @@
     </row>
     <row r="290">
       <c r="A290" t="str">
-        <v>289</v>
+        <v>332</v>
       </c>
       <c r="B290" t="str">
         <v>2024-03-14</v>
@@ -45370,7 +45370,7 @@
     </row>
     <row r="291">
       <c r="A291" t="str">
-        <v>290</v>
+        <v>340</v>
       </c>
       <c r="B291" t="str">
         <v>2024-04-01</v>
@@ -45393,7 +45393,7 @@
     </row>
     <row r="292">
       <c r="A292" t="str">
-        <v>291</v>
+        <v>342</v>
       </c>
       <c r="B292" t="str">
         <v>2024-04-02</v>
@@ -45416,7 +45416,7 @@
     </row>
     <row r="293">
       <c r="A293" t="str">
-        <v>292</v>
+        <v>343</v>
       </c>
       <c r="B293" t="str">
         <v>2024-04-02</v>
@@ -45439,7 +45439,7 @@
     </row>
     <row r="294">
       <c r="A294" t="str">
-        <v>293</v>
+        <v>344</v>
       </c>
       <c r="B294" t="str">
         <v>2024-04-02</v>
@@ -45462,7 +45462,7 @@
     </row>
     <row r="295">
       <c r="A295" t="str">
-        <v>294</v>
+        <v>347</v>
       </c>
       <c r="B295" t="str">
         <v>2024-04-04</v>
@@ -45485,7 +45485,7 @@
     </row>
     <row r="296">
       <c r="A296" t="str">
-        <v>295</v>
+        <v>349</v>
       </c>
       <c r="B296" t="str">
         <v>2024-04-05</v>
@@ -45508,7 +45508,7 @@
     </row>
     <row r="297">
       <c r="A297" t="str">
-        <v>296</v>
+        <v>350</v>
       </c>
       <c r="B297" t="str">
         <v>2024-04-05</v>
@@ -45531,7 +45531,7 @@
     </row>
     <row r="298">
       <c r="A298" t="str">
-        <v>297</v>
+        <v>351</v>
       </c>
       <c r="B298" t="str">
         <v>2024-04-06</v>
@@ -45554,7 +45554,7 @@
     </row>
     <row r="299">
       <c r="A299" t="str">
-        <v>298</v>
+        <v>353</v>
       </c>
       <c r="B299" t="str">
         <v>2024-04-07</v>
@@ -45577,7 +45577,7 @@
     </row>
     <row r="300">
       <c r="A300" t="str">
-        <v>299</v>
+        <v>354</v>
       </c>
       <c r="B300" t="str">
         <v>2024-04-08</v>
@@ -45600,7 +45600,7 @@
     </row>
     <row r="301">
       <c r="A301" t="str">
-        <v>300</v>
+        <v>355</v>
       </c>
       <c r="B301" t="str">
         <v>2024-04-08</v>
@@ -45623,7 +45623,7 @@
     </row>
     <row r="302">
       <c r="A302" t="str">
-        <v>301</v>
+        <v>356</v>
       </c>
       <c r="B302" t="str">
         <v>2024-04-08</v>
@@ -45646,7 +45646,7 @@
     </row>
     <row r="303">
       <c r="A303" t="str">
-        <v>302</v>
+        <v>357</v>
       </c>
       <c r="B303" t="str">
         <v>2024-04-09</v>
@@ -45669,7 +45669,7 @@
     </row>
     <row r="304">
       <c r="A304" t="str">
-        <v>303</v>
+        <v>359</v>
       </c>
       <c r="B304" t="str">
         <v>2024-04-10</v>
@@ -45692,7 +45692,7 @@
     </row>
     <row r="305">
       <c r="A305" t="str">
-        <v>304</v>
+        <v>360</v>
       </c>
       <c r="B305" t="str">
         <v>2024-04-10</v>
@@ -45715,7 +45715,7 @@
     </row>
     <row r="306">
       <c r="A306" t="str">
-        <v>305</v>
+        <v>362</v>
       </c>
       <c r="B306" t="str">
         <v>2024-04-11</v>
@@ -45738,7 +45738,7 @@
     </row>
     <row r="307">
       <c r="A307" t="str">
-        <v>306</v>
+        <v>365</v>
       </c>
       <c r="B307" t="str">
         <v>2024-04-16</v>
@@ -45761,7 +45761,7 @@
     </row>
     <row r="308">
       <c r="A308" t="str">
-        <v>307</v>
+        <v>367</v>
       </c>
       <c r="B308" t="str">
         <v>2024-04-19</v>
@@ -45784,7 +45784,7 @@
     </row>
     <row r="309">
       <c r="A309" t="str">
-        <v>308</v>
+        <v>369</v>
       </c>
       <c r="B309" t="str">
         <v>2024-04-20</v>
@@ -45807,7 +45807,7 @@
     </row>
     <row r="310">
       <c r="A310" t="str">
-        <v>309</v>
+        <v>370</v>
       </c>
       <c r="B310" t="str">
         <v>2024-04-20</v>
@@ -45830,7 +45830,7 @@
     </row>
     <row r="311">
       <c r="A311" t="str">
-        <v>310</v>
+        <v>371</v>
       </c>
       <c r="B311" t="str">
         <v>2024-04-20</v>
@@ -45853,7 +45853,7 @@
     </row>
     <row r="312">
       <c r="A312" t="str">
-        <v>311</v>
+        <v>372</v>
       </c>
       <c r="B312" t="str">
         <v>2024-04-20</v>
@@ -45876,7 +45876,7 @@
     </row>
     <row r="313">
       <c r="A313" t="str">
-        <v>312</v>
+        <v>373</v>
       </c>
       <c r="B313" t="str">
         <v>2024-04-20</v>
@@ -45899,7 +45899,7 @@
     </row>
     <row r="314">
       <c r="A314" t="str">
-        <v>313</v>
+        <v>374</v>
       </c>
       <c r="B314" t="str">
         <v>2024-04-20</v>
@@ -45922,7 +45922,7 @@
     </row>
     <row r="315">
       <c r="A315" t="str">
-        <v>314</v>
+        <v>375</v>
       </c>
       <c r="B315" t="str">
         <v>2024-04-20</v>
@@ -45945,7 +45945,7 @@
     </row>
     <row r="316">
       <c r="A316" t="str">
-        <v>315</v>
+        <v>376</v>
       </c>
       <c r="B316" t="str">
         <v>2024-04-22</v>
@@ -45968,7 +45968,7 @@
     </row>
     <row r="317">
       <c r="A317" t="str">
-        <v>316</v>
+        <v>377</v>
       </c>
       <c r="B317" t="str">
         <v>2024-04-23</v>
@@ -45991,7 +45991,7 @@
     </row>
     <row r="318">
       <c r="A318" t="str">
-        <v>317</v>
+        <v>379</v>
       </c>
       <c r="B318" t="str">
         <v>2024-04-26</v>
@@ -46014,7 +46014,7 @@
     </row>
     <row r="319">
       <c r="A319" t="str">
-        <v>318</v>
+        <v>380</v>
       </c>
       <c r="B319" t="str">
         <v>2024-04-26</v>
@@ -46037,7 +46037,7 @@
     </row>
     <row r="320">
       <c r="A320" t="str">
-        <v>319</v>
+        <v>381</v>
       </c>
       <c r="B320" t="str">
         <v>2024-04-27</v>
@@ -46060,7 +46060,7 @@
     </row>
     <row r="321">
       <c r="A321" t="str">
-        <v>320</v>
+        <v>382</v>
       </c>
       <c r="B321" t="str">
         <v>2024-04-28</v>
@@ -46083,7 +46083,7 @@
     </row>
     <row r="322">
       <c r="A322" t="str">
-        <v>321</v>
+        <v>383</v>
       </c>
       <c r="B322" t="str">
         <v>2024-04-30</v>
@@ -46106,7 +46106,7 @@
     </row>
     <row r="323">
       <c r="A323" t="str">
-        <v>322</v>
+        <v>384</v>
       </c>
       <c r="B323" t="str">
         <v>2024-04-30</v>
@@ -46129,7 +46129,7 @@
     </row>
     <row r="324">
       <c r="A324" t="str">
-        <v>323</v>
+        <v>385</v>
       </c>
       <c r="B324" t="str">
         <v>2024-04-30</v>
@@ -46152,7 +46152,7 @@
     </row>
     <row r="325">
       <c r="A325" t="str">
-        <v>324</v>
+        <v>386</v>
       </c>
       <c r="B325" t="str">
         <v>2024-05-01</v>
@@ -46175,7 +46175,7 @@
     </row>
     <row r="326">
       <c r="A326" t="str">
-        <v>325</v>
+        <v>387</v>
       </c>
       <c r="B326" t="str">
         <v>2024-05-02</v>
@@ -46198,7 +46198,7 @@
     </row>
     <row r="327">
       <c r="A327" t="str">
-        <v>326</v>
+        <v>388</v>
       </c>
       <c r="B327" t="str">
         <v>2024-05-03</v>
@@ -46221,7 +46221,7 @@
     </row>
     <row r="328">
       <c r="A328" t="str">
-        <v>327</v>
+        <v>389</v>
       </c>
       <c r="B328" t="str">
         <v>2024-05-03</v>
@@ -46244,7 +46244,7 @@
     </row>
     <row r="329">
       <c r="A329" t="str">
-        <v>328</v>
+        <v>390</v>
       </c>
       <c r="B329" t="str">
         <v>2024-05-04</v>
@@ -46267,7 +46267,7 @@
     </row>
     <row r="330">
       <c r="A330" t="str">
-        <v>329</v>
+        <v>391</v>
       </c>
       <c r="B330" t="str">
         <v>2024-05-04</v>
@@ -46290,7 +46290,7 @@
     </row>
     <row r="331">
       <c r="A331" t="str">
-        <v>330</v>
+        <v>393</v>
       </c>
       <c r="B331" t="str">
         <v>2024-05-05</v>
@@ -46313,7 +46313,7 @@
     </row>
     <row r="332">
       <c r="A332" t="str">
-        <v>331</v>
+        <v>394</v>
       </c>
       <c r="B332" t="str">
         <v>2024-05-06</v>
@@ -46336,7 +46336,7 @@
     </row>
     <row r="333">
       <c r="A333" t="str">
-        <v>332</v>
+        <v>395</v>
       </c>
       <c r="B333" t="str">
         <v>2024-05-06</v>
@@ -46359,7 +46359,7 @@
     </row>
     <row r="334">
       <c r="A334" t="str">
-        <v>333</v>
+        <v>396</v>
       </c>
       <c r="B334" t="str">
         <v>2024-05-07</v>
@@ -46382,7 +46382,7 @@
     </row>
     <row r="335">
       <c r="A335" t="str">
-        <v>334</v>
+        <v>398</v>
       </c>
       <c r="B335" t="str">
         <v>2024-05-09</v>
@@ -46405,7 +46405,7 @@
     </row>
     <row r="336">
       <c r="A336" t="str">
-        <v>335</v>
+        <v>399</v>
       </c>
       <c r="B336" t="str">
         <v>2024-05-10</v>
@@ -46428,7 +46428,7 @@
     </row>
     <row r="337">
       <c r="A337" t="str">
-        <v>336</v>
+        <v>400</v>
       </c>
       <c r="B337" t="str">
         <v>2024-05-11</v>
@@ -46451,7 +46451,7 @@
     </row>
     <row r="338">
       <c r="A338" t="str">
-        <v>337</v>
+        <v>401</v>
       </c>
       <c r="B338" t="str">
         <v>2024-05-11</v>
@@ -46474,7 +46474,7 @@
     </row>
     <row r="339">
       <c r="A339" t="str">
-        <v>338</v>
+        <v>402</v>
       </c>
       <c r="B339" t="str">
         <v>2024-05-11</v>
@@ -46497,7 +46497,7 @@
     </row>
     <row r="340">
       <c r="A340" t="str">
-        <v>339</v>
+        <v>403</v>
       </c>
       <c r="B340" t="str">
         <v>2024-05-11</v>
@@ -46520,7 +46520,7 @@
     </row>
     <row r="341">
       <c r="A341" t="str">
-        <v>340</v>
+        <v>404</v>
       </c>
       <c r="B341" t="str">
         <v>2024-05-11</v>
@@ -46543,7 +46543,7 @@
     </row>
     <row r="342">
       <c r="A342" t="str">
-        <v>341</v>
+        <v>405</v>
       </c>
       <c r="B342" t="str">
         <v>2024-05-11</v>
@@ -46566,7 +46566,7 @@
     </row>
     <row r="343">
       <c r="A343" t="str">
-        <v>342</v>
+        <v>406</v>
       </c>
       <c r="B343" t="str">
         <v>2024-05-11</v>
@@ -46589,7 +46589,7 @@
     </row>
     <row r="344">
       <c r="A344" t="str">
-        <v>343</v>
+        <v>407</v>
       </c>
       <c r="B344" t="str">
         <v>2024-05-11</v>
@@ -46612,7 +46612,7 @@
     </row>
     <row r="345">
       <c r="A345" t="str">
-        <v>344</v>
+        <v>408</v>
       </c>
       <c r="B345" t="str">
         <v>2024-05-12</v>
@@ -46635,7 +46635,7 @@
     </row>
     <row r="346">
       <c r="A346" t="str">
-        <v>345</v>
+        <v>409</v>
       </c>
       <c r="B346" t="str">
         <v>2024-05-12</v>
@@ -46658,7 +46658,7 @@
     </row>
     <row r="347">
       <c r="A347" t="str">
-        <v>346</v>
+        <v>410</v>
       </c>
       <c r="B347" t="str">
         <v>2024-05-14</v>
@@ -46681,7 +46681,7 @@
     </row>
     <row r="348">
       <c r="A348" t="str">
-        <v>347</v>
+        <v>412</v>
       </c>
       <c r="B348" t="str">
         <v>2024-05-15</v>
@@ -46704,7 +46704,7 @@
     </row>
     <row r="349">
       <c r="A349" t="str">
-        <v>348</v>
+        <v>413</v>
       </c>
       <c r="B349" t="str">
         <v>2024-05-16</v>
@@ -46727,7 +46727,7 @@
     </row>
     <row r="350">
       <c r="A350" t="str">
-        <v>349</v>
+        <v>414</v>
       </c>
       <c r="B350" t="str">
         <v>2024-05-17</v>
@@ -46750,7 +46750,7 @@
     </row>
     <row r="351">
       <c r="A351" t="str">
-        <v>350</v>
+        <v>415</v>
       </c>
       <c r="B351" t="str">
         <v>2024-05-18</v>
@@ -46773,7 +46773,7 @@
     </row>
     <row r="352">
       <c r="A352" t="str">
-        <v>351</v>
+        <v>416</v>
       </c>
       <c r="B352" t="str">
         <v>2024-05-18</v>
@@ -46796,7 +46796,7 @@
     </row>
     <row r="353">
       <c r="A353" t="str">
-        <v>352</v>
+        <v>417</v>
       </c>
       <c r="B353" t="str">
         <v>2024-05-19</v>
@@ -46819,7 +46819,7 @@
     </row>
     <row r="354">
       <c r="A354" t="str">
-        <v>353</v>
+        <v>418</v>
       </c>
       <c r="B354" t="str">
         <v>2024-05-19</v>
@@ -46842,7 +46842,7 @@
     </row>
     <row r="355">
       <c r="A355" t="str">
-        <v>354</v>
+        <v>419</v>
       </c>
       <c r="B355" t="str">
         <v>2024-05-20</v>
@@ -46865,7 +46865,7 @@
     </row>
     <row r="356">
       <c r="A356" t="str">
-        <v>355</v>
+        <v>420</v>
       </c>
       <c r="B356" t="str">
         <v>2024-05-20</v>
@@ -46888,7 +46888,7 @@
     </row>
     <row r="357">
       <c r="A357" t="str">
-        <v>356</v>
+        <v>421</v>
       </c>
       <c r="B357" t="str">
         <v>2024-05-20</v>
@@ -46911,7 +46911,7 @@
     </row>
     <row r="358">
       <c r="A358" t="str">
-        <v>357</v>
+        <v>422</v>
       </c>
       <c r="B358" t="str">
         <v>2024-05-20</v>
@@ -46934,7 +46934,7 @@
     </row>
     <row r="359">
       <c r="A359" t="str">
-        <v>358</v>
+        <v>423</v>
       </c>
       <c r="B359" t="str">
         <v>2024-05-20</v>
@@ -46957,7 +46957,7 @@
     </row>
     <row r="360">
       <c r="A360" t="str">
-        <v>359</v>
+        <v>424</v>
       </c>
       <c r="B360" t="str">
         <v>2024-05-20</v>
@@ -46980,7 +46980,7 @@
     </row>
     <row r="361">
       <c r="A361" t="str">
-        <v>360</v>
+        <v>425</v>
       </c>
       <c r="B361" t="str">
         <v>2024-05-20</v>
@@ -47003,7 +47003,7 @@
     </row>
     <row r="362">
       <c r="A362" t="str">
-        <v>361</v>
+        <v>427</v>
       </c>
       <c r="B362" t="str">
         <v>2024-05-21</v>
@@ -47026,7 +47026,7 @@
     </row>
     <row r="363">
       <c r="A363" t="str">
-        <v>362</v>
+        <v>428</v>
       </c>
       <c r="B363" t="str">
         <v>2024-05-21</v>
@@ -47049,7 +47049,7 @@
     </row>
     <row r="364">
       <c r="A364" t="str">
-        <v>363</v>
+        <v>429</v>
       </c>
       <c r="B364" t="str">
         <v>2024-05-21</v>
@@ -47072,7 +47072,7 @@
     </row>
     <row r="365">
       <c r="A365" t="str">
-        <v>364</v>
+        <v>430</v>
       </c>
       <c r="B365" t="str">
         <v>2024-05-21</v>
@@ -47095,7 +47095,7 @@
     </row>
     <row r="366">
       <c r="A366" t="str">
-        <v>365</v>
+        <v>431</v>
       </c>
       <c r="B366" t="str">
         <v>2024-05-21</v>
@@ -47118,7 +47118,7 @@
     </row>
     <row r="367">
       <c r="A367" t="str">
-        <v>366</v>
+        <v>432</v>
       </c>
       <c r="B367" t="str">
         <v>2024-05-21</v>
@@ -47141,7 +47141,7 @@
     </row>
     <row r="368">
       <c r="A368" t="str">
-        <v>367</v>
+        <v>433</v>
       </c>
       <c r="B368" t="str">
         <v>2024-05-21</v>
@@ -47164,7 +47164,7 @@
     </row>
     <row r="369">
       <c r="A369" t="str">
-        <v>368</v>
+        <v>434</v>
       </c>
       <c r="B369" t="str">
         <v>2024-05-22</v>
@@ -47187,7 +47187,7 @@
     </row>
     <row r="370">
       <c r="A370" t="str">
-        <v>369</v>
+        <v>435</v>
       </c>
       <c r="B370" t="str">
         <v>2024-05-23</v>
@@ -47210,7 +47210,7 @@
     </row>
     <row r="371">
       <c r="A371" t="str">
-        <v>370</v>
+        <v>436</v>
       </c>
       <c r="B371" t="str">
         <v>2024-05-24</v>
@@ -47233,7 +47233,7 @@
     </row>
     <row r="372">
       <c r="A372" t="str">
-        <v>371</v>
+        <v>437</v>
       </c>
       <c r="B372" t="str">
         <v>2024-05-25</v>
@@ -47256,7 +47256,7 @@
     </row>
     <row r="373">
       <c r="A373" t="str">
-        <v>372</v>
+        <v>438</v>
       </c>
       <c r="B373" t="str">
         <v>2024-05-25</v>
@@ -47279,7 +47279,7 @@
     </row>
     <row r="374">
       <c r="A374" t="str">
-        <v>373</v>
+        <v>439</v>
       </c>
       <c r="B374" t="str">
         <v>2024-05-26</v>
@@ -47302,7 +47302,7 @@
     </row>
     <row r="375">
       <c r="A375" t="str">
-        <v>374</v>
+        <v>440</v>
       </c>
       <c r="B375" t="str">
         <v>2024-05-26</v>
@@ -47325,7 +47325,7 @@
     </row>
     <row r="376">
       <c r="A376" t="str">
-        <v>375</v>
+        <v>441</v>
       </c>
       <c r="B376" t="str">
         <v>2024-05-26</v>
@@ -47348,7 +47348,7 @@
     </row>
     <row r="377">
       <c r="A377" t="str">
-        <v>376</v>
+        <v>442</v>
       </c>
       <c r="B377" t="str">
         <v>2024-05-27</v>
@@ -47371,7 +47371,7 @@
     </row>
     <row r="378">
       <c r="A378" t="str">
-        <v>377</v>
+        <v>443</v>
       </c>
       <c r="B378" t="str">
         <v>2024-05-28</v>
@@ -47394,7 +47394,7 @@
     </row>
     <row r="379">
       <c r="A379" t="str">
-        <v>378</v>
+        <v>444</v>
       </c>
       <c r="B379" t="str">
         <v>2024-05-29</v>
@@ -47417,7 +47417,7 @@
     </row>
     <row r="380">
       <c r="A380" t="str">
-        <v>379</v>
+        <v>445</v>
       </c>
       <c r="B380" t="str">
         <v>2024-05-30</v>
@@ -47440,7 +47440,7 @@
     </row>
     <row r="381">
       <c r="A381" t="str">
-        <v>380</v>
+        <v>446</v>
       </c>
       <c r="B381" t="str">
         <v>2024-05-31</v>
@@ -47463,7 +47463,7 @@
     </row>
     <row r="382">
       <c r="A382" t="str">
-        <v>381</v>
+        <v>447</v>
       </c>
       <c r="B382" t="str">
         <v>2024-05-31</v>
@@ -47486,7 +47486,7 @@
     </row>
     <row r="383">
       <c r="A383" t="str">
-        <v>382</v>
+        <v>448</v>
       </c>
       <c r="B383" t="str">
         <v>2024-05-31</v>
@@ -47509,7 +47509,7 @@
     </row>
     <row r="384">
       <c r="A384" t="str">
-        <v>383</v>
+        <v>449</v>
       </c>
       <c r="B384" t="str">
         <v>2024-05-31</v>
@@ -47532,7 +47532,7 @@
     </row>
     <row r="385">
       <c r="A385" t="str">
-        <v>384</v>
+        <v>450</v>
       </c>
       <c r="B385" t="str">
         <v>2024-05-31</v>
@@ -47555,7 +47555,7 @@
     </row>
     <row r="386">
       <c r="A386" t="str">
-        <v>385</v>
+        <v>451</v>
       </c>
       <c r="B386" t="str">
         <v>2024-05-31</v>
@@ -47578,7 +47578,7 @@
     </row>
     <row r="387">
       <c r="A387" t="str">
-        <v>386</v>
+        <v>452</v>
       </c>
       <c r="B387" t="str">
         <v>2024-05-31</v>
@@ -47601,7 +47601,7 @@
     </row>
     <row r="388">
       <c r="A388" t="str">
-        <v>387</v>
+        <v>453</v>
       </c>
       <c r="B388" t="str">
         <v>2024-05-31</v>
@@ -47624,7 +47624,7 @@
     </row>
     <row r="389">
       <c r="A389" t="str">
-        <v>388</v>
+        <v>455</v>
       </c>
       <c r="B389" t="str">
         <v>2024-06-01</v>
@@ -47647,7 +47647,7 @@
     </row>
     <row r="390">
       <c r="A390" t="str">
-        <v>389</v>
+        <v>456</v>
       </c>
       <c r="B390" t="str">
         <v>2024-06-01</v>
@@ -47670,7 +47670,7 @@
     </row>
     <row r="391">
       <c r="A391" t="str">
-        <v>390</v>
+        <v>457</v>
       </c>
       <c r="B391" t="str">
         <v>2024-06-01</v>
@@ -47693,7 +47693,7 @@
     </row>
     <row r="392">
       <c r="A392" t="str">
-        <v>391</v>
+        <v>458</v>
       </c>
       <c r="B392" t="str">
         <v>2024-06-01</v>
@@ -47716,7 +47716,7 @@
     </row>
     <row r="393">
       <c r="A393" t="str">
-        <v>392</v>
+        <v>459</v>
       </c>
       <c r="B393" t="str">
         <v>2024-06-01</v>
@@ -47739,7 +47739,7 @@
     </row>
     <row r="394">
       <c r="A394" t="str">
-        <v>393</v>
+        <v>460</v>
       </c>
       <c r="B394" t="str">
         <v>2024-06-01</v>
@@ -47762,7 +47762,7 @@
     </row>
     <row r="395">
       <c r="A395" t="str">
-        <v>394</v>
+        <v>461</v>
       </c>
       <c r="B395" t="str">
         <v>2024-06-01</v>
@@ -47785,7 +47785,7 @@
     </row>
     <row r="396">
       <c r="A396" t="str">
-        <v>395</v>
+        <v>462</v>
       </c>
       <c r="B396" t="str">
         <v>2024-06-01</v>
@@ -47808,7 +47808,7 @@
     </row>
     <row r="397">
       <c r="A397" t="str">
-        <v>396</v>
+        <v>463</v>
       </c>
       <c r="B397" t="str">
         <v>2024-06-01</v>
@@ -47831,7 +47831,7 @@
     </row>
     <row r="398">
       <c r="A398" t="str">
-        <v>397</v>
+        <v>464</v>
       </c>
       <c r="B398" t="str">
         <v>2024-06-02</v>
@@ -47854,7 +47854,7 @@
     </row>
     <row r="399">
       <c r="A399" t="str">
-        <v>398</v>
+        <v>466</v>
       </c>
       <c r="B399" t="str">
         <v>2024-06-03</v>
@@ -47877,7 +47877,7 @@
     </row>
     <row r="400">
       <c r="A400" t="str">
-        <v>399</v>
+        <v>467</v>
       </c>
       <c r="B400" t="str">
         <v>2024-06-04</v>
@@ -47900,7 +47900,7 @@
     </row>
     <row r="401">
       <c r="A401" t="str">
-        <v>400</v>
+        <v>469</v>
       </c>
       <c r="B401" t="str">
         <v>2024-06-06</v>
@@ -47923,7 +47923,7 @@
     </row>
     <row r="402">
       <c r="A402" t="str">
-        <v>401</v>
+        <v>470</v>
       </c>
       <c r="B402" t="str">
         <v>2024-06-07</v>
@@ -47946,7 +47946,7 @@
     </row>
     <row r="403">
       <c r="A403" t="str">
-        <v>402</v>
+        <v>471</v>
       </c>
       <c r="B403" t="str">
         <v>2024-06-08</v>
@@ -47969,7 +47969,7 @@
     </row>
     <row r="404">
       <c r="A404" t="str">
-        <v>403</v>
+        <v>472</v>
       </c>
       <c r="B404" t="str">
         <v>2024-06-08</v>
@@ -47992,7 +47992,7 @@
     </row>
     <row r="405">
       <c r="A405" t="str">
-        <v>404</v>
+        <v>473</v>
       </c>
       <c r="B405" t="str">
         <v>2024-06-08</v>
@@ -48015,7 +48015,7 @@
     </row>
     <row r="406">
       <c r="A406" t="str">
-        <v>405</v>
+        <v>474</v>
       </c>
       <c r="B406" t="str">
         <v>2024-06-08</v>
@@ -48038,7 +48038,7 @@
     </row>
     <row r="407">
       <c r="A407" t="str">
-        <v>406</v>
+        <v>475</v>
       </c>
       <c r="B407" t="str">
         <v>2024-06-08</v>
@@ -48061,7 +48061,7 @@
     </row>
     <row r="408">
       <c r="A408" t="str">
-        <v>407</v>
+        <v>476</v>
       </c>
       <c r="B408" t="str">
         <v>2024-06-08</v>
@@ -48084,7 +48084,7 @@
     </row>
     <row r="409">
       <c r="A409" t="str">
-        <v>408</v>
+        <v>477</v>
       </c>
       <c r="B409" t="str">
         <v>2024-06-08</v>
@@ -48107,7 +48107,7 @@
     </row>
     <row r="410">
       <c r="A410" t="str">
-        <v>409</v>
+        <v>478</v>
       </c>
       <c r="B410" t="str">
         <v>2024-06-08</v>
@@ -48130,7 +48130,7 @@
     </row>
     <row r="411">
       <c r="A411" t="str">
-        <v>410</v>
+        <v>479</v>
       </c>
       <c r="B411" t="str">
         <v>2024-06-08</v>
@@ -48153,7 +48153,7 @@
     </row>
     <row r="412">
       <c r="A412" t="str">
-        <v>411</v>
+        <v>480</v>
       </c>
       <c r="B412" t="str">
         <v>2024-06-08</v>
@@ -48176,7 +48176,7 @@
     </row>
     <row r="413">
       <c r="A413" t="str">
-        <v>412</v>
+        <v>481</v>
       </c>
       <c r="B413" t="str">
         <v>2024-06-08</v>
@@ -48199,7 +48199,7 @@
     </row>
     <row r="414">
       <c r="A414" t="str">
-        <v>413</v>
+        <v>482</v>
       </c>
       <c r="B414" t="str">
         <v>2024-06-09</v>
@@ -48222,7 +48222,7 @@
     </row>
     <row r="415">
       <c r="A415" t="str">
-        <v>414</v>
+        <v>483</v>
       </c>
       <c r="B415" t="str">
         <v>2024-06-10</v>
@@ -48245,7 +48245,7 @@
     </row>
     <row r="416">
       <c r="A416" t="str">
-        <v>415</v>
+        <v>484</v>
       </c>
       <c r="B416" t="str">
         <v>2024-06-11</v>
@@ -48268,7 +48268,7 @@
     </row>
     <row r="417">
       <c r="A417" t="str">
-        <v>416</v>
+        <v>485</v>
       </c>
       <c r="B417" t="str">
         <v>2024-06-12</v>
@@ -48291,7 +48291,7 @@
     </row>
     <row r="418">
       <c r="A418" t="str">
-        <v>417</v>
+        <v>486</v>
       </c>
       <c r="B418" t="str">
         <v>2024-06-13</v>
@@ -48314,7 +48314,7 @@
     </row>
     <row r="419">
       <c r="A419" t="str">
-        <v>418</v>
+        <v>487</v>
       </c>
       <c r="B419" t="str">
         <v>2024-06-14</v>
@@ -48337,7 +48337,7 @@
     </row>
     <row r="420">
       <c r="A420" t="str">
-        <v>419</v>
+        <v>488</v>
       </c>
       <c r="B420" t="str">
         <v>2024-06-16</v>
@@ -48360,7 +48360,7 @@
     </row>
     <row r="421">
       <c r="A421" t="str">
-        <v>420</v>
+        <v>489</v>
       </c>
       <c r="B421" t="str">
         <v>2024-06-17</v>
@@ -48383,7 +48383,7 @@
     </row>
     <row r="422">
       <c r="A422" t="str">
-        <v>421</v>
+        <v>490</v>
       </c>
       <c r="B422" t="str">
         <v>2024-06-18</v>
@@ -48406,7 +48406,7 @@
     </row>
     <row r="423">
       <c r="A423" t="str">
-        <v>422</v>
+        <v>491</v>
       </c>
       <c r="B423" t="str">
         <v>2024-06-20</v>
@@ -48429,7 +48429,7 @@
     </row>
     <row r="424">
       <c r="A424" t="str">
-        <v>423</v>
+        <v>493</v>
       </c>
       <c r="B424" t="str">
         <v>2024-07-01</v>
@@ -48452,7 +48452,7 @@
     </row>
     <row r="425">
       <c r="A425" t="str">
-        <v>424</v>
+        <v>494</v>
       </c>
       <c r="B425" t="str">
         <v>2024-07-01</v>
@@ -48475,7 +48475,7 @@
     </row>
     <row r="426">
       <c r="A426" t="str">
-        <v>425</v>
+        <v>495</v>
       </c>
       <c r="B426" t="str">
         <v>2024-07-01</v>
@@ -48498,7 +48498,7 @@
     </row>
     <row r="427">
       <c r="A427" t="str">
-        <v>426</v>
+        <v>497</v>
       </c>
       <c r="B427" t="str">
         <v>2024-10-05</v>
@@ -48521,7 +48521,7 @@
     </row>
     <row r="428">
       <c r="A428" t="str">
-        <v>427</v>
+        <v>498</v>
       </c>
       <c r="B428" t="str">
         <v>2024-10-05</v>
@@ -48544,7 +48544,7 @@
     </row>
     <row r="429">
       <c r="A429" t="str">
-        <v>428</v>
+        <v>499</v>
       </c>
       <c r="B429" t="str">
         <v>2024-10-05</v>
@@ -48567,7 +48567,7 @@
     </row>
     <row r="430">
       <c r="A430" t="str">
-        <v>429</v>
+        <v>500</v>
       </c>
       <c r="B430" t="str">
         <v>2024-10-05</v>
@@ -48590,7 +48590,7 @@
     </row>
     <row r="431">
       <c r="A431" t="str">
-        <v>430</v>
+        <v>501</v>
       </c>
       <c r="B431" t="str">
         <v>2024-10-05</v>
@@ -48613,7 +48613,7 @@
     </row>
     <row r="432">
       <c r="A432" t="str">
-        <v>431</v>
+        <v>502</v>
       </c>
       <c r="B432" t="str">
         <v>2024-10-05</v>
@@ -48636,7 +48636,7 @@
     </row>
     <row r="433">
       <c r="A433" t="str">
-        <v>432</v>
+        <v>503</v>
       </c>
       <c r="B433" t="str">
         <v>2024-10-05</v>
@@ -48659,7 +48659,7 @@
     </row>
     <row r="434">
       <c r="A434" t="str">
-        <v>433</v>
+        <v>511</v>
       </c>
       <c r="B434" t="str">
         <v>2024-11-17</v>
@@ -48682,7 +48682,7 @@
     </row>
     <row r="435">
       <c r="A435" t="str">
-        <v>434</v>
+        <v>512</v>
       </c>
       <c r="B435" t="str">
         <v>2024-11-18</v>
@@ -48705,7 +48705,7 @@
     </row>
     <row r="436">
       <c r="A436" t="str">
-        <v>435</v>
+        <v>516</v>
       </c>
       <c r="B436" t="str">
         <v>2024-12-07</v>
@@ -48728,7 +48728,7 @@
     </row>
     <row r="437">
       <c r="A437" t="str">
-        <v>436</v>
+        <v>517</v>
       </c>
       <c r="B437" t="str">
         <v>2024-12-08</v>
@@ -48751,7 +48751,7 @@
     </row>
     <row r="438">
       <c r="A438" t="str">
-        <v>437</v>
+        <v>518</v>
       </c>
       <c r="B438" t="str">
         <v>2024-12-08</v>
@@ -48774,7 +48774,7 @@
     </row>
     <row r="439">
       <c r="A439" t="str">
-        <v>438</v>
+        <v>519</v>
       </c>
       <c r="B439" t="str">
         <v>2024-12-09</v>
@@ -48797,7 +48797,7 @@
     </row>
     <row r="440">
       <c r="A440" t="str">
-        <v>439</v>
+        <v>520</v>
       </c>
       <c r="B440" t="str">
         <v>2024-12-17</v>
@@ -48820,7 +48820,7 @@
     </row>
     <row r="441">
       <c r="A441" t="str">
-        <v>440</v>
+        <v>521</v>
       </c>
       <c r="B441" t="str">
         <v>2024-12-18</v>
@@ -48843,7 +48843,7 @@
     </row>
     <row r="442">
       <c r="A442" t="str">
-        <v>441</v>
+        <v>522</v>
       </c>
       <c r="B442" t="str">
         <v>2024-12-20</v>
@@ -48866,7 +48866,7 @@
     </row>
     <row r="443">
       <c r="A443" t="str">
-        <v>442</v>
+        <v>523</v>
       </c>
       <c r="B443" t="str">
         <v>2024-12-21</v>
@@ -48889,7 +48889,7 @@
     </row>
     <row r="444">
       <c r="A444" t="str">
-        <v>443</v>
+        <v>524</v>
       </c>
       <c r="B444" t="str">
         <v>2024-12-21</v>
@@ -48912,7 +48912,7 @@
     </row>
     <row r="445">
       <c r="A445" t="str">
-        <v>444</v>
+        <v>525</v>
       </c>
       <c r="B445" t="str">
         <v>2024-12-25</v>
@@ -48935,7 +48935,7 @@
     </row>
     <row r="446">
       <c r="A446" t="str">
-        <v>445</v>
+        <v>526</v>
       </c>
       <c r="B446" t="str">
         <v>2024-12-26</v>
@@ -48958,7 +48958,7 @@
     </row>
     <row r="447">
       <c r="A447" t="str">
-        <v>446</v>
+        <v>528</v>
       </c>
       <c r="B447" t="str">
         <v>2024-12-31</v>
@@ -48981,7 +48981,7 @@
     </row>
     <row r="448">
       <c r="A448" t="str">
-        <v>447</v>
+        <v>529</v>
       </c>
       <c r="B448" t="str">
         <v>2025-01-02</v>
@@ -49004,7 +49004,7 @@
     </row>
     <row r="449">
       <c r="A449" t="str">
-        <v>448</v>
+        <v>530</v>
       </c>
       <c r="B449" t="str">
         <v>2025-01-02</v>
@@ -49027,7 +49027,7 @@
     </row>
     <row r="450">
       <c r="A450" t="str">
-        <v>449</v>
+        <v>531</v>
       </c>
       <c r="B450" t="str">
         <v>2025-01-02</v>
@@ -49050,7 +49050,7 @@
     </row>
     <row r="451">
       <c r="A451" t="str">
-        <v>450</v>
+        <v>532</v>
       </c>
       <c r="B451" t="str">
         <v>2025-01-02</v>
@@ -49073,7 +49073,7 @@
     </row>
     <row r="452">
       <c r="A452" t="str">
-        <v>451</v>
+        <v>533</v>
       </c>
       <c r="B452" t="str">
         <v>2025-01-02</v>
@@ -49096,7 +49096,7 @@
     </row>
     <row r="453">
       <c r="A453" t="str">
-        <v>452</v>
+        <v>534</v>
       </c>
       <c r="B453" t="str">
         <v>2025-01-03</v>
@@ -49119,7 +49119,7 @@
     </row>
     <row r="454">
       <c r="A454" t="str">
-        <v>453</v>
+        <v>535</v>
       </c>
       <c r="B454" t="str">
         <v>2025-01-03</v>
@@ -49142,7 +49142,7 @@
     </row>
     <row r="455">
       <c r="A455" t="str">
-        <v>454</v>
+        <v>536</v>
       </c>
       <c r="B455" t="str">
         <v>2025-01-03</v>
@@ -49165,7 +49165,7 @@
     </row>
     <row r="456">
       <c r="A456" t="str">
-        <v>455</v>
+        <v>537</v>
       </c>
       <c r="B456" t="str">
         <v>2025-01-05</v>
@@ -49188,7 +49188,7 @@
     </row>
     <row r="457">
       <c r="A457" t="str">
-        <v>456</v>
+        <v>541</v>
       </c>
       <c r="B457" t="str">
         <v>2025-03-08</v>
@@ -49211,7 +49211,7 @@
     </row>
     <row r="458">
       <c r="A458" t="str">
-        <v>457</v>
+        <v>542</v>
       </c>
       <c r="B458" t="str">
         <v>2025-03-09</v>
@@ -49234,7 +49234,7 @@
     </row>
     <row r="459">
       <c r="A459" t="str">
-        <v>458</v>
+        <v>543</v>
       </c>
       <c r="B459" t="str">
         <v>2025-03-09</v>
@@ -49257,7 +49257,7 @@
     </row>
     <row r="460">
       <c r="A460" t="str">
-        <v>459</v>
+        <v>544</v>
       </c>
       <c r="B460" t="str">
         <v>2025-03-10</v>
@@ -49280,7 +49280,7 @@
     </row>
     <row r="461">
       <c r="A461" t="str">
-        <v>460</v>
+        <v>545</v>
       </c>
       <c r="B461" t="str">
         <v>2025-03-10</v>
@@ -49303,7 +49303,7 @@
     </row>
     <row r="462">
       <c r="A462" t="str">
-        <v>461</v>
+        <v>547</v>
       </c>
       <c r="B462" t="str">
         <v>2025-03-11</v>
@@ -49326,7 +49326,7 @@
     </row>
     <row r="463">
       <c r="A463" t="str">
-        <v>462</v>
+        <v>548</v>
       </c>
       <c r="B463" t="str">
         <v>2025-03-12</v>
@@ -49349,7 +49349,7 @@
     </row>
     <row r="464">
       <c r="A464" t="str">
-        <v>463</v>
+        <v>549</v>
       </c>
       <c r="B464" t="str">
         <v>2025-03-13</v>
@@ -49372,7 +49372,7 @@
     </row>
     <row r="465">
       <c r="A465" t="str">
-        <v>464</v>
+        <v>550</v>
       </c>
       <c r="B465" t="str">
         <v>2025-03-13</v>
@@ -49395,7 +49395,7 @@
     </row>
     <row r="466">
       <c r="A466" t="str">
-        <v>465</v>
+        <v>551</v>
       </c>
       <c r="B466" t="str">
         <v>2025-03-13</v>
@@ -49418,7 +49418,7 @@
     </row>
     <row r="467">
       <c r="A467" t="str">
-        <v>466</v>
+        <v>552</v>
       </c>
       <c r="B467" t="str">
         <v>2025-03-13</v>
@@ -49441,7 +49441,7 @@
     </row>
     <row r="468">
       <c r="A468" t="str">
-        <v>467</v>
+        <v>553</v>
       </c>
       <c r="B468" t="str">
         <v>2025-03-13</v>
@@ -49464,7 +49464,7 @@
     </row>
     <row r="469">
       <c r="A469" t="str">
-        <v>468</v>
+        <v>554</v>
       </c>
       <c r="B469" t="str">
         <v>2025-03-16</v>
@@ -49487,7 +49487,7 @@
     </row>
     <row r="470">
       <c r="A470" t="str">
-        <v>469</v>
+        <v>555</v>
       </c>
       <c r="B470" t="str">
         <v>2025-03-17</v>
@@ -49510,7 +49510,7 @@
     </row>
     <row r="471">
       <c r="A471" t="str">
-        <v>470</v>
+        <v>556</v>
       </c>
       <c r="B471" t="str">
         <v>2025-03-18</v>
@@ -49533,7 +49533,7 @@
     </row>
     <row r="472">
       <c r="A472" t="str">
-        <v>471</v>
+        <v>557</v>
       </c>
       <c r="B472" t="str">
         <v>2025-03-18</v>
@@ -49556,7 +49556,7 @@
     </row>
     <row r="473">
       <c r="A473" t="str">
-        <v>472</v>
+        <v>558</v>
       </c>
       <c r="B473" t="str">
         <v>2025-03-19</v>
@@ -49579,7 +49579,7 @@
     </row>
     <row r="474">
       <c r="A474" t="str">
-        <v>473</v>
+        <v>559</v>
       </c>
       <c r="B474" t="str">
         <v>2025-03-20</v>
@@ -49602,7 +49602,7 @@
     </row>
     <row r="475">
       <c r="A475" t="str">
-        <v>474</v>
+        <v>560</v>
       </c>
       <c r="B475" t="str">
         <v>2025-03-21</v>
@@ -49625,7 +49625,7 @@
     </row>
     <row r="476">
       <c r="A476" t="str">
-        <v>475</v>
+        <v>561</v>
       </c>
       <c r="B476" t="str">
         <v>2025-03-21</v>
@@ -49648,7 +49648,7 @@
     </row>
     <row r="477">
       <c r="A477" t="str">
-        <v>476</v>
+        <v>562</v>
       </c>
       <c r="B477" t="str">
         <v>2025-03-21</v>
@@ -49671,7 +49671,7 @@
     </row>
     <row r="478">
       <c r="A478" t="str">
-        <v>477</v>
+        <v>563</v>
       </c>
       <c r="B478" t="str">
         <v>2025-03-23</v>
@@ -49694,7 +49694,7 @@
     </row>
     <row r="479">
       <c r="A479" t="str">
-        <v>478</v>
+        <v>564</v>
       </c>
       <c r="B479" t="str">
         <v>2025-03-24</v>
@@ -49717,7 +49717,7 @@
     </row>
     <row r="480">
       <c r="A480" t="str">
-        <v>479</v>
+        <v>565</v>
       </c>
       <c r="B480" t="str">
         <v>2025-03-25</v>
@@ -49740,7 +49740,7 @@
     </row>
     <row r="481">
       <c r="A481" t="str">
-        <v>480</v>
+        <v>566</v>
       </c>
       <c r="B481" t="str">
         <v>2025-03-25</v>
@@ -49763,7 +49763,7 @@
     </row>
     <row r="482">
       <c r="A482" t="str">
-        <v>481</v>
+        <v>567</v>
       </c>
       <c r="B482" t="str">
         <v>2025-03-25</v>
@@ -49786,7 +49786,7 @@
     </row>
     <row r="483">
       <c r="A483" t="str">
-        <v>482</v>
+        <v>568</v>
       </c>
       <c r="B483" t="str">
         <v>2025-03-25</v>
@@ -49809,7 +49809,7 @@
     </row>
     <row r="484">
       <c r="A484" t="str">
-        <v>483</v>
+        <v>569</v>
       </c>
       <c r="B484" t="str">
         <v>2025-03-27</v>
@@ -49832,7 +49832,7 @@
     </row>
     <row r="485">
       <c r="A485" t="str">
-        <v>484</v>
+        <v>570</v>
       </c>
       <c r="B485" t="str">
         <v>2025-03-28</v>
@@ -49855,7 +49855,7 @@
     </row>
     <row r="486">
       <c r="A486" t="str">
-        <v>485</v>
+        <v>571</v>
       </c>
       <c r="B486" t="str">
         <v>2025-03-29</v>
@@ -49878,7 +49878,7 @@
     </row>
     <row r="487">
       <c r="A487" t="str">
-        <v>486</v>
+        <v>572</v>
       </c>
       <c r="B487" t="str">
         <v>2025-03-31</v>
@@ -49901,7 +49901,7 @@
     </row>
     <row r="488">
       <c r="A488" t="str">
-        <v>487</v>
+        <v>573</v>
       </c>
       <c r="B488" t="str">
         <v>2025-03-31</v>
@@ -49924,7 +49924,7 @@
     </row>
     <row r="489">
       <c r="A489" t="str">
-        <v>488</v>
+        <v>574</v>
       </c>
       <c r="B489" t="str">
         <v>2025-03-31</v>
@@ -49947,7 +49947,7 @@
     </row>
     <row r="490">
       <c r="A490" t="str">
-        <v>489</v>
+        <v>575</v>
       </c>
       <c r="B490" t="str">
         <v>2025-04-01</v>
@@ -49970,7 +49970,7 @@
     </row>
     <row r="491">
       <c r="A491" t="str">
-        <v>490</v>
+        <v>576</v>
       </c>
       <c r="B491" t="str">
         <v>2025-04-01</v>
@@ -49993,7 +49993,7 @@
     </row>
     <row r="492">
       <c r="A492" t="str">
-        <v>491</v>
+        <v>577</v>
       </c>
       <c r="B492" t="str">
         <v>2025-04-01</v>
@@ -50016,7 +50016,7 @@
     </row>
     <row r="493">
       <c r="A493" t="str">
-        <v>492</v>
+        <v>578</v>
       </c>
       <c r="B493" t="str">
         <v>2025-04-01</v>
@@ -50039,7 +50039,7 @@
     </row>
     <row r="494">
       <c r="A494" t="str">
-        <v>493</v>
+        <v>579</v>
       </c>
       <c r="B494" t="str">
         <v>2025-04-01</v>
@@ -50062,7 +50062,7 @@
     </row>
     <row r="495">
       <c r="A495" t="str">
-        <v>494</v>
+        <v>581</v>
       </c>
       <c r="B495" t="str">
         <v>2025-04-02</v>
@@ -50085,7 +50085,7 @@
     </row>
     <row r="496">
       <c r="A496" t="str">
-        <v>495</v>
+        <v>582</v>
       </c>
       <c r="B496" t="str">
         <v>2025-04-02</v>
@@ -50108,7 +50108,7 @@
     </row>
     <row r="497">
       <c r="A497" t="str">
-        <v>496</v>
+        <v>583</v>
       </c>
       <c r="B497" t="str">
         <v>2025-04-05</v>
@@ -50131,7 +50131,7 @@
     </row>
     <row r="498">
       <c r="A498" t="str">
-        <v>497</v>
+        <v>584</v>
       </c>
       <c r="B498" t="str">
         <v>2025-04-06</v>
@@ -50154,7 +50154,7 @@
     </row>
     <row r="499">
       <c r="A499" t="str">
-        <v>498</v>
+        <v>585</v>
       </c>
       <c r="B499" t="str">
         <v>2025-04-07</v>
@@ -50177,7 +50177,7 @@
     </row>
     <row r="500">
       <c r="A500" t="str">
-        <v>499</v>
+        <v>586</v>
       </c>
       <c r="B500" t="str">
         <v>2025-04-08</v>
@@ -50200,7 +50200,7 @@
     </row>
     <row r="501">
       <c r="A501" t="str">
-        <v>500</v>
+        <v>587</v>
       </c>
       <c r="B501" t="str">
         <v>2025-04-08</v>
@@ -50223,7 +50223,7 @@
     </row>
     <row r="502">
       <c r="A502" t="str">
-        <v>501</v>
+        <v>588</v>
       </c>
       <c r="B502" t="str">
         <v>2025-04-09</v>
@@ -50246,7 +50246,7 @@
     </row>
     <row r="503">
       <c r="A503" t="str">
-        <v>502</v>
+        <v>589</v>
       </c>
       <c r="B503" t="str">
         <v>2025-04-09</v>
@@ -50269,7 +50269,7 @@
     </row>
     <row r="504">
       <c r="A504" t="str">
-        <v>503</v>
+        <v>590</v>
       </c>
       <c r="B504" t="str">
         <v>2025-04-11</v>
@@ -50292,7 +50292,7 @@
     </row>
     <row r="505">
       <c r="A505" t="str">
-        <v>504</v>
+        <v>591</v>
       </c>
       <c r="B505" t="str">
         <v>2025-04-12</v>
@@ -50315,7 +50315,7 @@
     </row>
     <row r="506">
       <c r="A506" t="str">
-        <v>505</v>
+        <v>592</v>
       </c>
       <c r="B506" t="str">
         <v>2025-04-13</v>
@@ -50338,7 +50338,7 @@
     </row>
     <row r="507">
       <c r="A507" t="str">
-        <v>506</v>
+        <v>593</v>
       </c>
       <c r="B507" t="str">
         <v>2025-04-14</v>
@@ -50361,7 +50361,7 @@
     </row>
     <row r="508">
       <c r="A508" t="str">
-        <v>507</v>
+        <v>594</v>
       </c>
       <c r="B508" t="str">
         <v>2025-04-14</v>
@@ -50384,7 +50384,7 @@
     </row>
     <row r="509">
       <c r="A509" t="str">
-        <v>508</v>
+        <v>595</v>
       </c>
       <c r="B509" t="str">
         <v>2025-04-18</v>
@@ -50407,7 +50407,7 @@
     </row>
     <row r="510">
       <c r="A510" t="str">
-        <v>509</v>
+        <v>596</v>
       </c>
       <c r="B510" t="str">
         <v>2025-04-20</v>
@@ -50430,7 +50430,7 @@
     </row>
     <row r="511">
       <c r="A511" t="str">
-        <v>510</v>
+        <v>597</v>
       </c>
       <c r="B511" t="str">
         <v>2025-04-21</v>
@@ -50453,7 +50453,7 @@
     </row>
     <row r="512">
       <c r="A512" t="str">
-        <v>511</v>
+        <v>598</v>
       </c>
       <c r="B512" t="str">
         <v>2025-04-22</v>
@@ -50476,7 +50476,7 @@
     </row>
     <row r="513">
       <c r="A513" t="str">
-        <v>512</v>
+        <v>599</v>
       </c>
       <c r="B513" t="str">
         <v>2025-04-22</v>
@@ -50499,7 +50499,7 @@
     </row>
     <row r="514">
       <c r="A514" t="str">
-        <v>513</v>
+        <v>600</v>
       </c>
       <c r="B514" t="str">
         <v>2025-04-23</v>
@@ -50522,7 +50522,7 @@
     </row>
     <row r="515">
       <c r="A515" t="str">
-        <v>514</v>
+        <v>601</v>
       </c>
       <c r="B515" t="str">
         <v>2025-04-24</v>
@@ -50545,7 +50545,7 @@
     </row>
     <row r="516">
       <c r="A516" t="str">
-        <v>515</v>
+        <v>604</v>
       </c>
       <c r="B516" t="str">
         <v>2025-04-27</v>
@@ -50568,7 +50568,7 @@
     </row>
     <row r="517">
       <c r="A517" t="str">
-        <v>516</v>
+        <v>605</v>
       </c>
       <c r="B517" t="str">
         <v>2025-04-28</v>
@@ -50591,7 +50591,7 @@
     </row>
     <row r="518">
       <c r="A518" t="str">
-        <v>517</v>
+        <v>606</v>
       </c>
       <c r="B518" t="str">
         <v>2025-04-29</v>
@@ -50614,7 +50614,7 @@
     </row>
     <row r="519">
       <c r="A519" t="str">
-        <v>518</v>
+        <v>608</v>
       </c>
       <c r="B519" t="str">
         <v>2025-05-01</v>
@@ -50637,7 +50637,7 @@
     </row>
     <row r="520">
       <c r="A520" t="str">
-        <v>519</v>
+        <v>609</v>
       </c>
       <c r="B520" t="str">
         <v>2025-05-01</v>
@@ -50660,7 +50660,7 @@
     </row>
     <row r="521">
       <c r="A521" t="str">
-        <v>520</v>
+        <v>610</v>
       </c>
       <c r="B521" t="str">
         <v>2025-05-01</v>
@@ -50683,7 +50683,7 @@
     </row>
     <row r="522">
       <c r="A522" t="str">
-        <v>521</v>
+        <v>611</v>
       </c>
       <c r="B522" t="str">
         <v>2025-05-01</v>
@@ -50706,7 +50706,7 @@
     </row>
     <row r="523">
       <c r="A523" t="str">
-        <v>522</v>
+        <v>613</v>
       </c>
       <c r="B523" t="str">
         <v>2025-05-03</v>
@@ -50729,7 +50729,7 @@
     </row>
     <row r="524">
       <c r="A524" t="str">
-        <v>523</v>
+        <v>614</v>
       </c>
       <c r="B524" t="str">
         <v>2025-05-04</v>
@@ -50752,7 +50752,7 @@
     </row>
     <row r="525">
       <c r="A525" t="str">
-        <v>524</v>
+        <v>618</v>
       </c>
       <c r="B525" t="str">
         <v>2025-05-06</v>
@@ -50775,7 +50775,7 @@
     </row>
     <row r="526">
       <c r="A526" t="str">
-        <v>525</v>
+        <v>619</v>
       </c>
       <c r="B526" t="str">
         <v>2025-05-07</v>
@@ -50798,7 +50798,7 @@
     </row>
     <row r="527">
       <c r="A527" t="str">
-        <v>526</v>
+        <v>623</v>
       </c>
       <c r="B527" t="str">
         <v>2025-05-11</v>
@@ -50821,7 +50821,7 @@
     </row>
     <row r="528">
       <c r="A528" t="str">
-        <v>527</v>
+        <v>624</v>
       </c>
       <c r="B528" t="str">
         <v>2025-05-13</v>
@@ -50844,7 +50844,7 @@
     </row>
     <row r="529">
       <c r="A529" t="str">
-        <v>528</v>
+        <v>626</v>
       </c>
       <c r="B529" t="str">
         <v>2025-05-15</v>
@@ -50867,7 +50867,7 @@
     </row>
     <row r="530">
       <c r="A530" t="str">
-        <v>529</v>
+        <v>627</v>
       </c>
       <c r="B530" t="str">
         <v>2025-05-16</v>
@@ -50890,7 +50890,7 @@
     </row>
     <row r="531">
       <c r="A531" t="str">
-        <v>530</v>
+        <v>628</v>
       </c>
       <c r="B531" t="str">
         <v>2025-05-18</v>
@@ -50913,7 +50913,7 @@
     </row>
     <row r="532">
       <c r="A532" t="str">
-        <v>531</v>
+        <v>629</v>
       </c>
       <c r="B532" t="str">
         <v>2025-05-19</v>
@@ -50936,7 +50936,7 @@
     </row>
     <row r="533">
       <c r="A533" t="str">
-        <v>532</v>
+        <v>630</v>
       </c>
       <c r="B533" t="str">
         <v>2025-05-20</v>
@@ -50959,7 +50959,7 @@
     </row>
     <row r="534">
       <c r="A534" t="str">
-        <v>533</v>
+        <v>631</v>
       </c>
       <c r="B534" t="str">
         <v>2025-05-22</v>
@@ -50982,7 +50982,7 @@
     </row>
     <row r="535">
       <c r="A535" t="str">
-        <v>534</v>
+        <v>632</v>
       </c>
       <c r="B535" t="str">
         <v>2025-05-23</v>
@@ -51005,7 +51005,7 @@
     </row>
     <row r="536">
       <c r="A536" t="str">
-        <v>535</v>
+        <v>633</v>
       </c>
       <c r="B536" t="str">
         <v>2025-05-26</v>
@@ -51028,7 +51028,7 @@
     </row>
     <row r="537">
       <c r="A537" t="str">
-        <v>536</v>
+        <v>634</v>
       </c>
       <c r="B537" t="str">
         <v>2025-05-27</v>
@@ -51051,7 +51051,7 @@
     </row>
     <row r="538">
       <c r="A538" t="str">
-        <v>537</v>
+        <v>635</v>
       </c>
       <c r="B538" t="str">
         <v>2025-05-29</v>
@@ -51074,7 +51074,7 @@
     </row>
     <row r="539">
       <c r="A539" t="str">
-        <v>538</v>
+        <v>636</v>
       </c>
       <c r="B539" t="str">
         <v>2025-05-30</v>
@@ -51097,7 +51097,7 @@
     </row>
     <row r="540">
       <c r="A540" t="str">
-        <v>539</v>
+        <v>637</v>
       </c>
       <c r="B540" t="str">
         <v>2025-05-30</v>
@@ -51120,7 +51120,7 @@
     </row>
     <row r="541">
       <c r="A541" t="str">
-        <v>540</v>
+        <v>638</v>
       </c>
       <c r="B541" t="str">
         <v>2025-05-30</v>
@@ -51143,7 +51143,7 @@
     </row>
     <row r="542">
       <c r="A542" t="str">
-        <v>541</v>
+        <v>639</v>
       </c>
       <c r="B542" t="str">
         <v>2025-06-01</v>
@@ -51166,7 +51166,7 @@
     </row>
     <row r="543">
       <c r="A543" t="str">
-        <v>542</v>
+        <v>640</v>
       </c>
       <c r="B543" t="str">
         <v>2025-06-02</v>
@@ -51189,7 +51189,7 @@
     </row>
     <row r="544">
       <c r="A544" t="str">
-        <v>543</v>
+        <v>641</v>
       </c>
       <c r="B544" t="str">
         <v>2025-06-05</v>
@@ -51212,7 +51212,7 @@
     </row>
     <row r="545">
       <c r="A545" t="str">
-        <v>544</v>
+        <v>642</v>
       </c>
       <c r="B545" t="str">
         <v>2025-06-09</v>
@@ -51235,7 +51235,7 @@
     </row>
     <row r="546">
       <c r="A546" t="str">
-        <v>545</v>
+        <v>643</v>
       </c>
       <c r="B546" t="str">
         <v>2025-06-10</v>
@@ -51258,7 +51258,7 @@
     </row>
     <row r="547">
       <c r="A547" t="str">
-        <v>546</v>
+        <v>644</v>
       </c>
       <c r="B547" t="str">
         <v>2025-06-10</v>
@@ -51281,7 +51281,7 @@
     </row>
     <row r="548">
       <c r="A548" t="str">
-        <v>547</v>
+        <v>645</v>
       </c>
       <c r="B548" t="str">
         <v>2025-06-10</v>
@@ -51304,7 +51304,7 @@
     </row>
     <row r="549">
       <c r="A549" t="str">
-        <v>548</v>
+        <v>646</v>
       </c>
       <c r="B549" t="str">
         <v>2025-06-10</v>
@@ -51327,7 +51327,7 @@
     </row>
     <row r="550">
       <c r="A550" t="str">
-        <v>549</v>
+        <v>647</v>
       </c>
       <c r="B550" t="str">
         <v>2025-06-10</v>
@@ -51350,7 +51350,7 @@
     </row>
     <row r="551">
       <c r="A551" t="str">
-        <v>550</v>
+        <v>648</v>
       </c>
       <c r="B551" t="str">
         <v>2025-06-10</v>
@@ -51373,7 +51373,7 @@
     </row>
     <row r="552">
       <c r="A552" t="str">
-        <v>551</v>
+        <v>649</v>
       </c>
       <c r="B552" t="str">
         <v>2025-06-10</v>
@@ -51396,7 +51396,7 @@
     </row>
     <row r="553">
       <c r="A553" t="str">
-        <v>552</v>
+        <v>650</v>
       </c>
       <c r="B553" t="str">
         <v>2025-06-10</v>
@@ -51419,7 +51419,7 @@
     </row>
     <row r="554">
       <c r="A554" t="str">
-        <v>553</v>
+        <v>651</v>
       </c>
       <c r="B554" t="str">
         <v>2025-06-10</v>
@@ -51442,7 +51442,7 @@
     </row>
     <row r="555">
       <c r="A555" t="str">
-        <v>554</v>
+        <v>652</v>
       </c>
       <c r="B555" t="str">
         <v>2025-06-10</v>
@@ -51465,7 +51465,7 @@
     </row>
     <row r="556">
       <c r="A556" t="str">
-        <v>555</v>
+        <v>653</v>
       </c>
       <c r="B556" t="str">
         <v>2025-06-10</v>
@@ -51488,7 +51488,7 @@
     </row>
     <row r="557">
       <c r="A557" t="str">
-        <v>556</v>
+        <v>654</v>
       </c>
       <c r="B557" t="str">
         <v>2025-06-10</v>

</xml_diff>

<commit_message>
Enhance Gitai application with new search functionality for income and expense filters in index.html. Update JavaScript files to support search queries in income and expense modules. Increment data snapshot version in config.js. Add new expense tracking images and documents, along with JSON files for M2 expenses. Update existing Excel workbooks to reflect recent changes and improve overall data management.
</commit_message>
<xml_diff>
--- a/Gitai-M1.xlsx
+++ b/Gitai-M1.xlsx
@@ -468,7 +468,7 @@
         <v>Gitai.xlsx</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-07-31T17:48:11.960Z</v>
+        <v>2026-07-31T18:48:06.318Z</v>
       </c>
       <c r="E2">
         <v>1174</v>
@@ -46313,7 +46313,7 @@
     </row>
     <row r="332">
       <c r="A332" t="str">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B332" t="str">
         <v>2023-01-19</v>
@@ -46336,7 +46336,7 @@
     </row>
     <row r="333">
       <c r="A333" t="str">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B333" t="str">
         <v>2023-01-20</v>
@@ -46359,7 +46359,7 @@
     </row>
     <row r="334">
       <c r="A334" t="str">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B334" t="str">
         <v>2023-01-21</v>
@@ -46382,7 +46382,7 @@
     </row>
     <row r="335">
       <c r="A335" t="str">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="B335" t="str">
         <v>2023-01-22</v>
@@ -46405,7 +46405,7 @@
     </row>
     <row r="336">
       <c r="A336" t="str">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="B336" t="str">
         <v>2023-01-24</v>
@@ -46428,7 +46428,7 @@
     </row>
     <row r="337">
       <c r="A337" t="str">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="B337" t="str">
         <v>2023-01-25</v>
@@ -46451,7 +46451,7 @@
     </row>
     <row r="338">
       <c r="A338" t="str">
-        <v>343</v>
+        <v>355</v>
       </c>
       <c r="B338" t="str">
         <v>2023-01-28</v>
@@ -46474,7 +46474,7 @@
     </row>
     <row r="339">
       <c r="A339" t="str">
-        <v>344</v>
+        <v>356</v>
       </c>
       <c r="B339" t="str">
         <v>2023-01-29</v>
@@ -46497,7 +46497,7 @@
     </row>
     <row r="340">
       <c r="A340" t="str">
-        <v>345</v>
+        <v>357</v>
       </c>
       <c r="B340" t="str">
         <v>2023-01-30</v>
@@ -46520,7 +46520,7 @@
     </row>
     <row r="341">
       <c r="A341" t="str">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="B341" t="str">
         <v>2023-01-30</v>
@@ -46543,7 +46543,7 @@
     </row>
     <row r="342">
       <c r="A342" t="str">
-        <v>347</v>
+        <v>359</v>
       </c>
       <c r="B342" t="str">
         <v>2023-01-31</v>
@@ -46566,7 +46566,7 @@
     </row>
     <row r="343">
       <c r="A343" t="str">
-        <v>348</v>
+        <v>360</v>
       </c>
       <c r="B343" t="str">
         <v>2023-01-31</v>
@@ -46589,7 +46589,7 @@
     </row>
     <row r="344">
       <c r="A344" t="str">
-        <v>349</v>
+        <v>361</v>
       </c>
       <c r="B344" t="str">
         <v>2023-02-05</v>
@@ -46612,7 +46612,7 @@
     </row>
     <row r="345">
       <c r="A345" t="str">
-        <v>350</v>
+        <v>362</v>
       </c>
       <c r="B345" t="str">
         <v>2023-02-06</v>
@@ -46635,7 +46635,7 @@
     </row>
     <row r="346">
       <c r="A346" t="str">
-        <v>351</v>
+        <v>363</v>
       </c>
       <c r="B346" t="str">
         <v>2023-02-07</v>
@@ -46658,7 +46658,7 @@
     </row>
     <row r="347">
       <c r="A347" t="str">
-        <v>352</v>
+        <v>364</v>
       </c>
       <c r="B347" t="str">
         <v>2023-02-08</v>
@@ -46681,7 +46681,7 @@
     </row>
     <row r="348">
       <c r="A348" t="str">
-        <v>353</v>
+        <v>365</v>
       </c>
       <c r="B348" t="str">
         <v>2023-02-09</v>
@@ -46704,7 +46704,7 @@
     </row>
     <row r="349">
       <c r="A349" t="str">
-        <v>354</v>
+        <v>367</v>
       </c>
       <c r="B349" t="str">
         <v>2023-02-10</v>
@@ -46727,7 +46727,7 @@
     </row>
     <row r="350">
       <c r="A350" t="str">
-        <v>355</v>
+        <v>369</v>
       </c>
       <c r="B350" t="str">
         <v>2023-02-11</v>
@@ -46750,7 +46750,7 @@
     </row>
     <row r="351">
       <c r="A351" t="str">
-        <v>356</v>
+        <v>370</v>
       </c>
       <c r="B351" t="str">
         <v>2023-02-11</v>
@@ -46773,7 +46773,7 @@
     </row>
     <row r="352">
       <c r="A352" t="str">
-        <v>357</v>
+        <v>372</v>
       </c>
       <c r="B352" t="str">
         <v>2023-02-12</v>
@@ -46796,7 +46796,7 @@
     </row>
     <row r="353">
       <c r="A353" t="str">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="B353" t="str">
         <v>2023-02-13</v>
@@ -46819,7 +46819,7 @@
     </row>
     <row r="354">
       <c r="A354" t="str">
-        <v>359</v>
+        <v>374</v>
       </c>
       <c r="B354" t="str">
         <v>2023-02-14</v>
@@ -46842,7 +46842,7 @@
     </row>
     <row r="355">
       <c r="A355" t="str">
-        <v>360</v>
+        <v>375</v>
       </c>
       <c r="B355" t="str">
         <v>2023-02-14</v>
@@ -46865,7 +46865,7 @@
     </row>
     <row r="356">
       <c r="A356" t="str">
-        <v>361</v>
+        <v>379</v>
       </c>
       <c r="B356" t="str">
         <v>2023-02-15</v>
@@ -46888,7 +46888,7 @@
     </row>
     <row r="357">
       <c r="A357" t="str">
-        <v>362</v>
+        <v>380</v>
       </c>
       <c r="B357" t="str">
         <v>2023-02-15</v>
@@ -46911,7 +46911,7 @@
     </row>
     <row r="358">
       <c r="A358" t="str">
-        <v>363</v>
+        <v>381</v>
       </c>
       <c r="B358" t="str">
         <v>2023-02-16</v>
@@ -46934,7 +46934,7 @@
     </row>
     <row r="359">
       <c r="A359" t="str">
-        <v>364</v>
+        <v>383</v>
       </c>
       <c r="B359" t="str">
         <v>2023-02-18</v>
@@ -46957,7 +46957,7 @@
     </row>
     <row r="360">
       <c r="A360" t="str">
-        <v>365</v>
+        <v>384</v>
       </c>
       <c r="B360" t="str">
         <v>2023-02-19</v>
@@ -46980,7 +46980,7 @@
     </row>
     <row r="361">
       <c r="A361" t="str">
-        <v>366</v>
+        <v>385</v>
       </c>
       <c r="B361" t="str">
         <v>2023-02-19</v>
@@ -47003,7 +47003,7 @@
     </row>
     <row r="362">
       <c r="A362" t="str">
-        <v>367</v>
+        <v>386</v>
       </c>
       <c r="B362" t="str">
         <v>2023-02-20</v>
@@ -47026,7 +47026,7 @@
     </row>
     <row r="363">
       <c r="A363" t="str">
-        <v>368</v>
+        <v>390</v>
       </c>
       <c r="B363" t="str">
         <v>2023-02-24</v>
@@ -47049,7 +47049,7 @@
     </row>
     <row r="364">
       <c r="A364" t="str">
-        <v>369</v>
+        <v>391</v>
       </c>
       <c r="B364" t="str">
         <v>2023-02-24</v>
@@ -47072,7 +47072,7 @@
     </row>
     <row r="365">
       <c r="A365" t="str">
-        <v>370</v>
+        <v>392</v>
       </c>
       <c r="B365" t="str">
         <v>2023-02-25</v>
@@ -47095,7 +47095,7 @@
     </row>
     <row r="366">
       <c r="A366" t="str">
-        <v>371</v>
+        <v>393</v>
       </c>
       <c r="B366" t="str">
         <v>2023-02-25</v>
@@ -47118,7 +47118,7 @@
     </row>
     <row r="367">
       <c r="A367" t="str">
-        <v>372</v>
+        <v>394</v>
       </c>
       <c r="B367" t="str">
         <v>2023-02-25</v>
@@ -47141,7 +47141,7 @@
     </row>
     <row r="368">
       <c r="A368" t="str">
-        <v>374</v>
+        <v>398</v>
       </c>
       <c r="B368" t="str">
         <v>2023-03-09</v>
@@ -47164,7 +47164,7 @@
     </row>
     <row r="369">
       <c r="A369" t="str">
-        <v>375</v>
+        <v>399</v>
       </c>
       <c r="B369" t="str">
         <v>2023-03-10</v>
@@ -47187,7 +47187,7 @@
     </row>
     <row r="370">
       <c r="A370" t="str">
-        <v>376</v>
+        <v>400</v>
       </c>
       <c r="B370" t="str">
         <v>2023-03-11</v>
@@ -47210,7 +47210,7 @@
     </row>
     <row r="371">
       <c r="A371" t="str">
-        <v>377</v>
+        <v>401</v>
       </c>
       <c r="B371" t="str">
         <v>2023-03-12</v>
@@ -47233,7 +47233,7 @@
     </row>
     <row r="372">
       <c r="A372" t="str">
-        <v>378</v>
+        <v>404</v>
       </c>
       <c r="B372" t="str">
         <v>2023-03-15</v>
@@ -47256,7 +47256,7 @@
     </row>
     <row r="373">
       <c r="A373" t="str">
-        <v>379</v>
+        <v>405</v>
       </c>
       <c r="B373" t="str">
         <v>2023-03-15</v>
@@ -47279,7 +47279,7 @@
     </row>
     <row r="374">
       <c r="A374" t="str">
-        <v>380</v>
+        <v>407</v>
       </c>
       <c r="B374" t="str">
         <v>2023-03-16</v>
@@ -47302,7 +47302,7 @@
     </row>
     <row r="375">
       <c r="A375" t="str">
-        <v>381</v>
+        <v>408</v>
       </c>
       <c r="B375" t="str">
         <v>2023-03-16</v>
@@ -47325,7 +47325,7 @@
     </row>
     <row r="376">
       <c r="A376" t="str">
-        <v>382</v>
+        <v>411</v>
       </c>
       <c r="B376" t="str">
         <v>2023-03-23</v>
@@ -47348,7 +47348,7 @@
     </row>
     <row r="377">
       <c r="A377" t="str">
-        <v>383</v>
+        <v>412</v>
       </c>
       <c r="B377" t="str">
         <v>2023-03-24</v>
@@ -47371,7 +47371,7 @@
     </row>
     <row r="378">
       <c r="A378" t="str">
-        <v>384</v>
+        <v>415</v>
       </c>
       <c r="B378" t="str">
         <v>2023-03-27</v>
@@ -47394,7 +47394,7 @@
     </row>
     <row r="379">
       <c r="A379" t="str">
-        <v>385</v>
+        <v>417</v>
       </c>
       <c r="B379" t="str">
         <v>2023-03-28</v>
@@ -47417,7 +47417,7 @@
     </row>
     <row r="380">
       <c r="A380" t="str">
-        <v>386</v>
+        <v>419</v>
       </c>
       <c r="B380" t="str">
         <v>2023-03-31</v>
@@ -47440,7 +47440,7 @@
     </row>
     <row r="381">
       <c r="A381" t="str">
-        <v>387</v>
+        <v>420</v>
       </c>
       <c r="B381" t="str">
         <v>2023-04-01</v>
@@ -47463,7 +47463,7 @@
     </row>
     <row r="382">
       <c r="A382" t="str">
-        <v>388</v>
+        <v>422</v>
       </c>
       <c r="B382" t="str">
         <v>2023-04-03</v>
@@ -47486,7 +47486,7 @@
     </row>
     <row r="383">
       <c r="A383" t="str">
-        <v>389</v>
+        <v>423</v>
       </c>
       <c r="B383" t="str">
         <v>2023-04-04</v>
@@ -47509,7 +47509,7 @@
     </row>
     <row r="384">
       <c r="A384" t="str">
-        <v>390</v>
+        <v>425</v>
       </c>
       <c r="B384" t="str">
         <v>2023-04-07</v>
@@ -47532,7 +47532,7 @@
     </row>
     <row r="385">
       <c r="A385" t="str">
-        <v>391</v>
+        <v>426</v>
       </c>
       <c r="B385" t="str">
         <v>2023-04-07</v>
@@ -47555,7 +47555,7 @@
     </row>
     <row r="386">
       <c r="A386" t="str">
-        <v>392</v>
+        <v>428</v>
       </c>
       <c r="B386" t="str">
         <v>2023-04-08</v>
@@ -47578,7 +47578,7 @@
     </row>
     <row r="387">
       <c r="A387" t="str">
-        <v>393</v>
+        <v>429</v>
       </c>
       <c r="B387" t="str">
         <v>2023-04-08</v>
@@ -47601,7 +47601,7 @@
     </row>
     <row r="388">
       <c r="A388" t="str">
-        <v>394</v>
+        <v>430</v>
       </c>
       <c r="B388" t="str">
         <v>2023-04-09</v>
@@ -47624,7 +47624,7 @@
     </row>
     <row r="389">
       <c r="A389" t="str">
-        <v>395</v>
+        <v>431</v>
       </c>
       <c r="B389" t="str">
         <v>2023-04-10</v>
@@ -47647,7 +47647,7 @@
     </row>
     <row r="390">
       <c r="A390" t="str">
-        <v>396</v>
+        <v>432</v>
       </c>
       <c r="B390" t="str">
         <v>2023-04-11</v>
@@ -47670,7 +47670,7 @@
     </row>
     <row r="391">
       <c r="A391" t="str">
-        <v>397</v>
+        <v>433</v>
       </c>
       <c r="B391" t="str">
         <v>2023-04-12</v>
@@ -47693,7 +47693,7 @@
     </row>
     <row r="392">
       <c r="A392" t="str">
-        <v>399</v>
+        <v>435</v>
       </c>
       <c r="B392" t="str">
         <v>2023-04-13</v>
@@ -47716,7 +47716,7 @@
     </row>
     <row r="393">
       <c r="A393" t="str">
-        <v>400</v>
+        <v>437</v>
       </c>
       <c r="B393" t="str">
         <v>2023-04-14</v>
@@ -47739,7 +47739,7 @@
     </row>
     <row r="394">
       <c r="A394" t="str">
-        <v>401</v>
+        <v>438</v>
       </c>
       <c r="B394" t="str">
         <v>2023-04-16</v>
@@ -47762,7 +47762,7 @@
     </row>
     <row r="395">
       <c r="A395" t="str">
-        <v>402</v>
+        <v>439</v>
       </c>
       <c r="B395" t="str">
         <v>2023-04-17</v>
@@ -47785,7 +47785,7 @@
     </row>
     <row r="396">
       <c r="A396" t="str">
-        <v>403</v>
+        <v>441</v>
       </c>
       <c r="B396" t="str">
         <v>2023-04-18</v>
@@ -47808,7 +47808,7 @@
     </row>
     <row r="397">
       <c r="A397" t="str">
-        <v>404</v>
+        <v>444</v>
       </c>
       <c r="B397" t="str">
         <v>2023-04-19</v>
@@ -47831,7 +47831,7 @@
     </row>
     <row r="398">
       <c r="A398" t="str">
-        <v>405</v>
+        <v>445</v>
       </c>
       <c r="B398" t="str">
         <v>2023-04-19</v>
@@ -47854,7 +47854,7 @@
     </row>
     <row r="399">
       <c r="A399" t="str">
-        <v>406</v>
+        <v>446</v>
       </c>
       <c r="B399" t="str">
         <v>2023-04-19</v>
@@ -47877,7 +47877,7 @@
     </row>
     <row r="400">
       <c r="A400" t="str">
-        <v>407</v>
+        <v>447</v>
       </c>
       <c r="B400" t="str">
         <v>2023-04-19</v>
@@ -47900,7 +47900,7 @@
     </row>
     <row r="401">
       <c r="A401" t="str">
-        <v>408</v>
+        <v>448</v>
       </c>
       <c r="B401" t="str">
         <v>2023-04-19</v>
@@ -47923,7 +47923,7 @@
     </row>
     <row r="402">
       <c r="A402" t="str">
-        <v>409</v>
+        <v>449</v>
       </c>
       <c r="B402" t="str">
         <v>2023-04-19</v>
@@ -47946,7 +47946,7 @@
     </row>
     <row r="403">
       <c r="A403" t="str">
-        <v>410</v>
+        <v>450</v>
       </c>
       <c r="B403" t="str">
         <v>2023-04-19</v>
@@ -47969,7 +47969,7 @@
     </row>
     <row r="404">
       <c r="A404" t="str">
-        <v>411</v>
+        <v>451</v>
       </c>
       <c r="B404" t="str">
         <v>2023-04-19</v>
@@ -47992,7 +47992,7 @@
     </row>
     <row r="405">
       <c r="A405" t="str">
-        <v>412</v>
+        <v>452</v>
       </c>
       <c r="B405" t="str">
         <v>2023-04-19</v>
@@ -48015,7 +48015,7 @@
     </row>
     <row r="406">
       <c r="A406" t="str">
-        <v>413</v>
+        <v>453</v>
       </c>
       <c r="B406" t="str">
         <v>2023-04-19</v>
@@ -48038,7 +48038,7 @@
     </row>
     <row r="407">
       <c r="A407" t="str">
-        <v>414</v>
+        <v>454</v>
       </c>
       <c r="B407" t="str">
         <v>2023-04-19</v>
@@ -48061,7 +48061,7 @@
     </row>
     <row r="408">
       <c r="A408" t="str">
-        <v>415</v>
+        <v>455</v>
       </c>
       <c r="B408" t="str">
         <v>2023-04-19</v>
@@ -48084,7 +48084,7 @@
     </row>
     <row r="409">
       <c r="A409" t="str">
-        <v>416</v>
+        <v>456</v>
       </c>
       <c r="B409" t="str">
         <v>2023-04-19</v>
@@ -48107,7 +48107,7 @@
     </row>
     <row r="410">
       <c r="A410" t="str">
-        <v>417</v>
+        <v>457</v>
       </c>
       <c r="B410" t="str">
         <v>2023-04-19</v>
@@ -48130,7 +48130,7 @@
     </row>
     <row r="411">
       <c r="A411" t="str">
-        <v>418</v>
+        <v>458</v>
       </c>
       <c r="B411" t="str">
         <v>2023-04-19</v>
@@ -48153,7 +48153,7 @@
     </row>
     <row r="412">
       <c r="A412" t="str">
-        <v>423</v>
+        <v>513</v>
       </c>
       <c r="B412" t="str">
         <v>2023-09-28</v>
@@ -48176,7 +48176,7 @@
     </row>
     <row r="413">
       <c r="A413" t="str">
-        <v>424</v>
+        <v>514</v>
       </c>
       <c r="B413" t="str">
         <v>2023-09-28</v>
@@ -48199,7 +48199,7 @@
     </row>
     <row r="414">
       <c r="A414" t="str">
-        <v>425</v>
+        <v>515</v>
       </c>
       <c r="B414" t="str">
         <v>2023-09-29</v>
@@ -48222,7 +48222,7 @@
     </row>
     <row r="415">
       <c r="A415" t="str">
-        <v>426</v>
+        <v>516</v>
       </c>
       <c r="B415" t="str">
         <v>2023-09-29</v>
@@ -48245,7 +48245,7 @@
     </row>
     <row r="416">
       <c r="A416" t="str">
-        <v>427</v>
+        <v>517</v>
       </c>
       <c r="B416" t="str">
         <v>2023-09-29</v>
@@ -48268,7 +48268,7 @@
     </row>
     <row r="417">
       <c r="A417" t="str">
-        <v>428</v>
+        <v>518</v>
       </c>
       <c r="B417" t="str">
         <v>2023-09-29</v>
@@ -48291,7 +48291,7 @@
     </row>
     <row r="418">
       <c r="A418" t="str">
-        <v>430</v>
+        <v>520</v>
       </c>
       <c r="B418" t="str">
         <v>2023-10-10</v>
@@ -48314,7 +48314,7 @@
     </row>
     <row r="419">
       <c r="A419" t="str">
-        <v>431</v>
+        <v>521</v>
       </c>
       <c r="B419" t="str">
         <v>2023-10-10</v>
@@ -48337,7 +48337,7 @@
     </row>
     <row r="420">
       <c r="A420" t="str">
-        <v>437</v>
+        <v>527</v>
       </c>
       <c r="B420" t="str">
         <v>2023-11-02</v>
@@ -48360,7 +48360,7 @@
     </row>
     <row r="421">
       <c r="A421" t="str">
-        <v>441</v>
+        <v>533</v>
       </c>
       <c r="B421" t="str">
         <v>2023-11-23</v>
@@ -48383,7 +48383,7 @@
     </row>
     <row r="422">
       <c r="A422" t="str">
-        <v>443</v>
+        <v>535</v>
       </c>
       <c r="B422" t="str">
         <v>2023-11-26</v>
@@ -48406,7 +48406,7 @@
     </row>
     <row r="423">
       <c r="A423" t="str">
-        <v>445</v>
+        <v>537</v>
       </c>
       <c r="B423" t="str">
         <v>2023-12-01</v>
@@ -48429,7 +48429,7 @@
     </row>
     <row r="424">
       <c r="A424" t="str">
-        <v>446</v>
+        <v>538</v>
       </c>
       <c r="B424" t="str">
         <v>2023-12-04</v>
@@ -48452,7 +48452,7 @@
     </row>
     <row r="425">
       <c r="A425" t="str">
-        <v>447</v>
+        <v>539</v>
       </c>
       <c r="B425" t="str">
         <v>2023-12-05</v>
@@ -48475,7 +48475,7 @@
     </row>
     <row r="426">
       <c r="A426" t="str">
-        <v>448</v>
+        <v>540</v>
       </c>
       <c r="B426" t="str">
         <v>2023-12-06</v>
@@ -48498,7 +48498,7 @@
     </row>
     <row r="427">
       <c r="A427" t="str">
-        <v>449</v>
+        <v>541</v>
       </c>
       <c r="B427" t="str">
         <v>2023-12-07</v>
@@ -48521,7 +48521,7 @@
     </row>
     <row r="428">
       <c r="A428" t="str">
-        <v>450</v>
+        <v>542</v>
       </c>
       <c r="B428" t="str">
         <v>2023-12-07</v>
@@ -48544,7 +48544,7 @@
     </row>
     <row r="429">
       <c r="A429" t="str">
-        <v>451</v>
+        <v>543</v>
       </c>
       <c r="B429" t="str">
         <v>2023-12-08</v>
@@ -48567,7 +48567,7 @@
     </row>
     <row r="430">
       <c r="A430" t="str">
-        <v>452</v>
+        <v>544</v>
       </c>
       <c r="B430" t="str">
         <v>2023-12-09</v>
@@ -48590,7 +48590,7 @@
     </row>
     <row r="431">
       <c r="A431" t="str">
-        <v>453</v>
+        <v>545</v>
       </c>
       <c r="B431" t="str">
         <v>2023-12-10</v>
@@ -48613,7 +48613,7 @@
     </row>
     <row r="432">
       <c r="A432" t="str">
-        <v>455</v>
+        <v>547</v>
       </c>
       <c r="B432" t="str">
         <v>2023-12-11</v>
@@ -48636,7 +48636,7 @@
     </row>
     <row r="433">
       <c r="A433" t="str">
-        <v>456</v>
+        <v>548</v>
       </c>
       <c r="B433" t="str">
         <v>2023-12-11</v>
@@ -48659,7 +48659,7 @@
     </row>
     <row r="434">
       <c r="A434" t="str">
-        <v>457</v>
+        <v>549</v>
       </c>
       <c r="B434" t="str">
         <v>2023-12-11</v>
@@ -48682,7 +48682,7 @@
     </row>
     <row r="435">
       <c r="A435" t="str">
-        <v>458</v>
+        <v>550</v>
       </c>
       <c r="B435" t="str">
         <v>2023-12-11</v>
@@ -48705,7 +48705,7 @@
     </row>
     <row r="436">
       <c r="A436" t="str">
-        <v>459</v>
+        <v>551</v>
       </c>
       <c r="B436" t="str">
         <v>2023-12-11</v>
@@ -48728,7 +48728,7 @@
     </row>
     <row r="437">
       <c r="A437" t="str">
-        <v>460</v>
+        <v>552</v>
       </c>
       <c r="B437" t="str">
         <v>2023-12-11</v>
@@ -48751,7 +48751,7 @@
     </row>
     <row r="438">
       <c r="A438" t="str">
-        <v>461</v>
+        <v>553</v>
       </c>
       <c r="B438" t="str">
         <v>2023-12-11</v>
@@ -48774,7 +48774,7 @@
     </row>
     <row r="439">
       <c r="A439" t="str">
-        <v>462</v>
+        <v>554</v>
       </c>
       <c r="B439" t="str">
         <v>2023-12-11</v>
@@ -48797,7 +48797,7 @@
     </row>
     <row r="440">
       <c r="A440" t="str">
-        <v>463</v>
+        <v>555</v>
       </c>
       <c r="B440" t="str">
         <v>2023-12-11</v>
@@ -48820,7 +48820,7 @@
     </row>
     <row r="441">
       <c r="A441" t="str">
-        <v>464</v>
+        <v>556</v>
       </c>
       <c r="B441" t="str">
         <v>2023-12-16</v>
@@ -48843,7 +48843,7 @@
     </row>
     <row r="442">
       <c r="A442" t="str">
-        <v>465</v>
+        <v>557</v>
       </c>
       <c r="B442" t="str">
         <v>2023-12-18</v>
@@ -48866,7 +48866,7 @@
     </row>
     <row r="443">
       <c r="A443" t="str">
-        <v>471</v>
+        <v>563</v>
       </c>
       <c r="B443" t="str">
         <v>2024-01-06</v>
@@ -48889,7 +48889,7 @@
     </row>
     <row r="444">
       <c r="A444" t="str">
-        <v>472</v>
+        <v>564</v>
       </c>
       <c r="B444" t="str">
         <v>2024-01-06</v>
@@ -48912,7 +48912,7 @@
     </row>
     <row r="445">
       <c r="A445" t="str">
-        <v>473</v>
+        <v>565</v>
       </c>
       <c r="B445" t="str">
         <v>2024-01-06</v>
@@ -48935,7 +48935,7 @@
     </row>
     <row r="446">
       <c r="A446" t="str">
-        <v>474</v>
+        <v>566</v>
       </c>
       <c r="B446" t="str">
         <v>2024-01-06</v>
@@ -48958,7 +48958,7 @@
     </row>
     <row r="447">
       <c r="A447" t="str">
-        <v>475</v>
+        <v>567</v>
       </c>
       <c r="B447" t="str">
         <v>2024-01-07</v>
@@ -48981,7 +48981,7 @@
     </row>
     <row r="448">
       <c r="A448" t="str">
-        <v>476</v>
+        <v>568</v>
       </c>
       <c r="B448" t="str">
         <v>2024-01-07</v>
@@ -49004,7 +49004,7 @@
     </row>
     <row r="449">
       <c r="A449" t="str">
-        <v>477</v>
+        <v>569</v>
       </c>
       <c r="B449" t="str">
         <v>2024-01-07</v>
@@ -49027,7 +49027,7 @@
     </row>
     <row r="450">
       <c r="A450" t="str">
-        <v>478</v>
+        <v>570</v>
       </c>
       <c r="B450" t="str">
         <v>2024-01-07</v>
@@ -49050,7 +49050,7 @@
     </row>
     <row r="451">
       <c r="A451" t="str">
-        <v>479</v>
+        <v>571</v>
       </c>
       <c r="B451" t="str">
         <v>2024-01-08</v>
@@ -49073,7 +49073,7 @@
     </row>
     <row r="452">
       <c r="A452" t="str">
-        <v>480</v>
+        <v>572</v>
       </c>
       <c r="B452" t="str">
         <v>2024-01-10</v>
@@ -49096,7 +49096,7 @@
     </row>
     <row r="453">
       <c r="A453" t="str">
-        <v>481</v>
+        <v>573</v>
       </c>
       <c r="B453" t="str">
         <v>2024-01-11</v>
@@ -49119,7 +49119,7 @@
     </row>
     <row r="454">
       <c r="A454" t="str">
-        <v>482</v>
+        <v>574</v>
       </c>
       <c r="B454" t="str">
         <v>2024-01-11</v>
@@ -49142,7 +49142,7 @@
     </row>
     <row r="455">
       <c r="A455" t="str">
-        <v>483</v>
+        <v>575</v>
       </c>
       <c r="B455" t="str">
         <v>2024-01-11</v>
@@ -49165,7 +49165,7 @@
     </row>
     <row r="456">
       <c r="A456" t="str">
-        <v>487</v>
+        <v>579</v>
       </c>
       <c r="B456" t="str">
         <v>2024-01-17</v>
@@ -49188,7 +49188,7 @@
     </row>
     <row r="457">
       <c r="A457" t="str">
-        <v>488</v>
+        <v>580</v>
       </c>
       <c r="B457" t="str">
         <v>2024-01-18</v>
@@ -49211,7 +49211,7 @@
     </row>
     <row r="458">
       <c r="A458" t="str">
-        <v>489</v>
+        <v>581</v>
       </c>
       <c r="B458" t="str">
         <v>2024-01-19</v>
@@ -49234,7 +49234,7 @@
     </row>
     <row r="459">
       <c r="A459" t="str">
-        <v>490</v>
+        <v>582</v>
       </c>
       <c r="B459" t="str">
         <v>2024-01-19</v>
@@ -49257,7 +49257,7 @@
     </row>
     <row r="460">
       <c r="A460" t="str">
-        <v>491</v>
+        <v>583</v>
       </c>
       <c r="B460" t="str">
         <v>2024-01-19</v>
@@ -49280,7 +49280,7 @@
     </row>
     <row r="461">
       <c r="A461" t="str">
-        <v>492</v>
+        <v>584</v>
       </c>
       <c r="B461" t="str">
         <v>2024-01-20</v>
@@ -49303,7 +49303,7 @@
     </row>
     <row r="462">
       <c r="A462" t="str">
-        <v>493</v>
+        <v>585</v>
       </c>
       <c r="B462" t="str">
         <v>2024-01-22</v>
@@ -49326,7 +49326,7 @@
     </row>
     <row r="463">
       <c r="A463" t="str">
-        <v>494</v>
+        <v>586</v>
       </c>
       <c r="B463" t="str">
         <v>2024-01-22</v>
@@ -49349,7 +49349,7 @@
     </row>
     <row r="464">
       <c r="A464" t="str">
-        <v>495</v>
+        <v>587</v>
       </c>
       <c r="B464" t="str">
         <v>2024-01-22</v>
@@ -49372,7 +49372,7 @@
     </row>
     <row r="465">
       <c r="A465" t="str">
-        <v>496</v>
+        <v>588</v>
       </c>
       <c r="B465" t="str">
         <v>2024-01-24</v>
@@ -49395,7 +49395,7 @@
     </row>
     <row r="466">
       <c r="A466" t="str">
-        <v>497</v>
+        <v>589</v>
       </c>
       <c r="B466" t="str">
         <v>2024-01-25</v>
@@ -49418,7 +49418,7 @@
     </row>
     <row r="467">
       <c r="A467" t="str">
-        <v>498</v>
+        <v>590</v>
       </c>
       <c r="B467" t="str">
         <v>2024-01-27</v>
@@ -49441,7 +49441,7 @@
     </row>
     <row r="468">
       <c r="A468" t="str">
-        <v>499</v>
+        <v>591</v>
       </c>
       <c r="B468" t="str">
         <v>2024-01-28</v>
@@ -49464,7 +49464,7 @@
     </row>
     <row r="469">
       <c r="A469" t="str">
-        <v>500</v>
+        <v>592</v>
       </c>
       <c r="B469" t="str">
         <v>2024-01-29</v>
@@ -49487,7 +49487,7 @@
     </row>
     <row r="470">
       <c r="A470" t="str">
-        <v>501</v>
+        <v>593</v>
       </c>
       <c r="B470" t="str">
         <v>2024-01-29</v>
@@ -49510,7 +49510,7 @@
     </row>
     <row r="471">
       <c r="A471" t="str">
-        <v>502</v>
+        <v>594</v>
       </c>
       <c r="B471" t="str">
         <v>2024-02-01</v>
@@ -49533,7 +49533,7 @@
     </row>
     <row r="472">
       <c r="A472" t="str">
-        <v>503</v>
+        <v>595</v>
       </c>
       <c r="B472" t="str">
         <v>2024-02-01</v>
@@ -49556,7 +49556,7 @@
     </row>
     <row r="473">
       <c r="A473" t="str">
-        <v>504</v>
+        <v>596</v>
       </c>
       <c r="B473" t="str">
         <v>2024-02-02</v>
@@ -49579,7 +49579,7 @@
     </row>
     <row r="474">
       <c r="A474" t="str">
-        <v>505</v>
+        <v>597</v>
       </c>
       <c r="B474" t="str">
         <v>2024-02-03</v>
@@ -49602,7 +49602,7 @@
     </row>
     <row r="475">
       <c r="A475" t="str">
-        <v>506</v>
+        <v>598</v>
       </c>
       <c r="B475" t="str">
         <v>2024-02-03</v>
@@ -49625,7 +49625,7 @@
     </row>
     <row r="476">
       <c r="A476" t="str">
-        <v>507</v>
+        <v>599</v>
       </c>
       <c r="B476" t="str">
         <v>2024-02-06</v>
@@ -49648,7 +49648,7 @@
     </row>
     <row r="477">
       <c r="A477" t="str">
-        <v>508</v>
+        <v>600</v>
       </c>
       <c r="B477" t="str">
         <v>2024-02-06</v>
@@ -49671,7 +49671,7 @@
     </row>
     <row r="478">
       <c r="A478" t="str">
-        <v>509</v>
+        <v>601</v>
       </c>
       <c r="B478" t="str">
         <v>2024-02-06</v>
@@ -49694,7 +49694,7 @@
     </row>
     <row r="479">
       <c r="A479" t="str">
-        <v>510</v>
+        <v>602</v>
       </c>
       <c r="B479" t="str">
         <v>2024-02-06</v>
@@ -49717,7 +49717,7 @@
     </row>
     <row r="480">
       <c r="A480" t="str">
-        <v>511</v>
+        <v>603</v>
       </c>
       <c r="B480" t="str">
         <v>2024-02-08</v>
@@ -49740,7 +49740,7 @@
     </row>
     <row r="481">
       <c r="A481" t="str">
-        <v>512</v>
+        <v>604</v>
       </c>
       <c r="B481" t="str">
         <v>2024-02-10</v>
@@ -49763,7 +49763,7 @@
     </row>
     <row r="482">
       <c r="A482" t="str">
-        <v>513</v>
+        <v>605</v>
       </c>
       <c r="B482" t="str">
         <v>2024-02-11</v>
@@ -49786,7 +49786,7 @@
     </row>
     <row r="483">
       <c r="A483" t="str">
-        <v>515</v>
+        <v>607</v>
       </c>
       <c r="B483" t="str">
         <v>2024-02-13</v>
@@ -49809,7 +49809,7 @@
     </row>
     <row r="484">
       <c r="A484" t="str">
-        <v>516</v>
+        <v>608</v>
       </c>
       <c r="B484" t="str">
         <v>2024-02-14</v>
@@ -49832,7 +49832,7 @@
     </row>
     <row r="485">
       <c r="A485" t="str">
-        <v>517</v>
+        <v>609</v>
       </c>
       <c r="B485" t="str">
         <v>2024-02-14</v>
@@ -49855,7 +49855,7 @@
     </row>
     <row r="486">
       <c r="A486" t="str">
-        <v>518</v>
+        <v>610</v>
       </c>
       <c r="B486" t="str">
         <v>2024-02-14</v>
@@ -49878,7 +49878,7 @@
     </row>
     <row r="487">
       <c r="A487" t="str">
-        <v>519</v>
+        <v>611</v>
       </c>
       <c r="B487" t="str">
         <v>2024-02-15</v>
@@ -49901,7 +49901,7 @@
     </row>
     <row r="488">
       <c r="A488" t="str">
-        <v>520</v>
+        <v>612</v>
       </c>
       <c r="B488" t="str">
         <v>2024-02-15</v>
@@ -49924,7 +49924,7 @@
     </row>
     <row r="489">
       <c r="A489" t="str">
-        <v>521</v>
+        <v>613</v>
       </c>
       <c r="B489" t="str">
         <v>2024-02-16</v>
@@ -49947,7 +49947,7 @@
     </row>
     <row r="490">
       <c r="A490" t="str">
-        <v>523</v>
+        <v>615</v>
       </c>
       <c r="B490" t="str">
         <v>2024-02-24</v>
@@ -49970,7 +49970,7 @@
     </row>
     <row r="491">
       <c r="A491" t="str">
-        <v>525</v>
+        <v>617</v>
       </c>
       <c r="B491" t="str">
         <v>2024-02-25</v>
@@ -49993,7 +49993,7 @@
     </row>
     <row r="492">
       <c r="A492" t="str">
-        <v>526</v>
+        <v>618</v>
       </c>
       <c r="B492" t="str">
         <v>2024-02-26</v>
@@ -50016,7 +50016,7 @@
     </row>
     <row r="493">
       <c r="A493" t="str">
-        <v>529</v>
+        <v>621</v>
       </c>
       <c r="B493" t="str">
         <v>2024-02-28</v>
@@ -50039,7 +50039,7 @@
     </row>
     <row r="494">
       <c r="A494" t="str">
-        <v>530</v>
+        <v>622</v>
       </c>
       <c r="B494" t="str">
         <v>2024-02-29</v>
@@ -50062,7 +50062,7 @@
     </row>
     <row r="495">
       <c r="A495" t="str">
-        <v>532</v>
+        <v>624</v>
       </c>
       <c r="B495" t="str">
         <v>2024-03-01</v>
@@ -50085,7 +50085,7 @@
     </row>
     <row r="496">
       <c r="A496" t="str">
-        <v>534</v>
+        <v>626</v>
       </c>
       <c r="B496" t="str">
         <v>2024-03-02</v>
@@ -50108,7 +50108,7 @@
     </row>
     <row r="497">
       <c r="A497" t="str">
-        <v>535</v>
+        <v>627</v>
       </c>
       <c r="B497" t="str">
         <v>2024-03-02</v>
@@ -50131,7 +50131,7 @@
     </row>
     <row r="498">
       <c r="A498" t="str">
-        <v>536</v>
+        <v>628</v>
       </c>
       <c r="B498" t="str">
         <v>2024-03-03</v>
@@ -50154,7 +50154,7 @@
     </row>
     <row r="499">
       <c r="A499" t="str">
-        <v>537</v>
+        <v>629</v>
       </c>
       <c r="B499" t="str">
         <v>2024-03-04</v>
@@ -50177,7 +50177,7 @@
     </row>
     <row r="500">
       <c r="A500" t="str">
-        <v>538</v>
+        <v>630</v>
       </c>
       <c r="B500" t="str">
         <v>2024-03-05</v>
@@ -50200,7 +50200,7 @@
     </row>
     <row r="501">
       <c r="A501" t="str">
-        <v>539</v>
+        <v>631</v>
       </c>
       <c r="B501" t="str">
         <v>2024-03-05</v>
@@ -50223,7 +50223,7 @@
     </row>
     <row r="502">
       <c r="A502" t="str">
-        <v>540</v>
+        <v>632</v>
       </c>
       <c r="B502" t="str">
         <v>2024-03-06</v>
@@ -50246,7 +50246,7 @@
     </row>
     <row r="503">
       <c r="A503" t="str">
-        <v>542</v>
+        <v>634</v>
       </c>
       <c r="B503" t="str">
         <v>2024-03-07</v>
@@ -50269,7 +50269,7 @@
     </row>
     <row r="504">
       <c r="A504" t="str">
-        <v>546</v>
+        <v>641</v>
       </c>
       <c r="B504" t="str">
         <v>2024-03-14</v>
@@ -50292,7 +50292,7 @@
     </row>
     <row r="505">
       <c r="A505" t="str">
-        <v>547</v>
+        <v>642</v>
       </c>
       <c r="B505" t="str">
         <v>2024-03-14</v>
@@ -50315,7 +50315,7 @@
     </row>
     <row r="506">
       <c r="A506" t="str">
-        <v>548</v>
+        <v>643</v>
       </c>
       <c r="B506" t="str">
         <v>2024-03-14</v>
@@ -50338,7 +50338,7 @@
     </row>
     <row r="507">
       <c r="A507" t="str">
-        <v>549</v>
+        <v>644</v>
       </c>
       <c r="B507" t="str">
         <v>2024-03-14</v>
@@ -50361,7 +50361,7 @@
     </row>
     <row r="508">
       <c r="A508" t="str">
-        <v>550</v>
+        <v>645</v>
       </c>
       <c r="B508" t="str">
         <v>2024-03-14</v>
@@ -50384,7 +50384,7 @@
     </row>
     <row r="509">
       <c r="A509" t="str">
-        <v>551</v>
+        <v>646</v>
       </c>
       <c r="B509" t="str">
         <v>2024-03-14</v>
@@ -50407,7 +50407,7 @@
     </row>
     <row r="510">
       <c r="A510" t="str">
-        <v>552</v>
+        <v>647</v>
       </c>
       <c r="B510" t="str">
         <v>2024-03-14</v>
@@ -50430,7 +50430,7 @@
     </row>
     <row r="511">
       <c r="A511" t="str">
-        <v>553</v>
+        <v>648</v>
       </c>
       <c r="B511" t="str">
         <v>2024-03-14</v>
@@ -50453,7 +50453,7 @@
     </row>
     <row r="512">
       <c r="A512" t="str">
-        <v>561</v>
+        <v>660</v>
       </c>
       <c r="B512" t="str">
         <v>2024-04-01</v>
@@ -50476,7 +50476,7 @@
     </row>
     <row r="513">
       <c r="A513" t="str">
-        <v>563</v>
+        <v>662</v>
       </c>
       <c r="B513" t="str">
         <v>2024-04-02</v>
@@ -50499,7 +50499,7 @@
     </row>
     <row r="514">
       <c r="A514" t="str">
-        <v>564</v>
+        <v>663</v>
       </c>
       <c r="B514" t="str">
         <v>2024-04-02</v>
@@ -50522,7 +50522,7 @@
     </row>
     <row r="515">
       <c r="A515" t="str">
-        <v>565</v>
+        <v>664</v>
       </c>
       <c r="B515" t="str">
         <v>2024-04-02</v>
@@ -50545,7 +50545,7 @@
     </row>
     <row r="516">
       <c r="A516" t="str">
-        <v>568</v>
+        <v>667</v>
       </c>
       <c r="B516" t="str">
         <v>2024-04-04</v>
@@ -50568,7 +50568,7 @@
     </row>
     <row r="517">
       <c r="A517" t="str">
-        <v>570</v>
+        <v>669</v>
       </c>
       <c r="B517" t="str">
         <v>2024-04-05</v>
@@ -50591,7 +50591,7 @@
     </row>
     <row r="518">
       <c r="A518" t="str">
-        <v>571</v>
+        <v>670</v>
       </c>
       <c r="B518" t="str">
         <v>2024-04-05</v>
@@ -50614,7 +50614,7 @@
     </row>
     <row r="519">
       <c r="A519" t="str">
-        <v>572</v>
+        <v>671</v>
       </c>
       <c r="B519" t="str">
         <v>2024-04-06</v>
@@ -50637,7 +50637,7 @@
     </row>
     <row r="520">
       <c r="A520" t="str">
-        <v>574</v>
+        <v>674</v>
       </c>
       <c r="B520" t="str">
         <v>2024-04-07</v>
@@ -50660,7 +50660,7 @@
     </row>
     <row r="521">
       <c r="A521" t="str">
-        <v>575</v>
+        <v>675</v>
       </c>
       <c r="B521" t="str">
         <v>2024-04-08</v>
@@ -50683,7 +50683,7 @@
     </row>
     <row r="522">
       <c r="A522" t="str">
-        <v>576</v>
+        <v>676</v>
       </c>
       <c r="B522" t="str">
         <v>2024-04-08</v>
@@ -50706,7 +50706,7 @@
     </row>
     <row r="523">
       <c r="A523" t="str">
-        <v>577</v>
+        <v>677</v>
       </c>
       <c r="B523" t="str">
         <v>2024-04-08</v>
@@ -50729,7 +50729,7 @@
     </row>
     <row r="524">
       <c r="A524" t="str">
-        <v>578</v>
+        <v>678</v>
       </c>
       <c r="B524" t="str">
         <v>2024-04-09</v>
@@ -50752,7 +50752,7 @@
     </row>
     <row r="525">
       <c r="A525" t="str">
-        <v>580</v>
+        <v>680</v>
       </c>
       <c r="B525" t="str">
         <v>2024-04-10</v>
@@ -50775,7 +50775,7 @@
     </row>
     <row r="526">
       <c r="A526" t="str">
-        <v>581</v>
+        <v>681</v>
       </c>
       <c r="B526" t="str">
         <v>2024-04-10</v>
@@ -50798,7 +50798,7 @@
     </row>
     <row r="527">
       <c r="A527" t="str">
-        <v>583</v>
+        <v>683</v>
       </c>
       <c r="B527" t="str">
         <v>2024-04-11</v>
@@ -50821,7 +50821,7 @@
     </row>
     <row r="528">
       <c r="A528" t="str">
-        <v>586</v>
+        <v>687</v>
       </c>
       <c r="B528" t="str">
         <v>2024-04-16</v>
@@ -50844,7 +50844,7 @@
     </row>
     <row r="529">
       <c r="A529" t="str">
-        <v>588</v>
+        <v>689</v>
       </c>
       <c r="B529" t="str">
         <v>2024-04-19</v>
@@ -50867,7 +50867,7 @@
     </row>
     <row r="530">
       <c r="A530" t="str">
-        <v>590</v>
+        <v>691</v>
       </c>
       <c r="B530" t="str">
         <v>2024-04-20</v>
@@ -50890,7 +50890,7 @@
     </row>
     <row r="531">
       <c r="A531" t="str">
-        <v>591</v>
+        <v>692</v>
       </c>
       <c r="B531" t="str">
         <v>2024-04-20</v>
@@ -50913,7 +50913,7 @@
     </row>
     <row r="532">
       <c r="A532" t="str">
-        <v>592</v>
+        <v>693</v>
       </c>
       <c r="B532" t="str">
         <v>2024-04-20</v>
@@ -50936,7 +50936,7 @@
     </row>
     <row r="533">
       <c r="A533" t="str">
-        <v>593</v>
+        <v>694</v>
       </c>
       <c r="B533" t="str">
         <v>2024-04-20</v>
@@ -50959,7 +50959,7 @@
     </row>
     <row r="534">
       <c r="A534" t="str">
-        <v>594</v>
+        <v>695</v>
       </c>
       <c r="B534" t="str">
         <v>2024-04-20</v>
@@ -50982,7 +50982,7 @@
     </row>
     <row r="535">
       <c r="A535" t="str">
-        <v>595</v>
+        <v>696</v>
       </c>
       <c r="B535" t="str">
         <v>2024-04-20</v>
@@ -51005,7 +51005,7 @@
     </row>
     <row r="536">
       <c r="A536" t="str">
-        <v>596</v>
+        <v>697</v>
       </c>
       <c r="B536" t="str">
         <v>2024-04-20</v>
@@ -51028,7 +51028,7 @@
     </row>
     <row r="537">
       <c r="A537" t="str">
-        <v>597</v>
+        <v>698</v>
       </c>
       <c r="B537" t="str">
         <v>2024-04-22</v>
@@ -51051,7 +51051,7 @@
     </row>
     <row r="538">
       <c r="A538" t="str">
-        <v>598</v>
+        <v>699</v>
       </c>
       <c r="B538" t="str">
         <v>2024-04-23</v>
@@ -51074,7 +51074,7 @@
     </row>
     <row r="539">
       <c r="A539" t="str">
-        <v>600</v>
+        <v>701</v>
       </c>
       <c r="B539" t="str">
         <v>2024-04-26</v>
@@ -51097,7 +51097,7 @@
     </row>
     <row r="540">
       <c r="A540" t="str">
-        <v>601</v>
+        <v>702</v>
       </c>
       <c r="B540" t="str">
         <v>2024-04-26</v>
@@ -51120,7 +51120,7 @@
     </row>
     <row r="541">
       <c r="A541" t="str">
-        <v>602</v>
+        <v>703</v>
       </c>
       <c r="B541" t="str">
         <v>2024-04-27</v>
@@ -51143,7 +51143,7 @@
     </row>
     <row r="542">
       <c r="A542" t="str">
-        <v>603</v>
+        <v>704</v>
       </c>
       <c r="B542" t="str">
         <v>2024-04-28</v>
@@ -51166,7 +51166,7 @@
     </row>
     <row r="543">
       <c r="A543" t="str">
-        <v>604</v>
+        <v>706</v>
       </c>
       <c r="B543" t="str">
         <v>2024-04-30</v>
@@ -51189,7 +51189,7 @@
     </row>
     <row r="544">
       <c r="A544" t="str">
-        <v>605</v>
+        <v>707</v>
       </c>
       <c r="B544" t="str">
         <v>2024-04-30</v>
@@ -51212,7 +51212,7 @@
     </row>
     <row r="545">
       <c r="A545" t="str">
-        <v>606</v>
+        <v>708</v>
       </c>
       <c r="B545" t="str">
         <v>2024-04-30</v>
@@ -51235,7 +51235,7 @@
     </row>
     <row r="546">
       <c r="A546" t="str">
-        <v>607</v>
+        <v>709</v>
       </c>
       <c r="B546" t="str">
         <v>2024-05-01</v>
@@ -51258,7 +51258,7 @@
     </row>
     <row r="547">
       <c r="A547" t="str">
-        <v>608</v>
+        <v>710</v>
       </c>
       <c r="B547" t="str">
         <v>2024-05-02</v>
@@ -51281,7 +51281,7 @@
     </row>
     <row r="548">
       <c r="A548" t="str">
-        <v>609</v>
+        <v>711</v>
       </c>
       <c r="B548" t="str">
         <v>2024-05-03</v>
@@ -51304,7 +51304,7 @@
     </row>
     <row r="549">
       <c r="A549" t="str">
-        <v>610</v>
+        <v>712</v>
       </c>
       <c r="B549" t="str">
         <v>2024-05-03</v>
@@ -51327,7 +51327,7 @@
     </row>
     <row r="550">
       <c r="A550" t="str">
-        <v>611</v>
+        <v>713</v>
       </c>
       <c r="B550" t="str">
         <v>2024-05-04</v>
@@ -51350,7 +51350,7 @@
     </row>
     <row r="551">
       <c r="A551" t="str">
-        <v>612</v>
+        <v>714</v>
       </c>
       <c r="B551" t="str">
         <v>2024-05-04</v>
@@ -51373,7 +51373,7 @@
     </row>
     <row r="552">
       <c r="A552" t="str">
-        <v>614</v>
+        <v>716</v>
       </c>
       <c r="B552" t="str">
         <v>2024-05-05</v>
@@ -51396,7 +51396,7 @@
     </row>
     <row r="553">
       <c r="A553" t="str">
-        <v>615</v>
+        <v>717</v>
       </c>
       <c r="B553" t="str">
         <v>2024-05-06</v>
@@ -51419,7 +51419,7 @@
     </row>
     <row r="554">
       <c r="A554" t="str">
-        <v>616</v>
+        <v>718</v>
       </c>
       <c r="B554" t="str">
         <v>2024-05-06</v>
@@ -51442,7 +51442,7 @@
     </row>
     <row r="555">
       <c r="A555" t="str">
-        <v>617</v>
+        <v>719</v>
       </c>
       <c r="B555" t="str">
         <v>2024-05-07</v>
@@ -51465,7 +51465,7 @@
     </row>
     <row r="556">
       <c r="A556" t="str">
-        <v>619</v>
+        <v>722</v>
       </c>
       <c r="B556" t="str">
         <v>2024-05-09</v>
@@ -51488,7 +51488,7 @@
     </row>
     <row r="557">
       <c r="A557" t="str">
-        <v>620</v>
+        <v>723</v>
       </c>
       <c r="B557" t="str">
         <v>2024-05-10</v>
@@ -51511,7 +51511,7 @@
     </row>
     <row r="558">
       <c r="A558" t="str">
-        <v>621</v>
+        <v>724</v>
       </c>
       <c r="B558" t="str">
         <v>2024-05-11</v>
@@ -51534,7 +51534,7 @@
     </row>
     <row r="559">
       <c r="A559" t="str">
-        <v>622</v>
+        <v>725</v>
       </c>
       <c r="B559" t="str">
         <v>2024-05-11</v>
@@ -51557,7 +51557,7 @@
     </row>
     <row r="560">
       <c r="A560" t="str">
-        <v>623</v>
+        <v>726</v>
       </c>
       <c r="B560" t="str">
         <v>2024-05-11</v>
@@ -51580,7 +51580,7 @@
     </row>
     <row r="561">
       <c r="A561" t="str">
-        <v>624</v>
+        <v>727</v>
       </c>
       <c r="B561" t="str">
         <v>2024-05-11</v>
@@ -51603,7 +51603,7 @@
     </row>
     <row r="562">
       <c r="A562" t="str">
-        <v>625</v>
+        <v>728</v>
       </c>
       <c r="B562" t="str">
         <v>2024-05-11</v>
@@ -51626,7 +51626,7 @@
     </row>
     <row r="563">
       <c r="A563" t="str">
-        <v>626</v>
+        <v>729</v>
       </c>
       <c r="B563" t="str">
         <v>2024-05-11</v>
@@ -51649,7 +51649,7 @@
     </row>
     <row r="564">
       <c r="A564" t="str">
-        <v>627</v>
+        <v>730</v>
       </c>
       <c r="B564" t="str">
         <v>2024-05-11</v>
@@ -51672,7 +51672,7 @@
     </row>
     <row r="565">
       <c r="A565" t="str">
-        <v>628</v>
+        <v>731</v>
       </c>
       <c r="B565" t="str">
         <v>2024-05-11</v>
@@ -51695,7 +51695,7 @@
     </row>
     <row r="566">
       <c r="A566" t="str">
-        <v>629</v>
+        <v>732</v>
       </c>
       <c r="B566" t="str">
         <v>2024-05-12</v>
@@ -51718,7 +51718,7 @@
     </row>
     <row r="567">
       <c r="A567" t="str">
-        <v>630</v>
+        <v>733</v>
       </c>
       <c r="B567" t="str">
         <v>2024-05-12</v>
@@ -51741,7 +51741,7 @@
     </row>
     <row r="568">
       <c r="A568" t="str">
-        <v>631</v>
+        <v>734</v>
       </c>
       <c r="B568" t="str">
         <v>2024-05-14</v>
@@ -51764,7 +51764,7 @@
     </row>
     <row r="569">
       <c r="A569" t="str">
-        <v>633</v>
+        <v>736</v>
       </c>
       <c r="B569" t="str">
         <v>2024-05-15</v>
@@ -51787,7 +51787,7 @@
     </row>
     <row r="570">
       <c r="A570" t="str">
-        <v>634</v>
+        <v>737</v>
       </c>
       <c r="B570" t="str">
         <v>2024-05-16</v>
@@ -51810,7 +51810,7 @@
     </row>
     <row r="571">
       <c r="A571" t="str">
-        <v>635</v>
+        <v>738</v>
       </c>
       <c r="B571" t="str">
         <v>2024-05-16</v>
@@ -51833,7 +51833,7 @@
     </row>
     <row r="572">
       <c r="A572" t="str">
-        <v>636</v>
+        <v>739</v>
       </c>
       <c r="B572" t="str">
         <v>2024-05-17</v>
@@ -51856,7 +51856,7 @@
     </row>
     <row r="573">
       <c r="A573" t="str">
-        <v>637</v>
+        <v>741</v>
       </c>
       <c r="B573" t="str">
         <v>2024-05-18</v>
@@ -51879,7 +51879,7 @@
     </row>
     <row r="574">
       <c r="A574" t="str">
-        <v>638</v>
+        <v>742</v>
       </c>
       <c r="B574" t="str">
         <v>2024-05-18</v>
@@ -51902,7 +51902,7 @@
     </row>
     <row r="575">
       <c r="A575" t="str">
-        <v>639</v>
+        <v>743</v>
       </c>
       <c r="B575" t="str">
         <v>2024-05-19</v>
@@ -51925,7 +51925,7 @@
     </row>
     <row r="576">
       <c r="A576" t="str">
-        <v>640</v>
+        <v>744</v>
       </c>
       <c r="B576" t="str">
         <v>2024-05-19</v>
@@ -51948,7 +51948,7 @@
     </row>
     <row r="577">
       <c r="A577" t="str">
-        <v>641</v>
+        <v>745</v>
       </c>
       <c r="B577" t="str">
         <v>2024-05-20</v>
@@ -51971,7 +51971,7 @@
     </row>
     <row r="578">
       <c r="A578" t="str">
-        <v>642</v>
+        <v>746</v>
       </c>
       <c r="B578" t="str">
         <v>2024-05-20</v>
@@ -51994,7 +51994,7 @@
     </row>
     <row r="579">
       <c r="A579" t="str">
-        <v>643</v>
+        <v>747</v>
       </c>
       <c r="B579" t="str">
         <v>2024-05-20</v>
@@ -52017,7 +52017,7 @@
     </row>
     <row r="580">
       <c r="A580" t="str">
-        <v>644</v>
+        <v>748</v>
       </c>
       <c r="B580" t="str">
         <v>2024-05-20</v>
@@ -52040,7 +52040,7 @@
     </row>
     <row r="581">
       <c r="A581" t="str">
-        <v>645</v>
+        <v>749</v>
       </c>
       <c r="B581" t="str">
         <v>2024-05-20</v>
@@ -52063,7 +52063,7 @@
     </row>
     <row r="582">
       <c r="A582" t="str">
-        <v>646</v>
+        <v>750</v>
       </c>
       <c r="B582" t="str">
         <v>2024-05-20</v>
@@ -52086,7 +52086,7 @@
     </row>
     <row r="583">
       <c r="A583" t="str">
-        <v>647</v>
+        <v>751</v>
       </c>
       <c r="B583" t="str">
         <v>2024-05-20</v>
@@ -52109,7 +52109,7 @@
     </row>
     <row r="584">
       <c r="A584" t="str">
-        <v>649</v>
+        <v>753</v>
       </c>
       <c r="B584" t="str">
         <v>2024-05-21</v>
@@ -52132,7 +52132,7 @@
     </row>
     <row r="585">
       <c r="A585" t="str">
-        <v>650</v>
+        <v>754</v>
       </c>
       <c r="B585" t="str">
         <v>2024-05-21</v>
@@ -52155,7 +52155,7 @@
     </row>
     <row r="586">
       <c r="A586" t="str">
-        <v>651</v>
+        <v>755</v>
       </c>
       <c r="B586" t="str">
         <v>2024-05-21</v>
@@ -52178,7 +52178,7 @@
     </row>
     <row r="587">
       <c r="A587" t="str">
-        <v>652</v>
+        <v>756</v>
       </c>
       <c r="B587" t="str">
         <v>2024-05-21</v>
@@ -52201,7 +52201,7 @@
     </row>
     <row r="588">
       <c r="A588" t="str">
-        <v>653</v>
+        <v>757</v>
       </c>
       <c r="B588" t="str">
         <v>2024-05-21</v>
@@ -52224,7 +52224,7 @@
     </row>
     <row r="589">
       <c r="A589" t="str">
-        <v>654</v>
+        <v>758</v>
       </c>
       <c r="B589" t="str">
         <v>2024-05-21</v>
@@ -52247,7 +52247,7 @@
     </row>
     <row r="590">
       <c r="A590" t="str">
-        <v>655</v>
+        <v>759</v>
       </c>
       <c r="B590" t="str">
         <v>2024-05-21</v>
@@ -52270,7 +52270,7 @@
     </row>
     <row r="591">
       <c r="A591" t="str">
-        <v>656</v>
+        <v>760</v>
       </c>
       <c r="B591" t="str">
         <v>2024-05-22</v>
@@ -52293,7 +52293,7 @@
     </row>
     <row r="592">
       <c r="A592" t="str">
-        <v>657</v>
+        <v>761</v>
       </c>
       <c r="B592" t="str">
         <v>2024-05-23</v>
@@ -52316,7 +52316,7 @@
     </row>
     <row r="593">
       <c r="A593" t="str">
-        <v>658</v>
+        <v>762</v>
       </c>
       <c r="B593" t="str">
         <v>2024-05-24</v>
@@ -52339,7 +52339,7 @@
     </row>
     <row r="594">
       <c r="A594" t="str">
-        <v>659</v>
+        <v>764</v>
       </c>
       <c r="B594" t="str">
         <v>2024-05-25</v>
@@ -52362,7 +52362,7 @@
     </row>
     <row r="595">
       <c r="A595" t="str">
-        <v>660</v>
+        <v>765</v>
       </c>
       <c r="B595" t="str">
         <v>2024-05-25</v>
@@ -52385,7 +52385,7 @@
     </row>
     <row r="596">
       <c r="A596" t="str">
-        <v>661</v>
+        <v>766</v>
       </c>
       <c r="B596" t="str">
         <v>2024-05-26</v>
@@ -52408,7 +52408,7 @@
     </row>
     <row r="597">
       <c r="A597" t="str">
-        <v>662</v>
+        <v>767</v>
       </c>
       <c r="B597" t="str">
         <v>2024-05-26</v>
@@ -52431,7 +52431,7 @@
     </row>
     <row r="598">
       <c r="A598" t="str">
-        <v>663</v>
+        <v>768</v>
       </c>
       <c r="B598" t="str">
         <v>2024-05-26</v>
@@ -52454,7 +52454,7 @@
     </row>
     <row r="599">
       <c r="A599" t="str">
-        <v>664</v>
+        <v>770</v>
       </c>
       <c r="B599" t="str">
         <v>2024-05-27</v>
@@ -52477,7 +52477,7 @@
     </row>
     <row r="600">
       <c r="A600" t="str">
-        <v>665</v>
+        <v>771</v>
       </c>
       <c r="B600" t="str">
         <v>2024-05-28</v>
@@ -52500,7 +52500,7 @@
     </row>
     <row r="601">
       <c r="A601" t="str">
-        <v>666</v>
+        <v>772</v>
       </c>
       <c r="B601" t="str">
         <v>2024-05-29</v>
@@ -52523,7 +52523,7 @@
     </row>
     <row r="602">
       <c r="A602" t="str">
-        <v>667</v>
+        <v>773</v>
       </c>
       <c r="B602" t="str">
         <v>2024-05-30</v>
@@ -52546,7 +52546,7 @@
     </row>
     <row r="603">
       <c r="A603" t="str">
-        <v>668</v>
+        <v>774</v>
       </c>
       <c r="B603" t="str">
         <v>2024-05-31</v>
@@ -52569,7 +52569,7 @@
     </row>
     <row r="604">
       <c r="A604" t="str">
-        <v>669</v>
+        <v>775</v>
       </c>
       <c r="B604" t="str">
         <v>2024-05-31</v>
@@ -52592,7 +52592,7 @@
     </row>
     <row r="605">
       <c r="A605" t="str">
-        <v>670</v>
+        <v>776</v>
       </c>
       <c r="B605" t="str">
         <v>2024-05-31</v>
@@ -52615,7 +52615,7 @@
     </row>
     <row r="606">
       <c r="A606" t="str">
-        <v>671</v>
+        <v>777</v>
       </c>
       <c r="B606" t="str">
         <v>2024-05-31</v>
@@ -52638,7 +52638,7 @@
     </row>
     <row r="607">
       <c r="A607" t="str">
-        <v>672</v>
+        <v>778</v>
       </c>
       <c r="B607" t="str">
         <v>2024-05-31</v>
@@ -52661,7 +52661,7 @@
     </row>
     <row r="608">
       <c r="A608" t="str">
-        <v>673</v>
+        <v>779</v>
       </c>
       <c r="B608" t="str">
         <v>2024-05-31</v>
@@ -52684,7 +52684,7 @@
     </row>
     <row r="609">
       <c r="A609" t="str">
-        <v>674</v>
+        <v>780</v>
       </c>
       <c r="B609" t="str">
         <v>2024-05-31</v>
@@ -52707,7 +52707,7 @@
     </row>
     <row r="610">
       <c r="A610" t="str">
-        <v>675</v>
+        <v>781</v>
       </c>
       <c r="B610" t="str">
         <v>2024-05-31</v>
@@ -52730,7 +52730,7 @@
     </row>
     <row r="611">
       <c r="A611" t="str">
-        <v>677</v>
+        <v>783</v>
       </c>
       <c r="B611" t="str">
         <v>2024-06-01</v>
@@ -52753,7 +52753,7 @@
     </row>
     <row r="612">
       <c r="A612" t="str">
-        <v>678</v>
+        <v>784</v>
       </c>
       <c r="B612" t="str">
         <v>2024-06-01</v>
@@ -52776,7 +52776,7 @@
     </row>
     <row r="613">
       <c r="A613" t="str">
-        <v>679</v>
+        <v>785</v>
       </c>
       <c r="B613" t="str">
         <v>2024-06-01</v>
@@ -52799,7 +52799,7 @@
     </row>
     <row r="614">
       <c r="A614" t="str">
-        <v>680</v>
+        <v>786</v>
       </c>
       <c r="B614" t="str">
         <v>2024-06-01</v>
@@ -52822,7 +52822,7 @@
     </row>
     <row r="615">
       <c r="A615" t="str">
-        <v>681</v>
+        <v>787</v>
       </c>
       <c r="B615" t="str">
         <v>2024-06-01</v>
@@ -52845,7 +52845,7 @@
     </row>
     <row r="616">
       <c r="A616" t="str">
-        <v>682</v>
+        <v>788</v>
       </c>
       <c r="B616" t="str">
         <v>2024-06-01</v>
@@ -52868,7 +52868,7 @@
     </row>
     <row r="617">
       <c r="A617" t="str">
-        <v>683</v>
+        <v>789</v>
       </c>
       <c r="B617" t="str">
         <v>2024-06-01</v>
@@ -52891,7 +52891,7 @@
     </row>
     <row r="618">
       <c r="A618" t="str">
-        <v>684</v>
+        <v>790</v>
       </c>
       <c r="B618" t="str">
         <v>2024-06-01</v>
@@ -52914,7 +52914,7 @@
     </row>
     <row r="619">
       <c r="A619" t="str">
-        <v>685</v>
+        <v>791</v>
       </c>
       <c r="B619" t="str">
         <v>2024-06-01</v>
@@ -52937,7 +52937,7 @@
     </row>
     <row r="620">
       <c r="A620" t="str">
-        <v>686</v>
+        <v>793</v>
       </c>
       <c r="B620" t="str">
         <v>2024-06-02</v>
@@ -52960,7 +52960,7 @@
     </row>
     <row r="621">
       <c r="A621" t="str">
-        <v>688</v>
+        <v>795</v>
       </c>
       <c r="B621" t="str">
         <v>2024-06-03</v>
@@ -52983,7 +52983,7 @@
     </row>
     <row r="622">
       <c r="A622" t="str">
-        <v>689</v>
+        <v>796</v>
       </c>
       <c r="B622" t="str">
         <v>2024-06-04</v>
@@ -53006,7 +53006,7 @@
     </row>
     <row r="623">
       <c r="A623" t="str">
-        <v>691</v>
+        <v>799</v>
       </c>
       <c r="B623" t="str">
         <v>2024-06-06</v>
@@ -53029,7 +53029,7 @@
     </row>
     <row r="624">
       <c r="A624" t="str">
-        <v>692</v>
+        <v>800</v>
       </c>
       <c r="B624" t="str">
         <v>2024-06-07</v>
@@ -53052,7 +53052,7 @@
     </row>
     <row r="625">
       <c r="A625" t="str">
-        <v>693</v>
+        <v>801</v>
       </c>
       <c r="B625" t="str">
         <v>2024-06-08</v>
@@ -53075,7 +53075,7 @@
     </row>
     <row r="626">
       <c r="A626" t="str">
-        <v>694</v>
+        <v>802</v>
       </c>
       <c r="B626" t="str">
         <v>2024-06-08</v>
@@ -53098,7 +53098,7 @@
     </row>
     <row r="627">
       <c r="A627" t="str">
-        <v>695</v>
+        <v>803</v>
       </c>
       <c r="B627" t="str">
         <v>2024-06-08</v>
@@ -53121,7 +53121,7 @@
     </row>
     <row r="628">
       <c r="A628" t="str">
-        <v>696</v>
+        <v>804</v>
       </c>
       <c r="B628" t="str">
         <v>2024-06-08</v>
@@ -53144,7 +53144,7 @@
     </row>
     <row r="629">
       <c r="A629" t="str">
-        <v>697</v>
+        <v>805</v>
       </c>
       <c r="B629" t="str">
         <v>2024-06-08</v>
@@ -53167,7 +53167,7 @@
     </row>
     <row r="630">
       <c r="A630" t="str">
-        <v>698</v>
+        <v>806</v>
       </c>
       <c r="B630" t="str">
         <v>2024-06-08</v>
@@ -53190,7 +53190,7 @@
     </row>
     <row r="631">
       <c r="A631" t="str">
-        <v>699</v>
+        <v>807</v>
       </c>
       <c r="B631" t="str">
         <v>2024-06-08</v>
@@ -53213,7 +53213,7 @@
     </row>
     <row r="632">
       <c r="A632" t="str">
-        <v>700</v>
+        <v>808</v>
       </c>
       <c r="B632" t="str">
         <v>2024-06-08</v>
@@ -53236,7 +53236,7 @@
     </row>
     <row r="633">
       <c r="A633" t="str">
-        <v>701</v>
+        <v>809</v>
       </c>
       <c r="B633" t="str">
         <v>2024-06-08</v>
@@ -53259,7 +53259,7 @@
     </row>
     <row r="634">
       <c r="A634" t="str">
-        <v>702</v>
+        <v>810</v>
       </c>
       <c r="B634" t="str">
         <v>2024-06-08</v>
@@ -53282,7 +53282,7 @@
     </row>
     <row r="635">
       <c r="A635" t="str">
-        <v>703</v>
+        <v>811</v>
       </c>
       <c r="B635" t="str">
         <v>2024-06-08</v>
@@ -53305,7 +53305,7 @@
     </row>
     <row r="636">
       <c r="A636" t="str">
-        <v>704</v>
+        <v>812</v>
       </c>
       <c r="B636" t="str">
         <v>2024-06-09</v>
@@ -53328,7 +53328,7 @@
     </row>
     <row r="637">
       <c r="A637" t="str">
-        <v>705</v>
+        <v>813</v>
       </c>
       <c r="B637" t="str">
         <v>2024-06-09</v>
@@ -53351,7 +53351,7 @@
     </row>
     <row r="638">
       <c r="A638" t="str">
-        <v>706</v>
+        <v>814</v>
       </c>
       <c r="B638" t="str">
         <v>2024-06-09</v>
@@ -53374,7 +53374,7 @@
     </row>
     <row r="639">
       <c r="A639" t="str">
-        <v>707</v>
+        <v>815</v>
       </c>
       <c r="B639" t="str">
         <v>2024-06-09</v>
@@ -53397,7 +53397,7 @@
     </row>
     <row r="640">
       <c r="A640" t="str">
-        <v>708</v>
+        <v>816</v>
       </c>
       <c r="B640" t="str">
         <v>2024-06-09</v>
@@ -53420,7 +53420,7 @@
     </row>
     <row r="641">
       <c r="A641" t="str">
-        <v>709</v>
+        <v>817</v>
       </c>
       <c r="B641" t="str">
         <v>2024-06-09</v>
@@ -53443,7 +53443,7 @@
     </row>
     <row r="642">
       <c r="A642" t="str">
-        <v>710</v>
+        <v>818</v>
       </c>
       <c r="B642" t="str">
         <v>2024-06-09</v>
@@ -53466,7 +53466,7 @@
     </row>
     <row r="643">
       <c r="A643" t="str">
-        <v>711</v>
+        <v>819</v>
       </c>
       <c r="B643" t="str">
         <v>2024-06-09</v>
@@ -53489,7 +53489,7 @@
     </row>
     <row r="644">
       <c r="A644" t="str">
-        <v>712</v>
+        <v>820</v>
       </c>
       <c r="B644" t="str">
         <v>2024-06-10</v>
@@ -53512,7 +53512,7 @@
     </row>
     <row r="645">
       <c r="A645" t="str">
-        <v>713</v>
+        <v>821</v>
       </c>
       <c r="B645" t="str">
         <v>2024-06-11</v>
@@ -53535,7 +53535,7 @@
     </row>
     <row r="646">
       <c r="A646" t="str">
-        <v>714</v>
+        <v>822</v>
       </c>
       <c r="B646" t="str">
         <v>2024-06-12</v>
@@ -53558,7 +53558,7 @@
     </row>
     <row r="647">
       <c r="A647" t="str">
-        <v>715</v>
+        <v>823</v>
       </c>
       <c r="B647" t="str">
         <v>2024-06-13</v>
@@ -53581,7 +53581,7 @@
     </row>
     <row r="648">
       <c r="A648" t="str">
-        <v>716</v>
+        <v>824</v>
       </c>
       <c r="B648" t="str">
         <v>2024-06-14</v>
@@ -53604,7 +53604,7 @@
     </row>
     <row r="649">
       <c r="A649" t="str">
-        <v>717</v>
+        <v>825</v>
       </c>
       <c r="B649" t="str">
         <v>2024-06-16</v>
@@ -53627,7 +53627,7 @@
     </row>
     <row r="650">
       <c r="A650" t="str">
-        <v>718</v>
+        <v>826</v>
       </c>
       <c r="B650" t="str">
         <v>2024-06-17</v>
@@ -53650,7 +53650,7 @@
     </row>
     <row r="651">
       <c r="A651" t="str">
-        <v>719</v>
+        <v>827</v>
       </c>
       <c r="B651" t="str">
         <v>2024-06-18</v>
@@ -53673,7 +53673,7 @@
     </row>
     <row r="652">
       <c r="A652" t="str">
-        <v>720</v>
+        <v>828</v>
       </c>
       <c r="B652" t="str">
         <v>2024-06-20</v>
@@ -53696,7 +53696,7 @@
     </row>
     <row r="653">
       <c r="A653" t="str">
-        <v>722</v>
+        <v>830</v>
       </c>
       <c r="B653" t="str">
         <v>2024-07-01</v>
@@ -53719,7 +53719,7 @@
     </row>
     <row r="654">
       <c r="A654" t="str">
-        <v>723</v>
+        <v>831</v>
       </c>
       <c r="B654" t="str">
         <v>2024-07-01</v>
@@ -53742,7 +53742,7 @@
     </row>
     <row r="655">
       <c r="A655" t="str">
-        <v>724</v>
+        <v>832</v>
       </c>
       <c r="B655" t="str">
         <v>2024-07-01</v>
@@ -53765,7 +53765,7 @@
     </row>
     <row r="656">
       <c r="A656" t="str">
-        <v>725</v>
+        <v>833</v>
       </c>
       <c r="B656" t="str">
         <v>2024-07-16</v>
@@ -53788,7 +53788,7 @@
     </row>
     <row r="657">
       <c r="A657" t="str">
-        <v>726</v>
+        <v>834</v>
       </c>
       <c r="B657" t="str">
         <v>2024-07-17</v>
@@ -53811,7 +53811,7 @@
     </row>
     <row r="658">
       <c r="A658" t="str">
-        <v>727</v>
+        <v>835</v>
       </c>
       <c r="B658" t="str">
         <v>2024-07-25</v>
@@ -53834,7 +53834,7 @@
     </row>
     <row r="659">
       <c r="A659" t="str">
-        <v>728</v>
+        <v>836</v>
       </c>
       <c r="B659" t="str">
         <v>2024-07-26</v>
@@ -53857,7 +53857,7 @@
     </row>
     <row r="660">
       <c r="A660" t="str">
-        <v>729</v>
+        <v>837</v>
       </c>
       <c r="B660" t="str">
         <v>2024-08-07</v>
@@ -53880,7 +53880,7 @@
     </row>
     <row r="661">
       <c r="A661" t="str">
-        <v>731</v>
+        <v>839</v>
       </c>
       <c r="B661" t="str">
         <v>2024-10-05</v>
@@ -53903,7 +53903,7 @@
     </row>
     <row r="662">
       <c r="A662" t="str">
-        <v>732</v>
+        <v>840</v>
       </c>
       <c r="B662" t="str">
         <v>2024-10-05</v>
@@ -53926,7 +53926,7 @@
     </row>
     <row r="663">
       <c r="A663" t="str">
-        <v>733</v>
+        <v>841</v>
       </c>
       <c r="B663" t="str">
         <v>2024-10-05</v>
@@ -53949,7 +53949,7 @@
     </row>
     <row r="664">
       <c r="A664" t="str">
-        <v>734</v>
+        <v>842</v>
       </c>
       <c r="B664" t="str">
         <v>2024-10-05</v>
@@ -53972,7 +53972,7 @@
     </row>
     <row r="665">
       <c r="A665" t="str">
-        <v>735</v>
+        <v>843</v>
       </c>
       <c r="B665" t="str">
         <v>2024-10-05</v>
@@ -53995,7 +53995,7 @@
     </row>
     <row r="666">
       <c r="A666" t="str">
-        <v>736</v>
+        <v>844</v>
       </c>
       <c r="B666" t="str">
         <v>2024-10-05</v>
@@ -54018,7 +54018,7 @@
     </row>
     <row r="667">
       <c r="A667" t="str">
-        <v>737</v>
+        <v>845</v>
       </c>
       <c r="B667" t="str">
         <v>2024-10-05</v>
@@ -54041,7 +54041,7 @@
     </row>
     <row r="668">
       <c r="A668" t="str">
-        <v>745</v>
+        <v>853</v>
       </c>
       <c r="B668" t="str">
         <v>2024-11-17</v>
@@ -54064,7 +54064,7 @@
     </row>
     <row r="669">
       <c r="A669" t="str">
-        <v>746</v>
+        <v>854</v>
       </c>
       <c r="B669" t="str">
         <v>2024-11-18</v>
@@ -54087,7 +54087,7 @@
     </row>
     <row r="670">
       <c r="A670" t="str">
-        <v>750</v>
+        <v>858</v>
       </c>
       <c r="B670" t="str">
         <v>2024-12-07</v>
@@ -54110,7 +54110,7 @@
     </row>
     <row r="671">
       <c r="A671" t="str">
-        <v>751</v>
+        <v>859</v>
       </c>
       <c r="B671" t="str">
         <v>2024-12-08</v>
@@ -54133,7 +54133,7 @@
     </row>
     <row r="672">
       <c r="A672" t="str">
-        <v>752</v>
+        <v>860</v>
       </c>
       <c r="B672" t="str">
         <v>2024-12-08</v>
@@ -54156,7 +54156,7 @@
     </row>
     <row r="673">
       <c r="A673" t="str">
-        <v>753</v>
+        <v>861</v>
       </c>
       <c r="B673" t="str">
         <v>2024-12-09</v>
@@ -54179,7 +54179,7 @@
     </row>
     <row r="674">
       <c r="A674" t="str">
-        <v>754</v>
+        <v>862</v>
       </c>
       <c r="B674" t="str">
         <v>2024-12-17</v>
@@ -54202,7 +54202,7 @@
     </row>
     <row r="675">
       <c r="A675" t="str">
-        <v>755</v>
+        <v>863</v>
       </c>
       <c r="B675" t="str">
         <v>2024-12-18</v>
@@ -54225,7 +54225,7 @@
     </row>
     <row r="676">
       <c r="A676" t="str">
-        <v>756</v>
+        <v>864</v>
       </c>
       <c r="B676" t="str">
         <v>2024-12-20</v>
@@ -54248,7 +54248,7 @@
     </row>
     <row r="677">
       <c r="A677" t="str">
-        <v>757</v>
+        <v>865</v>
       </c>
       <c r="B677" t="str">
         <v>2024-12-21</v>
@@ -54271,7 +54271,7 @@
     </row>
     <row r="678">
       <c r="A678" t="str">
-        <v>758</v>
+        <v>866</v>
       </c>
       <c r="B678" t="str">
         <v>2024-12-21</v>
@@ -54294,7 +54294,7 @@
     </row>
     <row r="679">
       <c r="A679" t="str">
-        <v>759</v>
+        <v>867</v>
       </c>
       <c r="B679" t="str">
         <v>2024-12-25</v>
@@ -54317,7 +54317,7 @@
     </row>
     <row r="680">
       <c r="A680" t="str">
-        <v>760</v>
+        <v>868</v>
       </c>
       <c r="B680" t="str">
         <v>2024-12-26</v>
@@ -54340,7 +54340,7 @@
     </row>
     <row r="681">
       <c r="A681" t="str">
-        <v>762</v>
+        <v>870</v>
       </c>
       <c r="B681" t="str">
         <v>2024-12-31</v>
@@ -54363,7 +54363,7 @@
     </row>
     <row r="682">
       <c r="A682" t="str">
-        <v>763</v>
+        <v>871</v>
       </c>
       <c r="B682" t="str">
         <v>2025-01-02</v>
@@ -54386,7 +54386,7 @@
     </row>
     <row r="683">
       <c r="A683" t="str">
-        <v>764</v>
+        <v>872</v>
       </c>
       <c r="B683" t="str">
         <v>2025-01-02</v>
@@ -54409,7 +54409,7 @@
     </row>
     <row r="684">
       <c r="A684" t="str">
-        <v>765</v>
+        <v>873</v>
       </c>
       <c r="B684" t="str">
         <v>2025-01-02</v>
@@ -54432,7 +54432,7 @@
     </row>
     <row r="685">
       <c r="A685" t="str">
-        <v>766</v>
+        <v>874</v>
       </c>
       <c r="B685" t="str">
         <v>2025-01-02</v>
@@ -54455,7 +54455,7 @@
     </row>
     <row r="686">
       <c r="A686" t="str">
-        <v>767</v>
+        <v>875</v>
       </c>
       <c r="B686" t="str">
         <v>2025-01-02</v>
@@ -54478,7 +54478,7 @@
     </row>
     <row r="687">
       <c r="A687" t="str">
-        <v>768</v>
+        <v>876</v>
       </c>
       <c r="B687" t="str">
         <v>2025-01-03</v>
@@ -54501,7 +54501,7 @@
     </row>
     <row r="688">
       <c r="A688" t="str">
-        <v>769</v>
+        <v>877</v>
       </c>
       <c r="B688" t="str">
         <v>2025-01-03</v>
@@ -54524,7 +54524,7 @@
     </row>
     <row r="689">
       <c r="A689" t="str">
-        <v>770</v>
+        <v>878</v>
       </c>
       <c r="B689" t="str">
         <v>2025-01-03</v>
@@ -54547,7 +54547,7 @@
     </row>
     <row r="690">
       <c r="A690" t="str">
-        <v>771</v>
+        <v>879</v>
       </c>
       <c r="B690" t="str">
         <v>2025-01-05</v>
@@ -54570,7 +54570,7 @@
     </row>
     <row r="691">
       <c r="A691" t="str">
-        <v>775</v>
+        <v>883</v>
       </c>
       <c r="B691" t="str">
         <v>2025-03-08</v>
@@ -54593,7 +54593,7 @@
     </row>
     <row r="692">
       <c r="A692" t="str">
-        <v>776</v>
+        <v>884</v>
       </c>
       <c r="B692" t="str">
         <v>2025-03-09</v>
@@ -54616,7 +54616,7 @@
     </row>
     <row r="693">
       <c r="A693" t="str">
-        <v>777</v>
+        <v>885</v>
       </c>
       <c r="B693" t="str">
         <v>2025-03-09</v>
@@ -54639,7 +54639,7 @@
     </row>
     <row r="694">
       <c r="A694" t="str">
-        <v>778</v>
+        <v>886</v>
       </c>
       <c r="B694" t="str">
         <v>2025-03-10</v>
@@ -54662,7 +54662,7 @@
     </row>
     <row r="695">
       <c r="A695" t="str">
-        <v>779</v>
+        <v>887</v>
       </c>
       <c r="B695" t="str">
         <v>2025-03-10</v>
@@ -54685,7 +54685,7 @@
     </row>
     <row r="696">
       <c r="A696" t="str">
-        <v>781</v>
+        <v>889</v>
       </c>
       <c r="B696" t="str">
         <v>2025-03-11</v>
@@ -54708,7 +54708,7 @@
     </row>
     <row r="697">
       <c r="A697" t="str">
-        <v>782</v>
+        <v>890</v>
       </c>
       <c r="B697" t="str">
         <v>2025-03-12</v>
@@ -54731,7 +54731,7 @@
     </row>
     <row r="698">
       <c r="A698" t="str">
-        <v>783</v>
+        <v>891</v>
       </c>
       <c r="B698" t="str">
         <v>2025-03-13</v>
@@ -54754,7 +54754,7 @@
     </row>
     <row r="699">
       <c r="A699" t="str">
-        <v>784</v>
+        <v>892</v>
       </c>
       <c r="B699" t="str">
         <v>2025-03-13</v>
@@ -54777,7 +54777,7 @@
     </row>
     <row r="700">
       <c r="A700" t="str">
-        <v>785</v>
+        <v>893</v>
       </c>
       <c r="B700" t="str">
         <v>2025-03-13</v>
@@ -54800,7 +54800,7 @@
     </row>
     <row r="701">
       <c r="A701" t="str">
-        <v>786</v>
+        <v>894</v>
       </c>
       <c r="B701" t="str">
         <v>2025-03-13</v>
@@ -54823,7 +54823,7 @@
     </row>
     <row r="702">
       <c r="A702" t="str">
-        <v>787</v>
+        <v>895</v>
       </c>
       <c r="B702" t="str">
         <v>2025-03-13</v>
@@ -54846,7 +54846,7 @@
     </row>
     <row r="703">
       <c r="A703" t="str">
-        <v>788</v>
+        <v>896</v>
       </c>
       <c r="B703" t="str">
         <v>2025-03-16</v>
@@ -54869,7 +54869,7 @@
     </row>
     <row r="704">
       <c r="A704" t="str">
-        <v>789</v>
+        <v>897</v>
       </c>
       <c r="B704" t="str">
         <v>2025-03-17</v>
@@ -54892,7 +54892,7 @@
     </row>
     <row r="705">
       <c r="A705" t="str">
-        <v>790</v>
+        <v>898</v>
       </c>
       <c r="B705" t="str">
         <v>2025-03-18</v>
@@ -54915,7 +54915,7 @@
     </row>
     <row r="706">
       <c r="A706" t="str">
-        <v>791</v>
+        <v>899</v>
       </c>
       <c r="B706" t="str">
         <v>2025-03-18</v>
@@ -54938,7 +54938,7 @@
     </row>
     <row r="707">
       <c r="A707" t="str">
-        <v>792</v>
+        <v>900</v>
       </c>
       <c r="B707" t="str">
         <v>2025-03-19</v>
@@ -54961,7 +54961,7 @@
     </row>
     <row r="708">
       <c r="A708" t="str">
-        <v>793</v>
+        <v>901</v>
       </c>
       <c r="B708" t="str">
         <v>2025-03-20</v>
@@ -54984,7 +54984,7 @@
     </row>
     <row r="709">
       <c r="A709" t="str">
-        <v>794</v>
+        <v>902</v>
       </c>
       <c r="B709" t="str">
         <v>2025-03-21</v>
@@ -55007,7 +55007,7 @@
     </row>
     <row r="710">
       <c r="A710" t="str">
-        <v>795</v>
+        <v>903</v>
       </c>
       <c r="B710" t="str">
         <v>2025-03-21</v>
@@ -55030,7 +55030,7 @@
     </row>
     <row r="711">
       <c r="A711" t="str">
-        <v>796</v>
+        <v>904</v>
       </c>
       <c r="B711" t="str">
         <v>2025-03-21</v>
@@ -55053,7 +55053,7 @@
     </row>
     <row r="712">
       <c r="A712" t="str">
-        <v>797</v>
+        <v>905</v>
       </c>
       <c r="B712" t="str">
         <v>2025-03-23</v>
@@ -55076,7 +55076,7 @@
     </row>
     <row r="713">
       <c r="A713" t="str">
-        <v>798</v>
+        <v>906</v>
       </c>
       <c r="B713" t="str">
         <v>2025-03-24</v>
@@ -55099,7 +55099,7 @@
     </row>
     <row r="714">
       <c r="A714" t="str">
-        <v>799</v>
+        <v>907</v>
       </c>
       <c r="B714" t="str">
         <v>2025-03-25</v>
@@ -55122,7 +55122,7 @@
     </row>
     <row r="715">
       <c r="A715" t="str">
-        <v>800</v>
+        <v>908</v>
       </c>
       <c r="B715" t="str">
         <v>2025-03-25</v>
@@ -55145,7 +55145,7 @@
     </row>
     <row r="716">
       <c r="A716" t="str">
-        <v>801</v>
+        <v>909</v>
       </c>
       <c r="B716" t="str">
         <v>2025-03-25</v>
@@ -55168,7 +55168,7 @@
     </row>
     <row r="717">
       <c r="A717" t="str">
-        <v>802</v>
+        <v>910</v>
       </c>
       <c r="B717" t="str">
         <v>2025-03-25</v>
@@ -55191,7 +55191,7 @@
     </row>
     <row r="718">
       <c r="A718" t="str">
-        <v>803</v>
+        <v>911</v>
       </c>
       <c r="B718" t="str">
         <v>2025-03-27</v>
@@ -55214,7 +55214,7 @@
     </row>
     <row r="719">
       <c r="A719" t="str">
-        <v>804</v>
+        <v>912</v>
       </c>
       <c r="B719" t="str">
         <v>2025-03-28</v>
@@ -55237,7 +55237,7 @@
     </row>
     <row r="720">
       <c r="A720" t="str">
-        <v>805</v>
+        <v>913</v>
       </c>
       <c r="B720" t="str">
         <v>2025-03-29</v>
@@ -55260,7 +55260,7 @@
     </row>
     <row r="721">
       <c r="A721" t="str">
-        <v>806</v>
+        <v>914</v>
       </c>
       <c r="B721" t="str">
         <v>2025-03-31</v>
@@ -55283,7 +55283,7 @@
     </row>
     <row r="722">
       <c r="A722" t="str">
-        <v>807</v>
+        <v>915</v>
       </c>
       <c r="B722" t="str">
         <v>2025-03-31</v>
@@ -55306,7 +55306,7 @@
     </row>
     <row r="723">
       <c r="A723" t="str">
-        <v>808</v>
+        <v>916</v>
       </c>
       <c r="B723" t="str">
         <v>2025-03-31</v>
@@ -55329,7 +55329,7 @@
     </row>
     <row r="724">
       <c r="A724" t="str">
-        <v>809</v>
+        <v>917</v>
       </c>
       <c r="B724" t="str">
         <v>2025-04-01</v>
@@ -55352,7 +55352,7 @@
     </row>
     <row r="725">
       <c r="A725" t="str">
-        <v>810</v>
+        <v>918</v>
       </c>
       <c r="B725" t="str">
         <v>2025-04-01</v>
@@ -55375,7 +55375,7 @@
     </row>
     <row r="726">
       <c r="A726" t="str">
-        <v>811</v>
+        <v>919</v>
       </c>
       <c r="B726" t="str">
         <v>2025-04-01</v>
@@ -55398,7 +55398,7 @@
     </row>
     <row r="727">
       <c r="A727" t="str">
-        <v>812</v>
+        <v>920</v>
       </c>
       <c r="B727" t="str">
         <v>2025-04-01</v>
@@ -55421,7 +55421,7 @@
     </row>
     <row r="728">
       <c r="A728" t="str">
-        <v>813</v>
+        <v>921</v>
       </c>
       <c r="B728" t="str">
         <v>2025-04-01</v>
@@ -55444,7 +55444,7 @@
     </row>
     <row r="729">
       <c r="A729" t="str">
-        <v>815</v>
+        <v>923</v>
       </c>
       <c r="B729" t="str">
         <v>2025-04-02</v>
@@ -55467,7 +55467,7 @@
     </row>
     <row r="730">
       <c r="A730" t="str">
-        <v>816</v>
+        <v>924</v>
       </c>
       <c r="B730" t="str">
         <v>2025-04-02</v>
@@ -55490,7 +55490,7 @@
     </row>
     <row r="731">
       <c r="A731" t="str">
-        <v>817</v>
+        <v>925</v>
       </c>
       <c r="B731" t="str">
         <v>2025-04-05</v>
@@ -55513,7 +55513,7 @@
     </row>
     <row r="732">
       <c r="A732" t="str">
-        <v>818</v>
+        <v>926</v>
       </c>
       <c r="B732" t="str">
         <v>2025-04-06</v>
@@ -55536,7 +55536,7 @@
     </row>
     <row r="733">
       <c r="A733" t="str">
-        <v>819</v>
+        <v>927</v>
       </c>
       <c r="B733" t="str">
         <v>2025-04-07</v>
@@ -55559,7 +55559,7 @@
     </row>
     <row r="734">
       <c r="A734" t="str">
-        <v>820</v>
+        <v>928</v>
       </c>
       <c r="B734" t="str">
         <v>2025-04-08</v>
@@ -55582,7 +55582,7 @@
     </row>
     <row r="735">
       <c r="A735" t="str">
-        <v>821</v>
+        <v>929</v>
       </c>
       <c r="B735" t="str">
         <v>2025-04-08</v>
@@ -55605,7 +55605,7 @@
     </row>
     <row r="736">
       <c r="A736" t="str">
-        <v>822</v>
+        <v>930</v>
       </c>
       <c r="B736" t="str">
         <v>2025-04-09</v>
@@ -55628,7 +55628,7 @@
     </row>
     <row r="737">
       <c r="A737" t="str">
-        <v>823</v>
+        <v>931</v>
       </c>
       <c r="B737" t="str">
         <v>2025-04-09</v>
@@ -55651,7 +55651,7 @@
     </row>
     <row r="738">
       <c r="A738" t="str">
-        <v>824</v>
+        <v>932</v>
       </c>
       <c r="B738" t="str">
         <v>2025-04-11</v>
@@ -55674,7 +55674,7 @@
     </row>
     <row r="739">
       <c r="A739" t="str">
-        <v>825</v>
+        <v>933</v>
       </c>
       <c r="B739" t="str">
         <v>2025-04-12</v>
@@ -55697,7 +55697,7 @@
     </row>
     <row r="740">
       <c r="A740" t="str">
-        <v>826</v>
+        <v>934</v>
       </c>
       <c r="B740" t="str">
         <v>2025-04-13</v>
@@ -55720,7 +55720,7 @@
     </row>
     <row r="741">
       <c r="A741" t="str">
-        <v>827</v>
+        <v>935</v>
       </c>
       <c r="B741" t="str">
         <v>2025-04-14</v>
@@ -55743,7 +55743,7 @@
     </row>
     <row r="742">
       <c r="A742" t="str">
-        <v>828</v>
+        <v>936</v>
       </c>
       <c r="B742" t="str">
         <v>2025-04-14</v>
@@ -55766,7 +55766,7 @@
     </row>
     <row r="743">
       <c r="A743" t="str">
-        <v>829</v>
+        <v>937</v>
       </c>
       <c r="B743" t="str">
         <v>2025-04-18</v>
@@ -55789,7 +55789,7 @@
     </row>
     <row r="744">
       <c r="A744" t="str">
-        <v>830</v>
+        <v>938</v>
       </c>
       <c r="B744" t="str">
         <v>2025-04-20</v>
@@ -55812,7 +55812,7 @@
     </row>
     <row r="745">
       <c r="A745" t="str">
-        <v>831</v>
+        <v>939</v>
       </c>
       <c r="B745" t="str">
         <v>2025-04-21</v>
@@ -55835,7 +55835,7 @@
     </row>
     <row r="746">
       <c r="A746" t="str">
-        <v>832</v>
+        <v>940</v>
       </c>
       <c r="B746" t="str">
         <v>2025-04-22</v>
@@ -55858,7 +55858,7 @@
     </row>
     <row r="747">
       <c r="A747" t="str">
-        <v>833</v>
+        <v>941</v>
       </c>
       <c r="B747" t="str">
         <v>2025-04-22</v>
@@ -55881,7 +55881,7 @@
     </row>
     <row r="748">
       <c r="A748" t="str">
-        <v>834</v>
+        <v>942</v>
       </c>
       <c r="B748" t="str">
         <v>2025-04-23</v>
@@ -55904,7 +55904,7 @@
     </row>
     <row r="749">
       <c r="A749" t="str">
-        <v>835</v>
+        <v>943</v>
       </c>
       <c r="B749" t="str">
         <v>2025-04-24</v>
@@ -55927,7 +55927,7 @@
     </row>
     <row r="750">
       <c r="A750" t="str">
-        <v>838</v>
+        <v>946</v>
       </c>
       <c r="B750" t="str">
         <v>2025-04-27</v>
@@ -55950,7 +55950,7 @@
     </row>
     <row r="751">
       <c r="A751" t="str">
-        <v>839</v>
+        <v>947</v>
       </c>
       <c r="B751" t="str">
         <v>2025-04-28</v>
@@ -55973,7 +55973,7 @@
     </row>
     <row r="752">
       <c r="A752" t="str">
-        <v>840</v>
+        <v>948</v>
       </c>
       <c r="B752" t="str">
         <v>2025-04-29</v>
@@ -55996,7 +55996,7 @@
     </row>
     <row r="753">
       <c r="A753" t="str">
-        <v>842</v>
+        <v>950</v>
       </c>
       <c r="B753" t="str">
         <v>2025-05-01</v>
@@ -56019,7 +56019,7 @@
     </row>
     <row r="754">
       <c r="A754" t="str">
-        <v>843</v>
+        <v>951</v>
       </c>
       <c r="B754" t="str">
         <v>2025-05-01</v>
@@ -56042,7 +56042,7 @@
     </row>
     <row r="755">
       <c r="A755" t="str">
-        <v>844</v>
+        <v>952</v>
       </c>
       <c r="B755" t="str">
         <v>2025-05-01</v>
@@ -56065,7 +56065,7 @@
     </row>
     <row r="756">
       <c r="A756" t="str">
-        <v>845</v>
+        <v>953</v>
       </c>
       <c r="B756" t="str">
         <v>2025-05-01</v>
@@ -56088,7 +56088,7 @@
     </row>
     <row r="757">
       <c r="A757" t="str">
-        <v>847</v>
+        <v>955</v>
       </c>
       <c r="B757" t="str">
         <v>2025-05-03</v>
@@ -56111,7 +56111,7 @@
     </row>
     <row r="758">
       <c r="A758" t="str">
-        <v>848</v>
+        <v>956</v>
       </c>
       <c r="B758" t="str">
         <v>2025-05-04</v>
@@ -56134,7 +56134,7 @@
     </row>
     <row r="759">
       <c r="A759" t="str">
-        <v>852</v>
+        <v>960</v>
       </c>
       <c r="B759" t="str">
         <v>2025-05-06</v>
@@ -56157,7 +56157,7 @@
     </row>
     <row r="760">
       <c r="A760" t="str">
-        <v>853</v>
+        <v>961</v>
       </c>
       <c r="B760" t="str">
         <v>2025-05-07</v>
@@ -56180,7 +56180,7 @@
     </row>
     <row r="761">
       <c r="A761" t="str">
-        <v>857</v>
+        <v>965</v>
       </c>
       <c r="B761" t="str">
         <v>2025-05-11</v>
@@ -56203,7 +56203,7 @@
     </row>
     <row r="762">
       <c r="A762" t="str">
-        <v>858</v>
+        <v>966</v>
       </c>
       <c r="B762" t="str">
         <v>2025-05-13</v>
@@ -56226,7 +56226,7 @@
     </row>
     <row r="763">
       <c r="A763" t="str">
-        <v>860</v>
+        <v>968</v>
       </c>
       <c r="B763" t="str">
         <v>2025-05-15</v>
@@ -56249,7 +56249,7 @@
     </row>
     <row r="764">
       <c r="A764" t="str">
-        <v>861</v>
+        <v>969</v>
       </c>
       <c r="B764" t="str">
         <v>2025-05-16</v>
@@ -56272,7 +56272,7 @@
     </row>
     <row r="765">
       <c r="A765" t="str">
-        <v>862</v>
+        <v>970</v>
       </c>
       <c r="B765" t="str">
         <v>2025-05-18</v>
@@ -56295,7 +56295,7 @@
     </row>
     <row r="766">
       <c r="A766" t="str">
-        <v>863</v>
+        <v>971</v>
       </c>
       <c r="B766" t="str">
         <v>2025-05-19</v>
@@ -56318,7 +56318,7 @@
     </row>
     <row r="767">
       <c r="A767" t="str">
-        <v>864</v>
+        <v>972</v>
       </c>
       <c r="B767" t="str">
         <v>2025-05-20</v>
@@ -56341,7 +56341,7 @@
     </row>
     <row r="768">
       <c r="A768" t="str">
-        <v>865</v>
+        <v>973</v>
       </c>
       <c r="B768" t="str">
         <v>2025-05-22</v>
@@ -56364,7 +56364,7 @@
     </row>
     <row r="769">
       <c r="A769" t="str">
-        <v>866</v>
+        <v>974</v>
       </c>
       <c r="B769" t="str">
         <v>2025-05-23</v>
@@ -56387,7 +56387,7 @@
     </row>
     <row r="770">
       <c r="A770" t="str">
-        <v>867</v>
+        <v>975</v>
       </c>
       <c r="B770" t="str">
         <v>2025-05-26</v>
@@ -56410,7 +56410,7 @@
     </row>
     <row r="771">
       <c r="A771" t="str">
-        <v>868</v>
+        <v>976</v>
       </c>
       <c r="B771" t="str">
         <v>2025-05-27</v>
@@ -56433,7 +56433,7 @@
     </row>
     <row r="772">
       <c r="A772" t="str">
-        <v>869</v>
+        <v>977</v>
       </c>
       <c r="B772" t="str">
         <v>2025-05-29</v>
@@ -56456,7 +56456,7 @@
     </row>
     <row r="773">
       <c r="A773" t="str">
-        <v>870</v>
+        <v>978</v>
       </c>
       <c r="B773" t="str">
         <v>2025-05-30</v>
@@ -56479,7 +56479,7 @@
     </row>
     <row r="774">
       <c r="A774" t="str">
-        <v>871</v>
+        <v>979</v>
       </c>
       <c r="B774" t="str">
         <v>2025-05-30</v>
@@ -56502,7 +56502,7 @@
     </row>
     <row r="775">
       <c r="A775" t="str">
-        <v>872</v>
+        <v>980</v>
       </c>
       <c r="B775" t="str">
         <v>2025-05-30</v>
@@ -56525,7 +56525,7 @@
     </row>
     <row r="776">
       <c r="A776" t="str">
-        <v>873</v>
+        <v>981</v>
       </c>
       <c r="B776" t="str">
         <v>2025-06-01</v>
@@ -56548,7 +56548,7 @@
     </row>
     <row r="777">
       <c r="A777" t="str">
-        <v>874</v>
+        <v>982</v>
       </c>
       <c r="B777" t="str">
         <v>2025-06-02</v>
@@ -56571,7 +56571,7 @@
     </row>
     <row r="778">
       <c r="A778" t="str">
-        <v>875</v>
+        <v>983</v>
       </c>
       <c r="B778" t="str">
         <v>2025-06-05</v>
@@ -56594,7 +56594,7 @@
     </row>
     <row r="779">
       <c r="A779" t="str">
-        <v>876</v>
+        <v>984</v>
       </c>
       <c r="B779" t="str">
         <v>2025-06-09</v>
@@ -56617,7 +56617,7 @@
     </row>
     <row r="780">
       <c r="A780" t="str">
-        <v>877</v>
+        <v>985</v>
       </c>
       <c r="B780" t="str">
         <v>2025-06-10</v>
@@ -56640,7 +56640,7 @@
     </row>
     <row r="781">
       <c r="A781" t="str">
-        <v>878</v>
+        <v>986</v>
       </c>
       <c r="B781" t="str">
         <v>2025-06-10</v>
@@ -56663,7 +56663,7 @@
     </row>
     <row r="782">
       <c r="A782" t="str">
-        <v>879</v>
+        <v>987</v>
       </c>
       <c r="B782" t="str">
         <v>2025-06-10</v>
@@ -56686,7 +56686,7 @@
     </row>
     <row r="783">
       <c r="A783" t="str">
-        <v>880</v>
+        <v>988</v>
       </c>
       <c r="B783" t="str">
         <v>2025-06-10</v>
@@ -56709,7 +56709,7 @@
     </row>
     <row r="784">
       <c r="A784" t="str">
-        <v>881</v>
+        <v>989</v>
       </c>
       <c r="B784" t="str">
         <v>2025-06-10</v>
@@ -56732,7 +56732,7 @@
     </row>
     <row r="785">
       <c r="A785" t="str">
-        <v>882</v>
+        <v>990</v>
       </c>
       <c r="B785" t="str">
         <v>2025-06-10</v>
@@ -56755,7 +56755,7 @@
     </row>
     <row r="786">
       <c r="A786" t="str">
-        <v>883</v>
+        <v>991</v>
       </c>
       <c r="B786" t="str">
         <v>2025-06-10</v>
@@ -56778,7 +56778,7 @@
     </row>
     <row r="787">
       <c r="A787" t="str">
-        <v>884</v>
+        <v>992</v>
       </c>
       <c r="B787" t="str">
         <v>2025-06-10</v>
@@ -56801,7 +56801,7 @@
     </row>
     <row r="788">
       <c r="A788" t="str">
-        <v>885</v>
+        <v>993</v>
       </c>
       <c r="B788" t="str">
         <v>2025-06-10</v>
@@ -56824,7 +56824,7 @@
     </row>
     <row r="789">
       <c r="A789" t="str">
-        <v>886</v>
+        <v>994</v>
       </c>
       <c r="B789" t="str">
         <v>2025-06-10</v>
@@ -56847,7 +56847,7 @@
     </row>
     <row r="790">
       <c r="A790" t="str">
-        <v>887</v>
+        <v>995</v>
       </c>
       <c r="B790" t="str">
         <v>2025-06-10</v>
@@ -56870,7 +56870,7 @@
     </row>
     <row r="791">
       <c r="A791" t="str">
-        <v>888</v>
+        <v>996</v>
       </c>
       <c r="B791" t="str">
         <v>2025-06-10</v>

</xml_diff>

<commit_message>
Enhance Gitai application by adding customer aliases functionality to improve name consistency across income and receivables modules. Update index.html to include new customer-aliases.js script and modify existing JavaScript files to utilize aliases for customer names. Increment versioning for related scripts to reflect these changes. Update Excel workbooks (Gitai-M1.xlsx, Gitai-M2.xlsx, Gitai.xlsx) to ensure data alignment with recent modifications.
</commit_message>
<xml_diff>
--- a/Gitai-M1.xlsx
+++ b/Gitai-M1.xlsx
@@ -7640,7 +7640,7 @@
         <v>2022-07-27</v>
       </c>
       <c r="C211" t="str">
-        <v>Dhore gajanan</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D211" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -8408,7 +8408,7 @@
         <v>2022-08-19</v>
       </c>
       <c r="C235" t="str">
-        <v>Dhore gajanan</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D235" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -11352,7 +11352,7 @@
         <v>2023-01-09</v>
       </c>
       <c r="C327" t="str">
-        <v>gajanan dhore</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D327" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -17048,7 +17048,7 @@
         <v>2023-06-11</v>
       </c>
       <c r="C505" t="str">
-        <v>dhore gajanan</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D505" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -18392,7 +18392,7 @@
         <v>2023-07-14</v>
       </c>
       <c r="C547" t="str">
-        <v>gajanan dhore</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D547" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -18424,7 +18424,7 @@
         <v>2023-07-15</v>
       </c>
       <c r="C548" t="str">
-        <v>gajanan dhore</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D548" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -18488,7 +18488,7 @@
         <v>2023-07-16</v>
       </c>
       <c r="C550" t="str">
-        <v>gajanan dhore</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D550" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -18520,7 +18520,7 @@
         <v>2023-07-23</v>
       </c>
       <c r="C551" t="str">
-        <v>gajanan dhore</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D551" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -18552,7 +18552,7 @@
         <v>2023-07-24</v>
       </c>
       <c r="C552" t="str">
-        <v>gajanan dhore</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D552" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -18584,7 +18584,7 @@
         <v>2023-08-06</v>
       </c>
       <c r="C553" t="str">
-        <v>gajanan dhore</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D553" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -18616,7 +18616,7 @@
         <v>2023-08-06</v>
       </c>
       <c r="C554" t="str">
-        <v>gajanan dhore</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D554" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -19352,7 +19352,7 @@
         <v>2023-12-01</v>
       </c>
       <c r="C577" t="str">
-        <v>गजानन दोरे सरपंच</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D577" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -19544,7 +19544,7 @@
         <v>2023-12-11</v>
       </c>
       <c r="C583" t="str">
-        <v>गजानन सरपंच</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D583" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -20536,7 +20536,7 @@
         <v>2024-01-11</v>
       </c>
       <c r="C614" t="str">
-        <v>गजानन ढोरे सरपंच</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D614" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -21528,7 +21528,7 @@
         <v>2024-02-01</v>
       </c>
       <c r="C645" t="str">
-        <v>गजानन सरपंच</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D645" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -24792,7 +24792,7 @@
         <v>2024-04-01</v>
       </c>
       <c r="C747" t="str">
-        <v>गजानन सरपंच</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D747" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -27160,7 +27160,7 @@
         <v>2024-05-11</v>
       </c>
       <c r="C821" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D821" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -27192,7 +27192,7 @@
         <v>2024-05-11</v>
       </c>
       <c r="C822" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D822" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -27224,7 +27224,7 @@
         <v>2024-05-11</v>
       </c>
       <c r="C823" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D823" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -27352,7 +27352,7 @@
         <v>2024-05-11</v>
       </c>
       <c r="C827" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D827" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -27384,7 +27384,7 @@
         <v>2024-05-11</v>
       </c>
       <c r="C828" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D828" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -27416,7 +27416,7 @@
         <v>2024-05-11</v>
       </c>
       <c r="C829" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D829" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -29528,7 +29528,7 @@
         <v>2024-05-21</v>
       </c>
       <c r="C895" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D895" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -29560,7 +29560,7 @@
         <v>2024-05-21</v>
       </c>
       <c r="C896" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D896" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -29592,7 +29592,7 @@
         <v>2024-05-21</v>
       </c>
       <c r="C897" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D897" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -29624,7 +29624,7 @@
         <v>2024-05-21</v>
       </c>
       <c r="C898" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D898" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -29752,7 +29752,7 @@
         <v>2024-05-21</v>
       </c>
       <c r="C902" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D902" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -29784,7 +29784,7 @@
         <v>2024-05-21</v>
       </c>
       <c r="C903" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D903" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -29848,7 +29848,7 @@
         <v>2024-05-21</v>
       </c>
       <c r="C905" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D905" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -29912,7 +29912,7 @@
         <v>2024-05-21</v>
       </c>
       <c r="C907" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D907" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -30008,7 +30008,7 @@
         <v>2024-05-21</v>
       </c>
       <c r="C910" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D910" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -31704,7 +31704,7 @@
         <v>2024-06-08</v>
       </c>
       <c r="C963" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D963" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -31736,7 +31736,7 @@
         <v>2024-06-08</v>
       </c>
       <c r="C964" t="str">
-        <v>Gajanan Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D964" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -31896,7 +31896,7 @@
         <v>2024-10-05</v>
       </c>
       <c r="C969" t="str">
-        <v>Gajanan Dore Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D969" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -35352,7 +35352,7 @@
         <v>2025-04-22</v>
       </c>
       <c r="C1077" t="str">
-        <v>गजानन सरपंच</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D1077" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>

</xml_diff>

<commit_message>
Update Gitai application with enhancements to customer aliases functionality, including surname normalization and improved matching logic. Modify index.html to reflect updated script versions for customer-aliases.js, income.js, and receivables.js. Update Excel workbooks (Gitai-M1.xlsx, Gitai-M2.xlsx, Gitai.xlsx) to ensure data consistency with recent changes.
</commit_message>
<xml_diff>
--- a/Gitai-M1.xlsx
+++ b/Gitai-M1.xlsx
@@ -19160,7 +19160,7 @@
         <v>2023-12-01</v>
       </c>
       <c r="C571" t="str">
-        <v>माधव बापुराव दोरे</v>
+        <v>माधव बापुराव ढोरे</v>
       </c>
       <c r="D571" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -19320,7 +19320,7 @@
         <v>2023-12-01</v>
       </c>
       <c r="C576" t="str">
-        <v>बापु दोरे</v>
+        <v>बापु ढोरे</v>
       </c>
       <c r="D576" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -19384,7 +19384,7 @@
         <v>2023-12-06</v>
       </c>
       <c r="C578" t="str">
-        <v>आदिनाथ जवन दोरे</v>
+        <v>आदिनाथ जवन ढोरे</v>
       </c>
       <c r="D578" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -19416,7 +19416,7 @@
         <v>2023-12-07</v>
       </c>
       <c r="C579" t="str">
-        <v>आदिनाथ जवन दोरे</v>
+        <v>आदिनाथ जवन ढोरे</v>
       </c>
       <c r="D579" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -19448,7 +19448,7 @@
         <v>2023-12-08</v>
       </c>
       <c r="C580" t="str">
-        <v>आदिनाथ जवन दोरे</v>
+        <v>आदिनाथ जवन ढोरे</v>
       </c>
       <c r="D580" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -19480,7 +19480,7 @@
         <v>2023-12-09</v>
       </c>
       <c r="C581" t="str">
-        <v>आदिनाथ जवन दोरे</v>
+        <v>आदिनाथ जवन ढोरे</v>
       </c>
       <c r="D581" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -19512,7 +19512,7 @@
         <v>2023-12-10</v>
       </c>
       <c r="C582" t="str">
-        <v>आदिनाथ जवन दोरे</v>
+        <v>आदिनाथ जवन ढोरे</v>
       </c>
       <c r="D582" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -21176,7 +21176,7 @@
         <v>2024-01-24</v>
       </c>
       <c r="C634" t="str">
-        <v>Shyama Shankar Thaure</v>
+        <v>Shyama Shankar Dhore</v>
       </c>
       <c r="D634" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -22808,7 +22808,7 @@
         <v>2024-02-20</v>
       </c>
       <c r="C685" t="str">
-        <v>Uddhav Thore</v>
+        <v>Uddhav Dhore</v>
       </c>
       <c r="D685" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -22840,7 +22840,7 @@
         <v>2024-02-20</v>
       </c>
       <c r="C686" t="str">
-        <v>Sandeep Thore Mandap</v>
+        <v>Sandeep Dhore Mandap</v>
       </c>
       <c r="D686" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -22872,7 +22872,7 @@
         <v>2024-02-20</v>
       </c>
       <c r="C687" t="str">
-        <v>Shankar Thore Chairman</v>
+        <v>Shankar Dhore Chairman</v>
       </c>
       <c r="D687" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -27096,7 +27096,7 @@
         <v>2024-05-11</v>
       </c>
       <c r="C819" t="str">
-        <v>Gajanan Thore Sarpanch</v>
+        <v>Gajanan Nannaji Dhore</v>
       </c>
       <c r="D819" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -28632,7 +28632,7 @@
         <v>2024-05-19</v>
       </c>
       <c r="C867" t="str">
-        <v>Raju Pandu Thombre</v>
+        <v>Raju Pandu Dhore</v>
       </c>
       <c r="D867" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -29208,7 +29208,7 @@
         <v>2024-05-20</v>
       </c>
       <c r="C885" t="str">
-        <v>Santosh Thore Daji</v>
+        <v>Santosh Dhore Daji</v>
       </c>
       <c r="D885" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -29272,7 +29272,7 @@
         <v>2024-05-20</v>
       </c>
       <c r="C887" t="str">
-        <v>Nitin Thombre</v>
+        <v>Nitin Dhore</v>
       </c>
       <c r="D887" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -29336,7 +29336,7 @@
         <v>2024-05-20</v>
       </c>
       <c r="C889" t="str">
-        <v>Shyama Thombre</v>
+        <v>Shyama Dhore</v>
       </c>
       <c r="D889" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -30104,7 +30104,7 @@
         <v>2024-05-31</v>
       </c>
       <c r="C913" t="str">
-        <v>Pappu Tore</v>
+        <v>Pappu Dhore</v>
       </c>
       <c r="D913" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -30264,7 +30264,7 @@
         <v>2024-05-31</v>
       </c>
       <c r="C918" t="str">
-        <v>Suryabhan Tore</v>
+        <v>Suryabhan Dhore</v>
       </c>
       <c r="D918" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -30552,7 +30552,7 @@
         <v>2024-05-31</v>
       </c>
       <c r="C927" t="str">
-        <v>Pandit Tore</v>
+        <v>Pandit Dhore</v>
       </c>
       <c r="D927" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -30648,7 +30648,7 @@
         <v>2024-06-01</v>
       </c>
       <c r="C930" t="str">
-        <v>Shyama Thore Viheer</v>
+        <v>Shyama Dhore Viheer</v>
       </c>
       <c r="D930" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -30680,7 +30680,7 @@
         <v>2024-06-01</v>
       </c>
       <c r="C931" t="str">
-        <v>Shyama Thore Viheer</v>
+        <v>Shyama Dhore Viheer</v>
       </c>
       <c r="D931" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -30744,7 +30744,7 @@
         <v>2024-06-01</v>
       </c>
       <c r="C933" t="str">
-        <v>Nitin Thore Samaiyk</v>
+        <v>Nitin Dhore Samaiyk</v>
       </c>
       <c r="D933" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -30776,7 +30776,7 @@
         <v>2024-06-01</v>
       </c>
       <c r="C934" t="str">
-        <v>Nitin Thore Samaiyk</v>
+        <v>Nitin Dhore Samaiyk</v>
       </c>
       <c r="D934" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -30808,7 +30808,7 @@
         <v>2024-06-01</v>
       </c>
       <c r="C935" t="str">
-        <v>Santosh Thore</v>
+        <v>Santosh Dhore</v>
       </c>
       <c r="D935" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -30840,7 +30840,7 @@
         <v>2024-06-01</v>
       </c>
       <c r="C936" t="str">
-        <v>Santosh Thore</v>
+        <v>Santosh Dhore</v>
       </c>
       <c r="D936" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -30872,7 +30872,7 @@
         <v>2024-06-01</v>
       </c>
       <c r="C937" t="str">
-        <v>Nitin Thore</v>
+        <v>Nitin Dhore</v>
       </c>
       <c r="D937" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -30904,7 +30904,7 @@
         <v>2024-06-01</v>
       </c>
       <c r="C938" t="str">
-        <v>Raosaheb Thore</v>
+        <v>Raosaheb Dhore</v>
       </c>
       <c r="D938" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -30968,7 +30968,7 @@
         <v>2024-06-01</v>
       </c>
       <c r="C940" t="str">
-        <v>Balaji Thore + Mujib</v>
+        <v>Balaji Dhore + Mujib</v>
       </c>
       <c r="D940" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -31032,7 +31032,7 @@
         <v>2024-06-01</v>
       </c>
       <c r="C942" t="str">
-        <v>Shriram Thore</v>
+        <v>Shriram Dhore</v>
       </c>
       <c r="D942" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -31064,7 +31064,7 @@
         <v>2024-06-01</v>
       </c>
       <c r="C943" t="str">
-        <v>Shriram Thore</v>
+        <v>Shriram Dhore</v>
       </c>
       <c r="D943" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -31096,7 +31096,7 @@
         <v>2024-06-01</v>
       </c>
       <c r="C944" t="str">
-        <v>Annaji Thore Mama</v>
+        <v>Annaji Dhore Mama</v>
       </c>
       <c r="D944" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -31544,7 +31544,7 @@
         <v>2024-06-08</v>
       </c>
       <c r="C958" t="str">
-        <v>Sham Tore</v>
+        <v>Sham Dhore</v>
       </c>
       <c r="D958" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -31928,7 +31928,7 @@
         <v>2024-10-05</v>
       </c>
       <c r="C970" t="str">
-        <v>Sonya Dore</v>
+        <v>Sonya Dhore</v>
       </c>
       <c r="D970" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -31960,7 +31960,7 @@
         <v>2024-10-05</v>
       </c>
       <c r="C971" t="str">
-        <v>Subhan Dore Khadda</v>
+        <v>Subhan Dhore Khadda</v>
       </c>
       <c r="D971" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -32088,7 +32088,7 @@
         <v>2024-10-05</v>
       </c>
       <c r="C975" t="str">
-        <v>Davakhana Dore</v>
+        <v>Davakhana Dhore</v>
       </c>
       <c r="D975" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -32120,7 +32120,7 @@
         <v>2024-10-05</v>
       </c>
       <c r="C976" t="str">
-        <v>Bandu Mama Dore Khadda</v>
+        <v>Bandu Mama Dhore Khadda</v>
       </c>
       <c r="D976" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -32152,7 +32152,7 @@
         <v>2024-10-05</v>
       </c>
       <c r="C977" t="str">
-        <v>Raj Nago Dore</v>
+        <v>Raj Nago Dhore</v>
       </c>
       <c r="D977" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -32184,7 +32184,7 @@
         <v>2024-10-05</v>
       </c>
       <c r="C978" t="str">
-        <v>Raj Nago Dore</v>
+        <v>Raj Nago Dhore</v>
       </c>
       <c r="D978" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -32216,7 +32216,7 @@
         <v>2024-10-05</v>
       </c>
       <c r="C979" t="str">
-        <v>Raj Nago Dore</v>
+        <v>Raj Nago Dhore</v>
       </c>
       <c r="D979" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -32248,7 +32248,7 @@
         <v>2024-10-05</v>
       </c>
       <c r="C980" t="str">
-        <v>Raj Nago Dore</v>
+        <v>Raj Nago Dhore</v>
       </c>
       <c r="D980" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -32312,7 +32312,7 @@
         <v>2024-10-05</v>
       </c>
       <c r="C982" t="str">
-        <v>Akshay Savan Dore</v>
+        <v>Akshay Savan Dhore</v>
       </c>
       <c r="D982" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -32376,7 +32376,7 @@
         <v>2025-01-02</v>
       </c>
       <c r="C984" t="str">
-        <v>Shivraj Thore</v>
+        <v>Shivraj Dhore</v>
       </c>
       <c r="D984" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -32408,7 +32408,7 @@
         <v>2025-01-02</v>
       </c>
       <c r="C985" t="str">
-        <v>Sunil Thore</v>
+        <v>Sunil Dhore</v>
       </c>
       <c r="D985" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -32536,7 +32536,7 @@
         <v>2025-01-02</v>
       </c>
       <c r="C989" t="str">
-        <v>Sambhaji Thore</v>
+        <v>Sambhaji Dhore</v>
       </c>
       <c r="D989" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -32696,7 +32696,7 @@
         <v>2025-01-02</v>
       </c>
       <c r="C994" t="str">
-        <v>Mayank Thore</v>
+        <v>Mayank Dhore</v>
       </c>
       <c r="D994" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -32728,7 +32728,7 @@
         <v>2025-01-02</v>
       </c>
       <c r="C995" t="str">
-        <v>Shyam Shankar Thore</v>
+        <v>Shyam Shankar Dhore</v>
       </c>
       <c r="D995" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -35448,7 +35448,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="C1080" t="str">
-        <v>गंगाधर पुंडलिक ठोंबरे</v>
+        <v>गंगाधर पुंडलिक ढोरे</v>
       </c>
       <c r="D1080" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -35480,7 +35480,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="C1081" t="str">
-        <v>भानुदास ठोरे + जवन</v>
+        <v>भानुदास ढोरे + जवन</v>
       </c>
       <c r="D1081" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -35544,7 +35544,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="C1083" t="str">
-        <v>जवन ठोरे</v>
+        <v>जवन ढोरे</v>
       </c>
       <c r="D1083" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -35672,7 +35672,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="C1087" t="str">
-        <v>सदाशिव सुदाम ठोरे</v>
+        <v>सदाशिव सुदाम ढोरे</v>
       </c>
       <c r="D1087" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -35864,7 +35864,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="C1093" t="str">
-        <v>श्यामा शंकर ठोरे</v>
+        <v>श्यामा शंकर ढोरे</v>
       </c>
       <c r="D1093" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -35928,7 +35928,7 @@
         <v>2025-05-30</v>
       </c>
       <c r="C1095" t="str">
-        <v>आदिनाथ ठौरे</v>
+        <v>आदिनाथ ढोरे</v>
       </c>
       <c r="D1095" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -36056,7 +36056,7 @@
         <v>2025-05-30</v>
       </c>
       <c r="C1099" t="str">
-        <v>उद्धव + देविदास ठौरे</v>
+        <v>उद्धव + देविदास ढोरे</v>
       </c>
       <c r="D1099" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -36184,7 +36184,7 @@
         <v>2025-05-30</v>
       </c>
       <c r="C1103" t="str">
-        <v>कपील ठौरे</v>
+        <v>कपील ढोरे</v>
       </c>
       <c r="D1103" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -36440,7 +36440,7 @@
         <v>2025-05-30</v>
       </c>
       <c r="C1111" t="str">
-        <v>काशिनाथ ठौरे</v>
+        <v>काशिनाथ ढोरे</v>
       </c>
       <c r="D1111" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -36984,7 +36984,7 @@
         <v>2025-06-10</v>
       </c>
       <c r="C1128" t="str">
-        <v>गजानन मारोती ठोंबरे</v>
+        <v>गजानन मारोती ढोरे</v>
       </c>
       <c r="D1128" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -37784,7 +37784,7 @@
         <v>2025-06-10</v>
       </c>
       <c r="C1153" t="str">
-        <v>अनंत ठौरे</v>
+        <v>अनंत ढोरे</v>
       </c>
       <c r="D1153" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -37976,7 +37976,7 @@
         <v>2025-06-10</v>
       </c>
       <c r="C1159" t="str">
-        <v>शामराव ठौरे</v>
+        <v>शामराव ढोरे</v>
       </c>
       <c r="D1159" t="str">
         <v>M1- Mahindra earthmaster sx iv 2022</v>
@@ -48735,7 +48735,7 @@
         <v/>
       </c>
       <c r="G465" t="str">
-        <v>शाम ठोरे | dateMappedFromIncome:true | p4 | imported from M1_book3_1.pdf</v>
+        <v>शाम ढोरे | dateMappedFromIncome:true | p4 | imported from M1_book3_1.pdf</v>
       </c>
     </row>
     <row r="466">

</xml_diff>